<commit_message>
Added skew compensation line directly to spreadsheet
</commit_message>
<xml_diff>
--- a/Parametric Skew Calibration.xlsx
+++ b/Parametric Skew Calibration.xlsx
@@ -5308,12 +5308,18 @@
         <f>IF(Helper!C4,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="15" t="str">
+      <c r="D10" s="12">
+        <v>119.91</v>
+      </c>
+      <c r="E10" s="13">
+        <v>119.89</v>
+      </c>
+      <c r="F10" s="14">
+        <v>119.93</v>
+      </c>
+      <c r="G10" s="15">
         <f t="shared" ref="G10:G37" si="1">IF(OR(B10="",ISBLANK(D10)), "", AVERAGE(D10:F10))</f>
-        <v/>
+        <v>119.91</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -5326,12 +5332,18 @@
         <f>IF(Helper!C5,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D11" s="18"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="21" t="str">
+      <c r="D11" s="18">
+        <v>79.92</v>
+      </c>
+      <c r="E11" s="19">
+        <v>80.2</v>
+      </c>
+      <c r="F11" s="20">
+        <v>79.98</v>
+      </c>
+      <c r="G11" s="21">
         <f t="shared" si="1"/>
-        <v/>
+        <v>80.03333333</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -5344,15 +5356,21 @@
         <f>IF(Helper!C6, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D12" s="18"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="21" t="str">
+      <c r="D12" s="18">
+        <v>40.08</v>
+      </c>
+      <c r="E12" s="19">
+        <v>39.99</v>
+      </c>
+      <c r="F12" s="20">
+        <v>40.04</v>
+      </c>
+      <c r="G12" s="21">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="15.75" customHeight="1">
+        <v>40.03666667</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" hidden="1" customHeight="1">
       <c r="A13" s="16"/>
       <c r="B13" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
@@ -5370,7 +5388,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1">
+    <row r="14" ht="15.75" hidden="1" customHeight="1">
       <c r="A14" s="25"/>
       <c r="B14" s="26" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
@@ -5400,12 +5418,18 @@
         <f>IF(Helper!C9,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="15" t="str">
+      <c r="D15" s="12">
+        <v>119.9</v>
+      </c>
+      <c r="E15" s="13">
+        <v>119.85</v>
+      </c>
+      <c r="F15" s="14">
+        <v>119.9</v>
+      </c>
+      <c r="G15" s="15">
         <f t="shared" si="1"/>
-        <v/>
+        <v>119.8833333</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -5418,12 +5442,18 @@
         <f>IF(Helper!C10,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D16" s="18"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="21" t="str">
+      <c r="D16" s="18">
+        <v>79.9</v>
+      </c>
+      <c r="E16" s="19">
+        <v>79.94</v>
+      </c>
+      <c r="F16" s="20">
+        <v>79.96</v>
+      </c>
+      <c r="G16" s="21">
         <f t="shared" si="1"/>
-        <v/>
+        <v>79.93333333</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
@@ -5436,15 +5466,21 @@
         <f>IF(Helper!C11, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D17" s="18"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="21" t="str">
+      <c r="D17" s="18">
+        <v>39.9</v>
+      </c>
+      <c r="E17" s="19">
+        <v>39.96</v>
+      </c>
+      <c r="F17" s="20">
+        <v>39.99</v>
+      </c>
+      <c r="G17" s="21">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1">
+        <v>39.95</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75" hidden="1" customHeight="1">
       <c r="A18" s="16"/>
       <c r="B18" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
@@ -5462,7 +5498,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" ht="15.75" hidden="1" customHeight="1">
       <c r="A19" s="25"/>
       <c r="B19" s="26" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
@@ -5492,12 +5528,18 @@
         <f>IF(Helper!C14,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D20" s="12"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="15" t="str">
+      <c r="D20" s="12">
+        <v>119.8</v>
+      </c>
+      <c r="E20" s="13">
+        <v>119.81</v>
+      </c>
+      <c r="F20" s="14">
+        <v>119.85</v>
+      </c>
+      <c r="G20" s="15">
         <f t="shared" si="1"/>
-        <v/>
+        <v>119.82</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -5510,12 +5552,18 @@
         <f>IF(Helper!C15,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D21" s="18"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="21" t="str">
+      <c r="D21" s="18">
+        <v>79.9</v>
+      </c>
+      <c r="E21" s="19">
+        <v>79.93</v>
+      </c>
+      <c r="F21" s="20">
+        <v>79.92</v>
+      </c>
+      <c r="G21" s="21">
         <f t="shared" si="1"/>
-        <v/>
+        <v>79.91666667</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -5528,15 +5576,21 @@
         <f>IF(Helper!C16, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D22" s="18"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="21" t="str">
+      <c r="D22" s="18">
+        <v>39.94</v>
+      </c>
+      <c r="E22" s="19">
+        <v>39.94</v>
+      </c>
+      <c r="F22" s="20">
+        <v>39.95</v>
+      </c>
+      <c r="G22" s="21">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
+        <v>39.94333333</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" hidden="1" customHeight="1">
       <c r="A23" s="16"/>
       <c r="B23" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
@@ -5554,7 +5608,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" ht="15.75" hidden="1" customHeight="1">
       <c r="A24" s="25"/>
       <c r="B24" s="26" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
@@ -5584,12 +5638,18 @@
         <f>IF(Helper!C19,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D25" s="12"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="15" t="str">
+      <c r="D25" s="12">
+        <v>119.91</v>
+      </c>
+      <c r="E25" s="13">
+        <v>119.86</v>
+      </c>
+      <c r="F25" s="14">
+        <v>119.91</v>
+      </c>
+      <c r="G25" s="15">
         <f t="shared" si="1"/>
-        <v/>
+        <v>119.8933333</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -5602,12 +5662,18 @@
         <f>IF(Helper!C20,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D26" s="18"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="21" t="str">
+      <c r="D26" s="18">
+        <v>79.85</v>
+      </c>
+      <c r="E26" s="19">
+        <v>79.88</v>
+      </c>
+      <c r="F26" s="20">
+        <v>79.98</v>
+      </c>
+      <c r="G26" s="21">
         <f t="shared" si="1"/>
-        <v/>
+        <v>79.90333333</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -5620,15 +5686,21 @@
         <f>IF(Helper!C21, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D27" s="18"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="21" t="str">
+      <c r="D27" s="18">
+        <v>39.85</v>
+      </c>
+      <c r="E27" s="19">
+        <v>39.94</v>
+      </c>
+      <c r="F27" s="20">
+        <v>39.98</v>
+      </c>
+      <c r="G27" s="21">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
+        <v>39.92333333</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" hidden="1" customHeight="1">
       <c r="A28" s="16"/>
       <c r="B28" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
@@ -5646,7 +5718,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" ht="15.75" hidden="1" customHeight="1">
       <c r="A29" s="16"/>
       <c r="B29" s="1" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
@@ -5676,12 +5748,18 @@
         <f>IF(Helper!C24,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D30" s="12"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="33" t="str">
+      <c r="D30" s="12">
+        <v>120.04</v>
+      </c>
+      <c r="E30" s="13">
+        <v>120.02</v>
+      </c>
+      <c r="F30" s="14">
+        <v>119.98</v>
+      </c>
+      <c r="G30" s="33">
         <f t="shared" si="1"/>
-        <v/>
+        <v>120.0133333</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
@@ -5694,15 +5772,21 @@
         <f>IF(Helper!C25,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D31" s="18"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="21" t="str">
+      <c r="D31" s="18">
+        <v>80.07</v>
+      </c>
+      <c r="E31" s="19">
+        <v>80.05</v>
+      </c>
+      <c r="F31" s="20">
+        <v>80.08</v>
+      </c>
+      <c r="G31" s="21">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
+        <v>80.06666667</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75" hidden="1" customHeight="1">
       <c r="A32" s="16"/>
       <c r="B32" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 3, "")</f>
@@ -5720,7 +5804,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" ht="15.75" hidden="1" customHeight="1">
       <c r="A33" s="16"/>
       <c r="B33" s="1" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
@@ -5750,12 +5834,18 @@
         <f>IF(Helper!C28,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D34" s="12"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="33" t="str">
+      <c r="D34" s="12">
+        <v>119.62</v>
+      </c>
+      <c r="E34" s="13">
+        <v>119.59</v>
+      </c>
+      <c r="F34" s="14">
+        <v>119.62</v>
+      </c>
+      <c r="G34" s="33">
         <f t="shared" si="1"/>
-        <v/>
+        <v>119.61</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
@@ -5768,15 +5858,21 @@
         <f>IF(Helper!C29,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D35" s="18"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="34" t="str">
+      <c r="D35" s="18">
+        <v>79.76</v>
+      </c>
+      <c r="E35" s="19">
+        <v>79.75</v>
+      </c>
+      <c r="F35" s="20">
+        <v>79.77</v>
+      </c>
+      <c r="G35" s="34">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
+        <v>79.76</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" hidden="1" customHeight="1">
       <c r="A36" s="16"/>
       <c r="B36" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 3, "")</f>
@@ -5794,7 +5890,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" ht="15.75" hidden="1" customHeight="1">
       <c r="A37" s="25"/>
       <c r="B37" s="26" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
@@ -10859,7 +10955,15 @@
       <c r="C1035" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="$C$9:$C$37"/>
+  <autoFilter ref="$C$9:$C$37">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="40.00"/>
+        <filter val="120.00"/>
+        <filter val="80.00"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="D10:F38">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>LEN(TRIM(D10))=0</formula>
@@ -10940,17 +11044,17 @@
         <v>46</v>
       </c>
       <c r="B4" s="40"/>
-      <c r="C4" s="40" t="str">
+      <c r="C4" s="40">
         <f>Helper!E43</f>
-        <v>#DIV/0!</v>
+        <v>-0.000412037037</v>
       </c>
       <c r="D4" s="44">
         <f>SQRT(SUMSQ(Helper!K4:K13))</f>
-        <v>0</v>
-      </c>
-      <c r="E4" s="45" t="str">
+        <v>0.0004159845239</v>
+      </c>
+      <c r="E4" s="45">
         <f t="shared" ref="E4:E5" si="1">-C4</f>
-        <v>#DIV/0!</v>
+        <v>0.000412037037</v>
       </c>
       <c r="G4" s="46" t="s">
         <v>47</v>
@@ -10964,17 +11068,17 @@
         <v>48</v>
       </c>
       <c r="B5" s="40"/>
-      <c r="C5" s="40" t="str">
+      <c r="C5" s="40">
         <f>Helper!E44</f>
-        <v>#DIV/0!</v>
+        <v>-0.001328703704</v>
       </c>
       <c r="D5" s="44">
         <f>SQRT(SUMSQ(Helper!K14:K23))</f>
-        <v>0</v>
-      </c>
-      <c r="E5" s="45" t="str">
+        <v>0.0003196121406</v>
+      </c>
+      <c r="E5" s="45">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>0.001328703704</v>
       </c>
       <c r="G5" s="48" t="s">
         <v>49</v>
@@ -11020,13 +11124,13 @@
         <v>54</v>
       </c>
       <c r="B8" s="23"/>
-      <c r="C8" s="23" t="str">
+      <c r="C8" s="23">
         <f>Helper!B41</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D8" s="54" t="str">
+        <v>89.79659109</v>
+      </c>
+      <c r="D8" s="54">
         <f>Helper!B43</f>
-        <v>#DIV/0!</v>
+        <v>0.01150995384</v>
       </c>
       <c r="E8" s="24"/>
       <c r="G8" s="55" t="s">
@@ -11041,17 +11145,17 @@
         <v>56</v>
       </c>
       <c r="B9" s="29"/>
-      <c r="C9" s="29" t="str">
+      <c r="C9" s="29">
         <f>C8-90</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D9" s="58" t="str">
+        <v>-0.2034089089</v>
+      </c>
+      <c r="D9" s="58">
         <f>Helper!B43</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E9" s="30" t="str">
+        <v>0.01150995384</v>
+      </c>
+      <c r="E9" s="30">
         <f>-C9</f>
-        <v>#DIV/0!</v>
+        <v>0.2034089089</v>
       </c>
       <c r="J9" s="23"/>
     </row>
@@ -11101,14 +11205,14 @@
       <c r="H14" s="16"/>
       <c r="I14" s="1" t="str">
         <f>"M92 X"&amp;ROUND(Helper!F43,3)&amp;" Y"&amp;ROUND(Helper!F44,3)</f>
-        <v>#DIV/0!</v>
+        <v>M92 X39.979 Y39.95</v>
       </c>
       <c r="M14" s="41"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="22" t="str">
         <f>"Length AC = "&amp;ROUND(Helper!B36,2)</f>
-        <v>#DIV/0!</v>
+        <v>Length AC = 120.05</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="41"/>
@@ -11120,7 +11224,7 @@
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="22" t="str">
         <f>"Length BD = "&amp;ROUND(Helper!B37,2)</f>
-        <v>#DIV/0!</v>
+        <v>Length BD = 119.62</v>
       </c>
       <c r="F16" s="41"/>
       <c r="H16" s="16" t="s">
@@ -11131,14 +11235,17 @@
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="22" t="str">
         <f>"Length AD = "&amp;ROUND(Helper!B38,2)</f>
-        <v>#DIV/0!</v>
+        <v>Length AD = 84.85</v>
       </c>
       <c r="F17" s="41"/>
       <c r="H17" s="16"/>
       <c r="M17" s="41"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="22"/>
+      <c r="A18" s="18" t="str">
+        <f>"CALC_MEASURED_SKEW AC="&amp;ROUND(Helper!B36,2)&amp;" BD="&amp;ROUND(Helper!B37,2)&amp;" AD="&amp;ROUND(Helper!B38,2)</f>
+        <v>CALC_MEASURED_SKEW AC=120.05 BD=119.62 AD=84.85</v>
+      </c>
       <c r="F18" s="41"/>
       <c r="H18" s="16" t="s">
         <v>65</v>
@@ -11157,9 +11264,9 @@
       <c r="A20" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="1" t="str">
+      <c r="B20" s="1">
         <f>ROUND(Helper!F43,3)</f>
-        <v>#DIV/0!</v>
+        <v>39.979</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>68</v>
@@ -11172,9 +11279,9 @@
       <c r="A21" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="B21" s="26" t="str">
+      <c r="B21" s="26">
         <f>ROUND(Helper!F44,3)</f>
-        <v>#DIV/0!</v>
+        <v>39.95</v>
       </c>
       <c r="C21" s="26" t="s">
         <v>69</v>
@@ -14250,35 +14357,35 @@
       </c>
       <c r="D4" s="8" t="b">
         <f t="shared" ref="D4:D31" si="2">IFERROR(AND(NOT(F4=0),NOT(F4=""),C4),FALSE())</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="62">
         <f>IF(D4,'Post-print worksheet'!C10,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="63" t="str">
+        <v>120</v>
+      </c>
+      <c r="F4" s="63">
         <f>IF(C4, IFERROR(AVERAGE('Post-print worksheet'!D10:F10),""),"")</f>
-        <v/>
+        <v>119.91</v>
       </c>
       <c r="G4" s="63">
         <f>IF(C4, IFERROR(STDEV('Post-print worksheet'!D10:F10),0),"")</f>
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="H4" s="63">
         <f>IF(C4, IFERROR(SQRT((Intro!$B$8/3)^2+G4^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I4" s="63" t="str">
+        <v>0.0202758751</v>
+      </c>
+      <c r="I4" s="63">
         <f t="shared" ref="I4:I31" si="3">IF(D4, IFERROR((F4-E4)/E4,0),"")</f>
-        <v/>
-      </c>
-      <c r="J4" s="63" t="str">
+        <v>-0.00075</v>
+      </c>
+      <c r="J4" s="63">
         <f t="shared" ref="J4:J22" si="4">IF(D4, 1/(($B$47+$B$48)*E4),"")</f>
-        <v/>
-      </c>
-      <c r="K4" s="63" t="str">
+        <v>0.001388888889</v>
+      </c>
+      <c r="K4" s="63">
         <f t="shared" ref="K4:K23" si="5">IF(D4,J4*H4,"")</f>
-        <v/>
+        <v>0.00002816093764</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -14293,35 +14400,35 @@
       </c>
       <c r="D5" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="64">
         <f>IF(D5,'Post-print worksheet'!C11,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="23" t="str">
+        <v>80</v>
+      </c>
+      <c r="F5" s="23">
         <f>IF(C5, IFERROR(AVERAGE('Post-print worksheet'!D11:F11),""),"")</f>
-        <v/>
+        <v>80.03333333</v>
       </c>
       <c r="G5" s="23">
         <f>IF(C5, IFERROR(STDEV('Post-print worksheet'!D11:F11),0),"")</f>
-        <v>0</v>
+        <v>0.1474222959</v>
       </c>
       <c r="H5" s="23">
         <f>IF(C5, IFERROR(SQRT((Intro!$B$8/3)^2+G5^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I5" s="23" t="str">
+        <v>0.1474599757</v>
+      </c>
+      <c r="I5" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J5" s="23" t="str">
+        <v>0.0004166666667</v>
+      </c>
+      <c r="J5" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K5" s="23" t="str">
+        <v>0.002083333333</v>
+      </c>
+      <c r="K5" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.0003072082828</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -14336,35 +14443,35 @@
       </c>
       <c r="D6" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="64">
         <f>IF(D6,'Post-print worksheet'!C12,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="23" t="str">
+        <v>40</v>
+      </c>
+      <c r="F6" s="23">
         <f>IF(C6, IFERROR(AVERAGE('Post-print worksheet'!D12:F12),""),"")</f>
-        <v/>
+        <v>40.03666667</v>
       </c>
       <c r="G6" s="23">
         <f>IF(C6, IFERROR(STDEV('Post-print worksheet'!D12:F12),0),"")</f>
-        <v>0</v>
+        <v>0.04509249753</v>
       </c>
       <c r="H6" s="23">
         <f>IF(C6, IFERROR(SQRT((Intro!$B$8/3)^2+G6^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I6" s="23" t="str">
+        <v>0.04521553322</v>
+      </c>
+      <c r="I6" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J6" s="23" t="str">
+        <v>0.0009166666667</v>
+      </c>
+      <c r="J6" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K6" s="23" t="str">
+        <v>0.004166666667</v>
+      </c>
+      <c r="K6" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.0001883980551</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -14467,35 +14574,35 @@
       </c>
       <c r="D9" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="64">
         <f>IF(D9,'Post-print worksheet'!C15,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="23" t="str">
+        <v>120</v>
+      </c>
+      <c r="F9" s="23">
         <f>IF(C9, IFERROR(AVERAGE('Post-print worksheet'!D15:F15),""),"")</f>
-        <v/>
+        <v>119.8833333</v>
       </c>
       <c r="G9" s="23">
         <f>IF(C9, IFERROR(STDEV('Post-print worksheet'!D15:F15),0),"")</f>
-        <v>0</v>
+        <v>0.02886751346</v>
       </c>
       <c r="H9" s="23">
         <f>IF(C9, IFERROR(SQRT((Intro!$B$8/3)^2+G9^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I9" s="23" t="str">
+        <v>0.02905932629</v>
+      </c>
+      <c r="I9" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J9" s="23" t="str">
+        <v>-0.0009722222222</v>
+      </c>
+      <c r="J9" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K9" s="23" t="str">
+        <v>0.001388888889</v>
+      </c>
+      <c r="K9" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.0000403601754</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -14510,35 +14617,35 @@
       </c>
       <c r="D10" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="64">
         <f>IF(D10,'Post-print worksheet'!C16,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="23" t="str">
+        <v>80</v>
+      </c>
+      <c r="F10" s="23">
         <f>IF(C10, IFERROR(AVERAGE('Post-print worksheet'!D16:F16),""),"")</f>
-        <v/>
+        <v>79.93333333</v>
       </c>
       <c r="G10" s="23">
         <f>IF(C10, IFERROR(STDEV('Post-print worksheet'!D16:F16),0),"")</f>
-        <v>0</v>
+        <v>0.03055050463</v>
       </c>
       <c r="H10" s="23">
         <f>IF(C10, IFERROR(SQRT((Intro!$B$8/3)^2+G10^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I10" s="23" t="str">
+        <v>0.03073181486</v>
+      </c>
+      <c r="I10" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J10" s="23" t="str">
+        <v>-0.0008333333333</v>
+      </c>
+      <c r="J10" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K10" s="23" t="str">
+        <v>0.002083333333</v>
+      </c>
+      <c r="K10" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.00006402461429</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -14553,35 +14660,35 @@
       </c>
       <c r="D11" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="64">
         <f>IF(D11,'Post-print worksheet'!C17,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="23" t="str">
+        <v>40</v>
+      </c>
+      <c r="F11" s="23">
         <f>IF(C11, IFERROR(AVERAGE('Post-print worksheet'!D17:F17),""),"")</f>
-        <v/>
+        <v>39.95</v>
       </c>
       <c r="G11" s="23">
         <f>IF(C11, IFERROR(STDEV('Post-print worksheet'!D17:F17),0),"")</f>
-        <v>0</v>
+        <v>0.04582575695</v>
       </c>
       <c r="H11" s="23">
         <f>IF(C11, IFERROR(SQRT((Intro!$B$8/3)^2+G11^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I11" s="23" t="str">
+        <v>0.04594682917</v>
+      </c>
+      <c r="I11" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J11" s="23" t="str">
+        <v>-0.00125</v>
+      </c>
+      <c r="J11" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K11" s="23" t="str">
+        <v>0.004166666667</v>
+      </c>
+      <c r="K11" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.0001914451216</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -14684,35 +14791,35 @@
       </c>
       <c r="D14" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="64">
         <f>IF(D14,'Post-print worksheet'!C20,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F14" s="23" t="str">
+        <v>120</v>
+      </c>
+      <c r="F14" s="23">
         <f>IF(C14, IFERROR(AVERAGE('Post-print worksheet'!D20:F20),""),"")</f>
-        <v/>
+        <v>119.82</v>
       </c>
       <c r="G14" s="23">
         <f>IF(C14, IFERROR(STDEV('Post-print worksheet'!D20:F20),0),"")</f>
-        <v>0</v>
+        <v>0.02645751311</v>
       </c>
       <c r="H14" s="23">
         <f>IF(C14, IFERROR(SQRT((Intro!$B$8/3)^2+G14^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I14" s="23" t="str">
+        <v>0.02666666667</v>
+      </c>
+      <c r="I14" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J14" s="23" t="str">
+        <v>-0.0015</v>
+      </c>
+      <c r="J14" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K14" s="23" t="str">
+        <v>0.001388888889</v>
+      </c>
+      <c r="K14" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.00003703703704</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
@@ -14727,35 +14834,35 @@
       </c>
       <c r="D15" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="64">
         <f>IF(D15,'Post-print worksheet'!C21,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="23" t="str">
+        <v>80</v>
+      </c>
+      <c r="F15" s="23">
         <f>IF(C15, IFERROR(AVERAGE('Post-print worksheet'!D21:F21),""),"")</f>
-        <v/>
+        <v>79.91666667</v>
       </c>
       <c r="G15" s="23">
         <f>IF(C15, IFERROR(STDEV('Post-print worksheet'!D21:F21),0),"")</f>
-        <v>0</v>
+        <v>0.01527525232</v>
       </c>
       <c r="H15" s="23">
         <f>IF(C15, IFERROR(SQRT((Intro!$B$8/3)^2+G15^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I15" s="23" t="str">
+        <v>0.0156347192</v>
+      </c>
+      <c r="I15" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J15" s="23" t="str">
+        <v>-0.001041666667</v>
+      </c>
+      <c r="J15" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K15" s="23" t="str">
+        <v>0.002083333333</v>
+      </c>
+      <c r="K15" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.00003257233167</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -14770,35 +14877,35 @@
       </c>
       <c r="D16" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="64">
         <f>IF(D16,'Post-print worksheet'!C22,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="23" t="str">
+        <v>40</v>
+      </c>
+      <c r="F16" s="23">
         <f>IF(C16, IFERROR(AVERAGE('Post-print worksheet'!D22:F22),""),"")</f>
-        <v/>
+        <v>39.94333333</v>
       </c>
       <c r="G16" s="23">
         <f>IF(C16, IFERROR(STDEV('Post-print worksheet'!D22:F22),0),"")</f>
-        <v>0</v>
+        <v>0.005773502692</v>
       </c>
       <c r="H16" s="23">
         <f>IF(C16, IFERROR(SQRT((Intro!$B$8/3)^2+G16^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I16" s="23" t="str">
+        <v>0.006666666667</v>
+      </c>
+      <c r="I16" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J16" s="23" t="str">
+        <v>-0.001416666667</v>
+      </c>
+      <c r="J16" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K16" s="23" t="str">
+        <v>0.004166666667</v>
+      </c>
+      <c r="K16" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.00002777777778</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
@@ -14901,35 +15008,35 @@
       </c>
       <c r="D19" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" s="64">
         <f>IF(D19,'Post-print worksheet'!C25,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F19" s="23" t="str">
+        <v>120</v>
+      </c>
+      <c r="F19" s="23">
         <f>IF(C19, IFERROR(AVERAGE('Post-print worksheet'!D25:F25),""),"")</f>
-        <v/>
+        <v>119.8933333</v>
       </c>
       <c r="G19" s="23">
         <f>IF(C19, IFERROR(STDEV('Post-print worksheet'!D25:F25),0),"")</f>
-        <v>0</v>
+        <v>0.02886751346</v>
       </c>
       <c r="H19" s="23">
         <f>IF(C19, IFERROR(SQRT((Intro!$B$8/3)^2+G19^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I19" s="23" t="str">
+        <v>0.02905932629</v>
+      </c>
+      <c r="I19" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J19" s="23" t="str">
+        <v>-0.0008888888889</v>
+      </c>
+      <c r="J19" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K19" s="23" t="str">
+        <v>0.001388888889</v>
+      </c>
+      <c r="K19" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.0000403601754</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
@@ -14944,35 +15051,35 @@
       </c>
       <c r="D20" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" s="64">
         <f>IF(D20,'Post-print worksheet'!C26,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F20" s="23" t="str">
+        <v>80</v>
+      </c>
+      <c r="F20" s="23">
         <f>IF(C20, IFERROR(AVERAGE('Post-print worksheet'!D26:F26),""),"")</f>
-        <v/>
+        <v>79.90333333</v>
       </c>
       <c r="G20" s="23">
         <f>IF(C20, IFERROR(STDEV('Post-print worksheet'!D26:F26),0),"")</f>
-        <v>0</v>
+        <v>0.06806859286</v>
       </c>
       <c r="H20" s="23">
         <f>IF(C20, IFERROR(SQRT((Intro!$B$8/3)^2+G20^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I20" s="23" t="str">
+        <v>0.068150161</v>
+      </c>
+      <c r="I20" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J20" s="23" t="str">
+        <v>-0.001208333333</v>
+      </c>
+      <c r="J20" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K20" s="23" t="str">
+        <v>0.002083333333</v>
+      </c>
+      <c r="K20" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.0001419795021</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -14987,35 +15094,35 @@
       </c>
       <c r="D21" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" s="64">
         <f>IF(D21,'Post-print worksheet'!C27,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F21" s="23" t="str">
+        <v>40</v>
+      </c>
+      <c r="F21" s="23">
         <f>IF(C21, IFERROR(AVERAGE('Post-print worksheet'!D27:F27),""),"")</f>
-        <v/>
+        <v>39.92333333</v>
       </c>
       <c r="G21" s="23">
         <f>IF(C21, IFERROR(STDEV('Post-print worksheet'!D27:F27),0),"")</f>
-        <v>0</v>
+        <v>0.06658328118</v>
       </c>
       <c r="H21" s="23">
         <f>IF(C21, IFERROR(SQRT((Intro!$B$8/3)^2+G21^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I21" s="23" t="str">
+        <v>0.06666666667</v>
+      </c>
+      <c r="I21" s="23">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J21" s="23" t="str">
+        <v>-0.001916666667</v>
+      </c>
+      <c r="J21" s="23">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K21" s="23" t="str">
+        <v>0.004166666667</v>
+      </c>
+      <c r="K21" s="23">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0.0002777777778</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -15118,27 +15225,27 @@
       </c>
       <c r="D24" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="64">
         <f>IF(D24,'Post-print worksheet'!C30,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F24" s="23" t="str">
+        <v>120</v>
+      </c>
+      <c r="F24" s="23">
         <f>IF(C24, IFERROR(AVERAGE('Post-print worksheet'!D30:F30),""),"")</f>
-        <v/>
+        <v>120.0133333</v>
       </c>
       <c r="G24" s="23">
         <f>IF(C24, IFERROR(STDEV('Post-print worksheet'!D30:F30),0),"")</f>
-        <v>0</v>
+        <v>0.03055050463</v>
       </c>
       <c r="H24" s="23">
         <f>IF(C24, IFERROR(SQRT((Intro!$B$8/3)^2+G24^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I24" s="23" t="str">
+        <v>0.03073181486</v>
+      </c>
+      <c r="I24" s="23">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.0001111111111</v>
       </c>
       <c r="J24" s="66"/>
       <c r="K24" s="66"/>
@@ -15155,27 +15262,27 @@
       </c>
       <c r="D25" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" s="64">
         <f>IF(D25,'Post-print worksheet'!C31,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F25" s="23" t="str">
+        <v>80</v>
+      </c>
+      <c r="F25" s="23">
         <f>IF(C25, IFERROR(AVERAGE('Post-print worksheet'!D31:F31),""),"")</f>
-        <v/>
+        <v>80.06666667</v>
       </c>
       <c r="G25" s="23">
         <f>IF(C25, IFERROR(STDEV('Post-print worksheet'!D31:F31),0),"")</f>
-        <v>0</v>
+        <v>0.01527525232</v>
       </c>
       <c r="H25" s="23">
         <f>IF(C25, IFERROR(SQRT((Intro!$B$8/3)^2+G25^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I25" s="23" t="str">
+        <v>0.0156347192</v>
+      </c>
+      <c r="I25" s="23">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.0008333333333</v>
       </c>
       <c r="J25" s="66"/>
       <c r="K25" s="66"/>
@@ -15268,27 +15375,27 @@
       </c>
       <c r="D28" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" s="64">
         <f>IF(D28,'Post-print worksheet'!C34,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F28" s="23" t="str">
+        <v>120</v>
+      </c>
+      <c r="F28" s="23">
         <f>IF(C28, IFERROR(AVERAGE('Post-print worksheet'!D34:F34),""),"")</f>
-        <v/>
+        <v>119.61</v>
       </c>
       <c r="G28" s="23">
         <f>IF(C28, IFERROR(STDEV('Post-print worksheet'!D34:F34),0),"")</f>
-        <v>0</v>
+        <v>0.01732050808</v>
       </c>
       <c r="H28" s="23">
         <f>IF(C28, IFERROR(SQRT((Intro!$B$8/3)^2+G28^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I28" s="23" t="str">
+        <v>0.01763834207</v>
+      </c>
+      <c r="I28" s="23">
         <f t="shared" si="3"/>
-        <v/>
+        <v>-0.00325</v>
       </c>
       <c r="J28" s="66"/>
       <c r="K28" s="66"/>
@@ -15304,27 +15411,27 @@
       </c>
       <c r="D29" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" s="64">
         <f>IF(D29,'Post-print worksheet'!C35,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="23" t="str">
+        <v>80</v>
+      </c>
+      <c r="F29" s="23">
         <f>IF(C29, IFERROR(AVERAGE('Post-print worksheet'!D35:F35),""),"")</f>
-        <v/>
+        <v>79.76</v>
       </c>
       <c r="G29" s="23">
         <f>IF(C29, IFERROR(STDEV('Post-print worksheet'!D35:F35),0),"")</f>
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H29" s="23">
         <f>IF(C29, IFERROR(SQRT((Intro!$B$8/3)^2+G29^2),0),"")</f>
-        <v>0.003333333333</v>
-      </c>
-      <c r="I29" s="23" t="str">
+        <v>0.01054092553</v>
+      </c>
+      <c r="I29" s="23">
         <f t="shared" si="3"/>
-        <v/>
+        <v>-0.003</v>
       </c>
       <c r="J29" s="66"/>
       <c r="K29" s="66"/>
@@ -15448,22 +15555,22 @@
       <c r="A36" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="B36" s="73" t="str">
+      <c r="B36" s="73">
         <f>SUM(F24:F27)/SUMPRODUCT(D24:D27*E24:E27)*Intro!$B$4</f>
-        <v>#DIV/0!</v>
+        <v>120.048</v>
       </c>
       <c r="C36" s="74"/>
-      <c r="D36" s="22" t="str">
+      <c r="D36" s="22">
         <f>SQRT(SUMSQ(H24:H27))/SUMPRODUCT(D24:D27*E24:E27)*Intro!$B$4</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E36" s="23" t="str">
+        <v>0.02068816087</v>
+      </c>
+      <c r="E36" s="23">
         <f>-B36/(2*B38*B39*SIN(B41*PI()/180))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F36" s="24" t="str">
+        <v>-0.008348545381</v>
+      </c>
+      <c r="F36" s="24">
         <f t="shared" ref="F36:F39" si="6">D36*E36</f>
-        <v>#DIV/0!</v>
+        <v>-0.0001727160498</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
@@ -15473,22 +15580,22 @@
       <c r="A37" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="B37" s="73" t="str">
+      <c r="B37" s="73">
         <f>SUM(F28:F31)/SUMPRODUCT(D28:D31*E28:E31)*Intro!$B$4</f>
-        <v>#DIV/0!</v>
+        <v>119.622</v>
       </c>
       <c r="C37" s="74"/>
-      <c r="D37" s="22" t="str">
+      <c r="D37" s="22">
         <f>SQRT(SUMSQ(H28:H31))/SUMPRODUCT(D28:D31*E28:E31)*Intro!$B$4</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E37" s="23" t="str">
+        <v>0.01232882801</v>
+      </c>
+      <c r="E37" s="23">
         <f>B37/(2*B38*B39*SIN(B41*PI()/180))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F37" s="24" t="str">
+        <v>0.008318919895</v>
+      </c>
+      <c r="F37" s="24">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0.0001025625326</v>
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
@@ -15497,22 +15604,22 @@
       <c r="A38" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B38" s="73" t="str">
+      <c r="B38" s="73">
         <f>SQRT(2)*Intro!B4/2*SUM(F4:F8)/(SUMPRODUCT(D4:D8*E4:E8))</f>
-        <v>#DIV/0!</v>
+        <v>84.84574267</v>
       </c>
       <c r="C38" s="74"/>
-      <c r="D38" s="22" t="str">
+      <c r="D38" s="22">
         <f>SQRT(2)*Intro!B4/2*SQRT(SUMSQ(H4:H8))/(SUMPRODUCT(D4:D8*E4:E8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E38" s="23" t="str">
+        <v>0.055</v>
+      </c>
+      <c r="E38" s="23">
         <f>(B36^2-B37^2)/(4*B38^2*B39*SIN(B41*PI()/180))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F38" s="24" t="str">
+        <v>0.0000418426428</v>
+      </c>
+      <c r="F38" s="24">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0.000002301345354</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
@@ -15521,22 +15628,22 @@
       <c r="A39" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="B39" s="73" t="str">
+      <c r="B39" s="73">
         <f>SQRT(2)*Intro!B4/2*SUM(F14:F18)/(SUMPRODUCT(D14:D18*E14:E18))</f>
-        <v>#DIV/0!</v>
+        <v>84.73967666</v>
       </c>
       <c r="C39" s="74"/>
-      <c r="D39" s="28" t="str">
+      <c r="D39" s="28">
         <f>SQRT(2)*Intro!B4/2*SQRT(SUMSQ(H14:H18))/(SUMPRODUCT(D14:D18*E14:E18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E39" s="29" t="str">
+        <v>0.01118033989</v>
+      </c>
+      <c r="E39" s="29">
         <f>(B36^2-B37^2)/(4*B38*B39^2*SIN(B41*PI()/180))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F39" s="30" t="str">
+        <v>0.00004189501594</v>
+      </c>
+      <c r="F39" s="30">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0.0000004684005178</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
@@ -15545,9 +15652,9 @@
       <c r="A40" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="B40" s="76" t="str">
+      <c r="B40" s="76">
         <f>(B36^2-B37^2)/(4*B38*B39)</f>
-        <v>#DIV/0!</v>
+        <v>0.003550147731</v>
       </c>
       <c r="C40" s="75"/>
       <c r="D40" s="75"/>
@@ -15560,9 +15667,9 @@
       <c r="A41" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="B41" s="76" t="str">
+      <c r="B41" s="76">
         <f>ACOS(B40)*180/PI()</f>
-        <v>#DIV/0!</v>
+        <v>89.79659109</v>
       </c>
       <c r="C41" s="75"/>
       <c r="D41" s="75"/>
@@ -15575,9 +15682,9 @@
       <c r="A42" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B42" s="76" t="str">
+      <c r="B42" s="76">
         <f>B41-90</f>
-        <v>#DIV/0!</v>
+        <v>-0.2034089089</v>
       </c>
       <c r="C42" s="75"/>
       <c r="D42" s="75" t="s">
@@ -15596,21 +15703,21 @@
       <c r="A43" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="B43" s="77" t="str">
+      <c r="B43" s="77">
         <f>SQRT(SUMSQ(F36:F39))*180/PI()</f>
-        <v>#DIV/0!</v>
+        <v>0.01150995384</v>
       </c>
       <c r="C43" s="75"/>
       <c r="D43" s="75" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="23" t="str">
+      <c r="E43" s="23">
         <f>AVERAGE(I4:I13)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F43" s="1" t="str">
+        <v>-0.000412037037</v>
+      </c>
+      <c r="F43" s="1">
         <f>Intro!B6*(SUM(F4:F13))/SUMPRODUCT(E4:E13*D4:D13)</f>
-        <v>#DIV/0!</v>
+        <v>39.97888889</v>
       </c>
       <c r="G43" s="75"/>
       <c r="H43" s="75"/>
@@ -15620,13 +15727,13 @@
       <c r="D44" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="78" t="str">
+      <c r="E44" s="78">
         <f>AVERAGE(I14:I23)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F44" s="6" t="str">
+        <v>-0.001328703704</v>
+      </c>
+      <c r="F44" s="6">
         <f>Intro!B6*(SUM(F14:F23))/SUMPRODUCT(E14:E23*D14:D23)</f>
-        <v>#DIV/0!</v>
+        <v>39.95</v>
       </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
@@ -15653,7 +15760,7 @@
       </c>
       <c r="B47" s="79">
         <f>COUNTIF(D4:D8, TRUE())</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
@@ -15665,7 +15772,7 @@
       </c>
       <c r="B48" s="79">
         <f>COUNTIF(D9:D13, TRUE())</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
@@ -15676,7 +15783,7 @@
       </c>
       <c r="B49" s="79">
         <f>COUNTIF(D14:D18, TRUE())</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
@@ -15687,7 +15794,7 @@
       </c>
       <c r="B50" s="79">
         <f>COUNTIF(D19:D23, TRUE())</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
@@ -15698,7 +15805,7 @@
       </c>
       <c r="B51" s="79">
         <f>COUNTIF(D24:D27, TRUE())</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
@@ -15709,7 +15816,7 @@
       </c>
       <c r="B52" s="81">
         <f>COUNTIF(D28:D31, TRUE())</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>

</xml_diff>

<commit_message>
Remove data that was in spreadsheet
</commit_message>
<xml_diff>
--- a/Parametric Skew Calibration.xlsx
+++ b/Parametric Skew Calibration.xlsx
@@ -5308,18 +5308,12 @@
         <f>IF(Helper!C4,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D10" s="12">
-        <v>119.91</v>
-      </c>
-      <c r="E10" s="13">
-        <v>119.89</v>
-      </c>
-      <c r="F10" s="14">
-        <v>119.93</v>
-      </c>
-      <c r="G10" s="15">
+      <c r="D10" s="12"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="15" t="str">
         <f t="shared" ref="G10:G37" si="1">IF(OR(B10="",ISBLANK(D10)), "", AVERAGE(D10:F10))</f>
-        <v>119.91</v>
+        <v/>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -5332,18 +5326,12 @@
         <f>IF(Helper!C5,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D11" s="18">
-        <v>79.92</v>
-      </c>
-      <c r="E11" s="19">
-        <v>80.2</v>
-      </c>
-      <c r="F11" s="20">
-        <v>79.98</v>
-      </c>
-      <c r="G11" s="21">
+      <c r="D11" s="18"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>80.03333333</v>
+        <v/>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -5356,21 +5344,15 @@
         <f>IF(Helper!C6, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D12" s="18">
-        <v>40.08</v>
-      </c>
-      <c r="E12" s="19">
-        <v>39.99</v>
-      </c>
-      <c r="F12" s="20">
-        <v>40.04</v>
-      </c>
-      <c r="G12" s="21">
+      <c r="D12" s="18"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>40.03666667</v>
-      </c>
-    </row>
-    <row r="13" ht="15.75" hidden="1" customHeight="1">
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="16"/>
       <c r="B13" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
@@ -5388,7 +5370,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="15.75" hidden="1" customHeight="1">
+    <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="25"/>
       <c r="B14" s="26" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
@@ -5418,18 +5400,12 @@
         <f>IF(Helper!C9,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D15" s="12">
-        <v>119.9</v>
-      </c>
-      <c r="E15" s="13">
-        <v>119.85</v>
-      </c>
-      <c r="F15" s="14">
-        <v>119.9</v>
-      </c>
-      <c r="G15" s="15">
+      <c r="D15" s="12"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="15" t="str">
         <f t="shared" si="1"/>
-        <v>119.8833333</v>
+        <v/>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -5442,18 +5418,12 @@
         <f>IF(Helper!C10,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D16" s="18">
-        <v>79.9</v>
-      </c>
-      <c r="E16" s="19">
-        <v>79.94</v>
-      </c>
-      <c r="F16" s="20">
-        <v>79.96</v>
-      </c>
-      <c r="G16" s="21">
+      <c r="D16" s="18"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>79.93333333</v>
+        <v/>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
@@ -5466,21 +5436,15 @@
         <f>IF(Helper!C11, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D17" s="18">
-        <v>39.9</v>
-      </c>
-      <c r="E17" s="19">
-        <v>39.96</v>
-      </c>
-      <c r="F17" s="20">
-        <v>39.99</v>
-      </c>
-      <c r="G17" s="21">
+      <c r="D17" s="18"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>39.95</v>
-      </c>
-    </row>
-    <row r="18" ht="15.75" hidden="1" customHeight="1">
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="16"/>
       <c r="B18" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
@@ -5498,7 +5462,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="15.75" hidden="1" customHeight="1">
+    <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="25"/>
       <c r="B19" s="26" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
@@ -5528,18 +5492,12 @@
         <f>IF(Helper!C14,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D20" s="12">
-        <v>119.8</v>
-      </c>
-      <c r="E20" s="13">
-        <v>119.81</v>
-      </c>
-      <c r="F20" s="14">
-        <v>119.85</v>
-      </c>
-      <c r="G20" s="15">
+      <c r="D20" s="12"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="15" t="str">
         <f t="shared" si="1"/>
-        <v>119.82</v>
+        <v/>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -5552,18 +5510,12 @@
         <f>IF(Helper!C15,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D21" s="18">
-        <v>79.9</v>
-      </c>
-      <c r="E21" s="19">
-        <v>79.93</v>
-      </c>
-      <c r="F21" s="20">
-        <v>79.92</v>
-      </c>
-      <c r="G21" s="21">
+      <c r="D21" s="18"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>79.91666667</v>
+        <v/>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -5576,21 +5528,15 @@
         <f>IF(Helper!C16, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D22" s="18">
-        <v>39.94</v>
-      </c>
-      <c r="E22" s="19">
-        <v>39.94</v>
-      </c>
-      <c r="F22" s="20">
-        <v>39.95</v>
-      </c>
-      <c r="G22" s="21">
+      <c r="D22" s="18"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>39.94333333</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" hidden="1" customHeight="1">
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="16"/>
       <c r="B23" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
@@ -5608,7 +5554,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="15.75" hidden="1" customHeight="1">
+    <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="25"/>
       <c r="B24" s="26" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
@@ -5638,18 +5584,12 @@
         <f>IF(Helper!C19,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D25" s="12">
-        <v>119.91</v>
-      </c>
-      <c r="E25" s="13">
-        <v>119.86</v>
-      </c>
-      <c r="F25" s="14">
-        <v>119.91</v>
-      </c>
-      <c r="G25" s="15">
+      <c r="D25" s="12"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="15" t="str">
         <f t="shared" si="1"/>
-        <v>119.8933333</v>
+        <v/>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -5662,18 +5602,12 @@
         <f>IF(Helper!C20,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D26" s="18">
-        <v>79.85</v>
-      </c>
-      <c r="E26" s="19">
-        <v>79.88</v>
-      </c>
-      <c r="F26" s="20">
-        <v>79.98</v>
-      </c>
-      <c r="G26" s="21">
+      <c r="D26" s="18"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>79.90333333</v>
+        <v/>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -5686,21 +5620,15 @@
         <f>IF(Helper!C21, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D27" s="18">
-        <v>39.85</v>
-      </c>
-      <c r="E27" s="19">
-        <v>39.94</v>
-      </c>
-      <c r="F27" s="20">
-        <v>39.98</v>
-      </c>
-      <c r="G27" s="21">
+      <c r="D27" s="18"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>39.92333333</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" hidden="1" customHeight="1">
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="16"/>
       <c r="B28" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
@@ -5718,7 +5646,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="15.75" hidden="1" customHeight="1">
+    <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="16"/>
       <c r="B29" s="1" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
@@ -5748,18 +5676,12 @@
         <f>IF(Helper!C24,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D30" s="12">
-        <v>120.04</v>
-      </c>
-      <c r="E30" s="13">
-        <v>120.02</v>
-      </c>
-      <c r="F30" s="14">
-        <v>119.98</v>
-      </c>
-      <c r="G30" s="33">
+      <c r="D30" s="12"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="33" t="str">
         <f t="shared" si="1"/>
-        <v>120.0133333</v>
+        <v/>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
@@ -5772,21 +5694,15 @@
         <f>IF(Helper!C25,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D31" s="18">
-        <v>80.07</v>
-      </c>
-      <c r="E31" s="19">
-        <v>80.05</v>
-      </c>
-      <c r="F31" s="20">
-        <v>80.08</v>
-      </c>
-      <c r="G31" s="21">
+      <c r="D31" s="18"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>80.06666667</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" hidden="1" customHeight="1">
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="16"/>
       <c r="B32" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 3, "")</f>
@@ -5804,7 +5720,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="15.75" hidden="1" customHeight="1">
+    <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="16"/>
       <c r="B33" s="1" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
@@ -5834,18 +5750,12 @@
         <f>IF(Helper!C28,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D34" s="12">
-        <v>119.62</v>
-      </c>
-      <c r="E34" s="13">
-        <v>119.59</v>
-      </c>
-      <c r="F34" s="14">
-        <v>119.62</v>
-      </c>
-      <c r="G34" s="33">
+      <c r="D34" s="12"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="33" t="str">
         <f t="shared" si="1"/>
-        <v>119.61</v>
+        <v/>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
@@ -5858,21 +5768,15 @@
         <f>IF(Helper!C29,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D35" s="18">
-        <v>79.76</v>
-      </c>
-      <c r="E35" s="19">
-        <v>79.75</v>
-      </c>
-      <c r="F35" s="20">
-        <v>79.77</v>
-      </c>
-      <c r="G35" s="34">
+      <c r="D35" s="18"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="34" t="str">
         <f t="shared" si="1"/>
-        <v>79.76</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" hidden="1" customHeight="1">
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="16"/>
       <c r="B36" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 3, "")</f>
@@ -5890,7 +5794,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="15.75" hidden="1" customHeight="1">
+    <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="25"/>
       <c r="B37" s="26" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
@@ -10955,15 +10859,7 @@
       <c r="C1035" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="$C$9:$C$37">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="40.00"/>
-        <filter val="120.00"/>
-        <filter val="80.00"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="$C$9:$C$37"/>
   <conditionalFormatting sqref="D10:F38">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>LEN(TRIM(D10))=0</formula>
@@ -11044,17 +10940,17 @@
         <v>46</v>
       </c>
       <c r="B4" s="40"/>
-      <c r="C4" s="40">
+      <c r="C4" s="40" t="str">
         <f>Helper!E43</f>
-        <v>-0.000412037037</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="D4" s="44">
         <f>SQRT(SUMSQ(Helper!K4:K13))</f>
-        <v>0.0004159845239</v>
-      </c>
-      <c r="E4" s="45">
+        <v>0</v>
+      </c>
+      <c r="E4" s="45" t="str">
         <f t="shared" ref="E4:E5" si="1">-C4</f>
-        <v>0.000412037037</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G4" s="46" t="s">
         <v>47</v>
@@ -11068,17 +10964,17 @@
         <v>48</v>
       </c>
       <c r="B5" s="40"/>
-      <c r="C5" s="40">
+      <c r="C5" s="40" t="str">
         <f>Helper!E44</f>
-        <v>-0.001328703704</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="D5" s="44">
         <f>SQRT(SUMSQ(Helper!K14:K23))</f>
-        <v>0.0003196121406</v>
-      </c>
-      <c r="E5" s="45">
+        <v>0</v>
+      </c>
+      <c r="E5" s="45" t="str">
         <f t="shared" si="1"/>
-        <v>0.001328703704</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G5" s="48" t="s">
         <v>49</v>
@@ -11124,13 +11020,13 @@
         <v>54</v>
       </c>
       <c r="B8" s="23"/>
-      <c r="C8" s="23">
+      <c r="C8" s="23" t="str">
         <f>Helper!B41</f>
-        <v>89.79659109</v>
-      </c>
-      <c r="D8" s="54">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D8" s="54" t="str">
         <f>Helper!B43</f>
-        <v>0.01150995384</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="E8" s="24"/>
       <c r="G8" s="55" t="s">
@@ -11145,17 +11041,17 @@
         <v>56</v>
       </c>
       <c r="B9" s="29"/>
-      <c r="C9" s="29">
+      <c r="C9" s="29" t="str">
         <f>C8-90</f>
-        <v>-0.2034089089</v>
-      </c>
-      <c r="D9" s="58">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D9" s="58" t="str">
         <f>Helper!B43</f>
-        <v>0.01150995384</v>
-      </c>
-      <c r="E9" s="30">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E9" s="30" t="str">
         <f>-C9</f>
-        <v>0.2034089089</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="J9" s="23"/>
     </row>
@@ -11205,14 +11101,14 @@
       <c r="H14" s="16"/>
       <c r="I14" s="1" t="str">
         <f>"M92 X"&amp;ROUND(Helper!F43,3)&amp;" Y"&amp;ROUND(Helper!F44,3)</f>
-        <v>M92 X39.979 Y39.95</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="M14" s="41"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="22" t="str">
         <f>"Length AC = "&amp;ROUND(Helper!B36,2)</f>
-        <v>Length AC = 120.05</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="41"/>
@@ -11224,7 +11120,7 @@
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="22" t="str">
         <f>"Length BD = "&amp;ROUND(Helper!B37,2)</f>
-        <v>Length BD = 119.62</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="F16" s="41"/>
       <c r="H16" s="16" t="s">
@@ -11235,7 +11131,7 @@
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="22" t="str">
         <f>"Length AD = "&amp;ROUND(Helper!B38,2)</f>
-        <v>Length AD = 84.85</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="F17" s="41"/>
       <c r="H17" s="16"/>
@@ -11244,7 +11140,7 @@
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="18" t="str">
         <f>"CALC_MEASURED_SKEW AC="&amp;ROUND(Helper!B36,2)&amp;" BD="&amp;ROUND(Helper!B37,2)&amp;" AD="&amp;ROUND(Helper!B38,2)</f>
-        <v>CALC_MEASURED_SKEW AC=120.05 BD=119.62 AD=84.85</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="F18" s="41"/>
       <c r="H18" s="16" t="s">
@@ -11264,9 +11160,9 @@
       <c r="A20" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="1" t="str">
         <f>ROUND(Helper!F43,3)</f>
-        <v>39.979</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>68</v>
@@ -11279,9 +11175,9 @@
       <c r="A21" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="B21" s="26">
+      <c r="B21" s="26" t="str">
         <f>ROUND(Helper!F44,3)</f>
-        <v>39.95</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C21" s="26" t="s">
         <v>69</v>
@@ -14357,35 +14253,35 @@
       </c>
       <c r="D4" s="8" t="b">
         <f t="shared" ref="D4:D31" si="2">IFERROR(AND(NOT(F4=0),NOT(F4=""),C4),FALSE())</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" s="62">
         <f>IF(D4,'Post-print worksheet'!C10,0)</f>
-        <v>120</v>
-      </c>
-      <c r="F4" s="63">
+        <v>0</v>
+      </c>
+      <c r="F4" s="63" t="str">
         <f>IF(C4, IFERROR(AVERAGE('Post-print worksheet'!D10:F10),""),"")</f>
-        <v>119.91</v>
+        <v/>
       </c>
       <c r="G4" s="63">
         <f>IF(C4, IFERROR(STDEV('Post-print worksheet'!D10:F10),0),"")</f>
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H4" s="63">
         <f>IF(C4, IFERROR(SQRT((Intro!$B$8/3)^2+G4^2),0),"")</f>
-        <v>0.0202758751</v>
-      </c>
-      <c r="I4" s="63">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I4" s="63" t="str">
         <f t="shared" ref="I4:I31" si="3">IF(D4, IFERROR((F4-E4)/E4,0),"")</f>
-        <v>-0.00075</v>
-      </c>
-      <c r="J4" s="63">
+        <v/>
+      </c>
+      <c r="J4" s="63" t="str">
         <f t="shared" ref="J4:J22" si="4">IF(D4, 1/(($B$47+$B$48)*E4),"")</f>
-        <v>0.001388888889</v>
-      </c>
-      <c r="K4" s="63">
+        <v/>
+      </c>
+      <c r="K4" s="63" t="str">
         <f t="shared" ref="K4:K23" si="5">IF(D4,J4*H4,"")</f>
-        <v>0.00002816093764</v>
+        <v/>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -14400,35 +14296,35 @@
       </c>
       <c r="D5" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="64">
         <f>IF(D5,'Post-print worksheet'!C11,0)</f>
-        <v>80</v>
-      </c>
-      <c r="F5" s="23">
+        <v>0</v>
+      </c>
+      <c r="F5" s="23" t="str">
         <f>IF(C5, IFERROR(AVERAGE('Post-print worksheet'!D11:F11),""),"")</f>
-        <v>80.03333333</v>
+        <v/>
       </c>
       <c r="G5" s="23">
         <f>IF(C5, IFERROR(STDEV('Post-print worksheet'!D11:F11),0),"")</f>
-        <v>0.1474222959</v>
+        <v>0</v>
       </c>
       <c r="H5" s="23">
         <f>IF(C5, IFERROR(SQRT((Intro!$B$8/3)^2+G5^2),0),"")</f>
-        <v>0.1474599757</v>
-      </c>
-      <c r="I5" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I5" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>0.0004166666667</v>
-      </c>
-      <c r="J5" s="23">
+        <v/>
+      </c>
+      <c r="J5" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.002083333333</v>
-      </c>
-      <c r="K5" s="23">
+        <v/>
+      </c>
+      <c r="K5" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.0003072082828</v>
+        <v/>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -14443,35 +14339,35 @@
       </c>
       <c r="D6" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="64">
         <f>IF(D6,'Post-print worksheet'!C12,0)</f>
-        <v>40</v>
-      </c>
-      <c r="F6" s="23">
+        <v>0</v>
+      </c>
+      <c r="F6" s="23" t="str">
         <f>IF(C6, IFERROR(AVERAGE('Post-print worksheet'!D12:F12),""),"")</f>
-        <v>40.03666667</v>
+        <v/>
       </c>
       <c r="G6" s="23">
         <f>IF(C6, IFERROR(STDEV('Post-print worksheet'!D12:F12),0),"")</f>
-        <v>0.04509249753</v>
+        <v>0</v>
       </c>
       <c r="H6" s="23">
         <f>IF(C6, IFERROR(SQRT((Intro!$B$8/3)^2+G6^2),0),"")</f>
-        <v>0.04521553322</v>
-      </c>
-      <c r="I6" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I6" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>0.0009166666667</v>
-      </c>
-      <c r="J6" s="23">
+        <v/>
+      </c>
+      <c r="J6" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.004166666667</v>
-      </c>
-      <c r="K6" s="23">
+        <v/>
+      </c>
+      <c r="K6" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.0001883980551</v>
+        <v/>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -14574,35 +14470,35 @@
       </c>
       <c r="D9" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="64">
         <f>IF(D9,'Post-print worksheet'!C15,0)</f>
-        <v>120</v>
-      </c>
-      <c r="F9" s="23">
+        <v>0</v>
+      </c>
+      <c r="F9" s="23" t="str">
         <f>IF(C9, IFERROR(AVERAGE('Post-print worksheet'!D15:F15),""),"")</f>
-        <v>119.8833333</v>
+        <v/>
       </c>
       <c r="G9" s="23">
         <f>IF(C9, IFERROR(STDEV('Post-print worksheet'!D15:F15),0),"")</f>
-        <v>0.02886751346</v>
+        <v>0</v>
       </c>
       <c r="H9" s="23">
         <f>IF(C9, IFERROR(SQRT((Intro!$B$8/3)^2+G9^2),0),"")</f>
-        <v>0.02905932629</v>
-      </c>
-      <c r="I9" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I9" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.0009722222222</v>
-      </c>
-      <c r="J9" s="23">
+        <v/>
+      </c>
+      <c r="J9" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.001388888889</v>
-      </c>
-      <c r="K9" s="23">
+        <v/>
+      </c>
+      <c r="K9" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.0000403601754</v>
+        <v/>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -14617,35 +14513,35 @@
       </c>
       <c r="D10" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="64">
         <f>IF(D10,'Post-print worksheet'!C16,0)</f>
-        <v>80</v>
-      </c>
-      <c r="F10" s="23">
+        <v>0</v>
+      </c>
+      <c r="F10" s="23" t="str">
         <f>IF(C10, IFERROR(AVERAGE('Post-print worksheet'!D16:F16),""),"")</f>
-        <v>79.93333333</v>
+        <v/>
       </c>
       <c r="G10" s="23">
         <f>IF(C10, IFERROR(STDEV('Post-print worksheet'!D16:F16),0),"")</f>
-        <v>0.03055050463</v>
+        <v>0</v>
       </c>
       <c r="H10" s="23">
         <f>IF(C10, IFERROR(SQRT((Intro!$B$8/3)^2+G10^2),0),"")</f>
-        <v>0.03073181486</v>
-      </c>
-      <c r="I10" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I10" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.0008333333333</v>
-      </c>
-      <c r="J10" s="23">
+        <v/>
+      </c>
+      <c r="J10" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.002083333333</v>
-      </c>
-      <c r="K10" s="23">
+        <v/>
+      </c>
+      <c r="K10" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.00006402461429</v>
+        <v/>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -14660,35 +14556,35 @@
       </c>
       <c r="D11" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" s="64">
         <f>IF(D11,'Post-print worksheet'!C17,0)</f>
-        <v>40</v>
-      </c>
-      <c r="F11" s="23">
+        <v>0</v>
+      </c>
+      <c r="F11" s="23" t="str">
         <f>IF(C11, IFERROR(AVERAGE('Post-print worksheet'!D17:F17),""),"")</f>
-        <v>39.95</v>
+        <v/>
       </c>
       <c r="G11" s="23">
         <f>IF(C11, IFERROR(STDEV('Post-print worksheet'!D17:F17),0),"")</f>
-        <v>0.04582575695</v>
+        <v>0</v>
       </c>
       <c r="H11" s="23">
         <f>IF(C11, IFERROR(SQRT((Intro!$B$8/3)^2+G11^2),0),"")</f>
-        <v>0.04594682917</v>
-      </c>
-      <c r="I11" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I11" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.00125</v>
-      </c>
-      <c r="J11" s="23">
+        <v/>
+      </c>
+      <c r="J11" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.004166666667</v>
-      </c>
-      <c r="K11" s="23">
+        <v/>
+      </c>
+      <c r="K11" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.0001914451216</v>
+        <v/>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -14791,35 +14687,35 @@
       </c>
       <c r="D14" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="64">
         <f>IF(D14,'Post-print worksheet'!C20,0)</f>
-        <v>120</v>
-      </c>
-      <c r="F14" s="23">
+        <v>0</v>
+      </c>
+      <c r="F14" s="23" t="str">
         <f>IF(C14, IFERROR(AVERAGE('Post-print worksheet'!D20:F20),""),"")</f>
-        <v>119.82</v>
+        <v/>
       </c>
       <c r="G14" s="23">
         <f>IF(C14, IFERROR(STDEV('Post-print worksheet'!D20:F20),0),"")</f>
-        <v>0.02645751311</v>
+        <v>0</v>
       </c>
       <c r="H14" s="23">
         <f>IF(C14, IFERROR(SQRT((Intro!$B$8/3)^2+G14^2),0),"")</f>
-        <v>0.02666666667</v>
-      </c>
-      <c r="I14" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I14" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.0015</v>
-      </c>
-      <c r="J14" s="23">
+        <v/>
+      </c>
+      <c r="J14" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.001388888889</v>
-      </c>
-      <c r="K14" s="23">
+        <v/>
+      </c>
+      <c r="K14" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.00003703703704</v>
+        <v/>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
@@ -14834,35 +14730,35 @@
       </c>
       <c r="D15" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="64">
         <f>IF(D15,'Post-print worksheet'!C21,0)</f>
-        <v>80</v>
-      </c>
-      <c r="F15" s="23">
+        <v>0</v>
+      </c>
+      <c r="F15" s="23" t="str">
         <f>IF(C15, IFERROR(AVERAGE('Post-print worksheet'!D21:F21),""),"")</f>
-        <v>79.91666667</v>
+        <v/>
       </c>
       <c r="G15" s="23">
         <f>IF(C15, IFERROR(STDEV('Post-print worksheet'!D21:F21),0),"")</f>
-        <v>0.01527525232</v>
+        <v>0</v>
       </c>
       <c r="H15" s="23">
         <f>IF(C15, IFERROR(SQRT((Intro!$B$8/3)^2+G15^2),0),"")</f>
-        <v>0.0156347192</v>
-      </c>
-      <c r="I15" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I15" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.001041666667</v>
-      </c>
-      <c r="J15" s="23">
+        <v/>
+      </c>
+      <c r="J15" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.002083333333</v>
-      </c>
-      <c r="K15" s="23">
+        <v/>
+      </c>
+      <c r="K15" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.00003257233167</v>
+        <v/>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -14877,35 +14773,35 @@
       </c>
       <c r="D16" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" s="64">
         <f>IF(D16,'Post-print worksheet'!C22,0)</f>
-        <v>40</v>
-      </c>
-      <c r="F16" s="23">
+        <v>0</v>
+      </c>
+      <c r="F16" s="23" t="str">
         <f>IF(C16, IFERROR(AVERAGE('Post-print worksheet'!D22:F22),""),"")</f>
-        <v>39.94333333</v>
+        <v/>
       </c>
       <c r="G16" s="23">
         <f>IF(C16, IFERROR(STDEV('Post-print worksheet'!D22:F22),0),"")</f>
-        <v>0.005773502692</v>
+        <v>0</v>
       </c>
       <c r="H16" s="23">
         <f>IF(C16, IFERROR(SQRT((Intro!$B$8/3)^2+G16^2),0),"")</f>
-        <v>0.006666666667</v>
-      </c>
-      <c r="I16" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I16" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.001416666667</v>
-      </c>
-      <c r="J16" s="23">
+        <v/>
+      </c>
+      <c r="J16" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.004166666667</v>
-      </c>
-      <c r="K16" s="23">
+        <v/>
+      </c>
+      <c r="K16" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.00002777777778</v>
+        <v/>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
@@ -15008,35 +14904,35 @@
       </c>
       <c r="D19" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" s="64">
         <f>IF(D19,'Post-print worksheet'!C25,0)</f>
-        <v>120</v>
-      </c>
-      <c r="F19" s="23">
+        <v>0</v>
+      </c>
+      <c r="F19" s="23" t="str">
         <f>IF(C19, IFERROR(AVERAGE('Post-print worksheet'!D25:F25),""),"")</f>
-        <v>119.8933333</v>
+        <v/>
       </c>
       <c r="G19" s="23">
         <f>IF(C19, IFERROR(STDEV('Post-print worksheet'!D25:F25),0),"")</f>
-        <v>0.02886751346</v>
+        <v>0</v>
       </c>
       <c r="H19" s="23">
         <f>IF(C19, IFERROR(SQRT((Intro!$B$8/3)^2+G19^2),0),"")</f>
-        <v>0.02905932629</v>
-      </c>
-      <c r="I19" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I19" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.0008888888889</v>
-      </c>
-      <c r="J19" s="23">
+        <v/>
+      </c>
+      <c r="J19" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.001388888889</v>
-      </c>
-      <c r="K19" s="23">
+        <v/>
+      </c>
+      <c r="K19" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.0000403601754</v>
+        <v/>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
@@ -15051,35 +14947,35 @@
       </c>
       <c r="D20" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" s="64">
         <f>IF(D20,'Post-print worksheet'!C26,0)</f>
-        <v>80</v>
-      </c>
-      <c r="F20" s="23">
+        <v>0</v>
+      </c>
+      <c r="F20" s="23" t="str">
         <f>IF(C20, IFERROR(AVERAGE('Post-print worksheet'!D26:F26),""),"")</f>
-        <v>79.90333333</v>
+        <v/>
       </c>
       <c r="G20" s="23">
         <f>IF(C20, IFERROR(STDEV('Post-print worksheet'!D26:F26),0),"")</f>
-        <v>0.06806859286</v>
+        <v>0</v>
       </c>
       <c r="H20" s="23">
         <f>IF(C20, IFERROR(SQRT((Intro!$B$8/3)^2+G20^2),0),"")</f>
-        <v>0.068150161</v>
-      </c>
-      <c r="I20" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I20" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.001208333333</v>
-      </c>
-      <c r="J20" s="23">
+        <v/>
+      </c>
+      <c r="J20" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.002083333333</v>
-      </c>
-      <c r="K20" s="23">
+        <v/>
+      </c>
+      <c r="K20" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.0001419795021</v>
+        <v/>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -15094,35 +14990,35 @@
       </c>
       <c r="D21" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" s="64">
         <f>IF(D21,'Post-print worksheet'!C27,0)</f>
-        <v>40</v>
-      </c>
-      <c r="F21" s="23">
+        <v>0</v>
+      </c>
+      <c r="F21" s="23" t="str">
         <f>IF(C21, IFERROR(AVERAGE('Post-print worksheet'!D27:F27),""),"")</f>
-        <v>39.92333333</v>
+        <v/>
       </c>
       <c r="G21" s="23">
         <f>IF(C21, IFERROR(STDEV('Post-print worksheet'!D27:F27),0),"")</f>
-        <v>0.06658328118</v>
+        <v>0</v>
       </c>
       <c r="H21" s="23">
         <f>IF(C21, IFERROR(SQRT((Intro!$B$8/3)^2+G21^2),0),"")</f>
-        <v>0.06666666667</v>
-      </c>
-      <c r="I21" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I21" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.001916666667</v>
-      </c>
-      <c r="J21" s="23">
+        <v/>
+      </c>
+      <c r="J21" s="23" t="str">
         <f t="shared" si="4"/>
-        <v>0.004166666667</v>
-      </c>
-      <c r="K21" s="23">
+        <v/>
+      </c>
+      <c r="K21" s="23" t="str">
         <f t="shared" si="5"/>
-        <v>0.0002777777778</v>
+        <v/>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -15225,27 +15121,27 @@
       </c>
       <c r="D24" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E24" s="64">
         <f>IF(D24,'Post-print worksheet'!C30,0)</f>
-        <v>120</v>
-      </c>
-      <c r="F24" s="23">
+        <v>0</v>
+      </c>
+      <c r="F24" s="23" t="str">
         <f>IF(C24, IFERROR(AVERAGE('Post-print worksheet'!D30:F30),""),"")</f>
-        <v>120.0133333</v>
+        <v/>
       </c>
       <c r="G24" s="23">
         <f>IF(C24, IFERROR(STDEV('Post-print worksheet'!D30:F30),0),"")</f>
-        <v>0.03055050463</v>
+        <v>0</v>
       </c>
       <c r="H24" s="23">
         <f>IF(C24, IFERROR(SQRT((Intro!$B$8/3)^2+G24^2),0),"")</f>
-        <v>0.03073181486</v>
-      </c>
-      <c r="I24" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I24" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>0.0001111111111</v>
+        <v/>
       </c>
       <c r="J24" s="66"/>
       <c r="K24" s="66"/>
@@ -15262,27 +15158,27 @@
       </c>
       <c r="D25" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="64">
         <f>IF(D25,'Post-print worksheet'!C31,0)</f>
-        <v>80</v>
-      </c>
-      <c r="F25" s="23">
+        <v>0</v>
+      </c>
+      <c r="F25" s="23" t="str">
         <f>IF(C25, IFERROR(AVERAGE('Post-print worksheet'!D31:F31),""),"")</f>
-        <v>80.06666667</v>
+        <v/>
       </c>
       <c r="G25" s="23">
         <f>IF(C25, IFERROR(STDEV('Post-print worksheet'!D31:F31),0),"")</f>
-        <v>0.01527525232</v>
+        <v>0</v>
       </c>
       <c r="H25" s="23">
         <f>IF(C25, IFERROR(SQRT((Intro!$B$8/3)^2+G25^2),0),"")</f>
-        <v>0.0156347192</v>
-      </c>
-      <c r="I25" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I25" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>0.0008333333333</v>
+        <v/>
       </c>
       <c r="J25" s="66"/>
       <c r="K25" s="66"/>
@@ -15375,27 +15271,27 @@
       </c>
       <c r="D28" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" s="64">
         <f>IF(D28,'Post-print worksheet'!C34,0)</f>
-        <v>120</v>
-      </c>
-      <c r="F28" s="23">
+        <v>0</v>
+      </c>
+      <c r="F28" s="23" t="str">
         <f>IF(C28, IFERROR(AVERAGE('Post-print worksheet'!D34:F34),""),"")</f>
-        <v>119.61</v>
+        <v/>
       </c>
       <c r="G28" s="23">
         <f>IF(C28, IFERROR(STDEV('Post-print worksheet'!D34:F34),0),"")</f>
-        <v>0.01732050808</v>
+        <v>0</v>
       </c>
       <c r="H28" s="23">
         <f>IF(C28, IFERROR(SQRT((Intro!$B$8/3)^2+G28^2),0),"")</f>
-        <v>0.01763834207</v>
-      </c>
-      <c r="I28" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I28" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.00325</v>
+        <v/>
       </c>
       <c r="J28" s="66"/>
       <c r="K28" s="66"/>
@@ -15411,27 +15307,27 @@
       </c>
       <c r="D29" s="1" t="b">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" s="64">
         <f>IF(D29,'Post-print worksheet'!C35,0)</f>
-        <v>80</v>
-      </c>
-      <c r="F29" s="23">
+        <v>0</v>
+      </c>
+      <c r="F29" s="23" t="str">
         <f>IF(C29, IFERROR(AVERAGE('Post-print worksheet'!D35:F35),""),"")</f>
-        <v>79.76</v>
+        <v/>
       </c>
       <c r="G29" s="23">
         <f>IF(C29, IFERROR(STDEV('Post-print worksheet'!D35:F35),0),"")</f>
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H29" s="23">
         <f>IF(C29, IFERROR(SQRT((Intro!$B$8/3)^2+G29^2),0),"")</f>
-        <v>0.01054092553</v>
-      </c>
-      <c r="I29" s="23">
+        <v>0.003333333333</v>
+      </c>
+      <c r="I29" s="23" t="str">
         <f t="shared" si="3"/>
-        <v>-0.003</v>
+        <v/>
       </c>
       <c r="J29" s="66"/>
       <c r="K29" s="66"/>
@@ -15555,22 +15451,22 @@
       <c r="A36" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="B36" s="73">
+      <c r="B36" s="73" t="str">
         <f>SUM(F24:F27)/SUMPRODUCT(D24:D27*E24:E27)*Intro!$B$4</f>
-        <v>120.048</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C36" s="74"/>
-      <c r="D36" s="22">
+      <c r="D36" s="22" t="str">
         <f>SQRT(SUMSQ(H24:H27))/SUMPRODUCT(D24:D27*E24:E27)*Intro!$B$4</f>
-        <v>0.02068816087</v>
-      </c>
-      <c r="E36" s="23">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E36" s="23" t="str">
         <f>-B36/(2*B38*B39*SIN(B41*PI()/180))</f>
-        <v>-0.008348545381</v>
-      </c>
-      <c r="F36" s="24">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F36" s="24" t="str">
         <f t="shared" ref="F36:F39" si="6">D36*E36</f>
-        <v>-0.0001727160498</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
@@ -15580,22 +15476,22 @@
       <c r="A37" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="B37" s="73">
+      <c r="B37" s="73" t="str">
         <f>SUM(F28:F31)/SUMPRODUCT(D28:D31*E28:E31)*Intro!$B$4</f>
-        <v>119.622</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C37" s="74"/>
-      <c r="D37" s="22">
+      <c r="D37" s="22" t="str">
         <f>SQRT(SUMSQ(H28:H31))/SUMPRODUCT(D28:D31*E28:E31)*Intro!$B$4</f>
-        <v>0.01232882801</v>
-      </c>
-      <c r="E37" s="23">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E37" s="23" t="str">
         <f>B37/(2*B38*B39*SIN(B41*PI()/180))</f>
-        <v>0.008318919895</v>
-      </c>
-      <c r="F37" s="24">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F37" s="24" t="str">
         <f t="shared" si="6"/>
-        <v>0.0001025625326</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
@@ -15604,22 +15500,22 @@
       <c r="A38" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B38" s="73">
+      <c r="B38" s="73" t="str">
         <f>SQRT(2)*Intro!B4/2*SUM(F4:F8)/(SUMPRODUCT(D4:D8*E4:E8))</f>
-        <v>84.84574267</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C38" s="74"/>
-      <c r="D38" s="22">
+      <c r="D38" s="22" t="str">
         <f>SQRT(2)*Intro!B4/2*SQRT(SUMSQ(H4:H8))/(SUMPRODUCT(D4:D8*E4:E8))</f>
-        <v>0.055</v>
-      </c>
-      <c r="E38" s="23">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E38" s="23" t="str">
         <f>(B36^2-B37^2)/(4*B38^2*B39*SIN(B41*PI()/180))</f>
-        <v>0.0000418426428</v>
-      </c>
-      <c r="F38" s="24">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F38" s="24" t="str">
         <f t="shared" si="6"/>
-        <v>0.000002301345354</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
@@ -15628,22 +15524,22 @@
       <c r="A39" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="B39" s="73">
+      <c r="B39" s="73" t="str">
         <f>SQRT(2)*Intro!B4/2*SUM(F14:F18)/(SUMPRODUCT(D14:D18*E14:E18))</f>
-        <v>84.73967666</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C39" s="74"/>
-      <c r="D39" s="28">
+      <c r="D39" s="28" t="str">
         <f>SQRT(2)*Intro!B4/2*SQRT(SUMSQ(H14:H18))/(SUMPRODUCT(D14:D18*E14:E18))</f>
-        <v>0.01118033989</v>
-      </c>
-      <c r="E39" s="29">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E39" s="29" t="str">
         <f>(B36^2-B37^2)/(4*B38*B39^2*SIN(B41*PI()/180))</f>
-        <v>0.00004189501594</v>
-      </c>
-      <c r="F39" s="30">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F39" s="30" t="str">
         <f t="shared" si="6"/>
-        <v>0.0000004684005178</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
@@ -15652,9 +15548,9 @@
       <c r="A40" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="B40" s="76">
+      <c r="B40" s="76" t="str">
         <f>(B36^2-B37^2)/(4*B38*B39)</f>
-        <v>0.003550147731</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C40" s="75"/>
       <c r="D40" s="75"/>
@@ -15667,9 +15563,9 @@
       <c r="A41" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="B41" s="76">
+      <c r="B41" s="76" t="str">
         <f>ACOS(B40)*180/PI()</f>
-        <v>89.79659109</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C41" s="75"/>
       <c r="D41" s="75"/>
@@ -15682,9 +15578,9 @@
       <c r="A42" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B42" s="76">
+      <c r="B42" s="76" t="str">
         <f>B41-90</f>
-        <v>-0.2034089089</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C42" s="75"/>
       <c r="D42" s="75" t="s">
@@ -15703,21 +15599,21 @@
       <c r="A43" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="B43" s="77">
+      <c r="B43" s="77" t="str">
         <f>SQRT(SUMSQ(F36:F39))*180/PI()</f>
-        <v>0.01150995384</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C43" s="75"/>
       <c r="D43" s="75" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="23">
+      <c r="E43" s="23" t="str">
         <f>AVERAGE(I4:I13)</f>
-        <v>-0.000412037037</v>
-      </c>
-      <c r="F43" s="1">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F43" s="1" t="str">
         <f>Intro!B6*(SUM(F4:F13))/SUMPRODUCT(E4:E13*D4:D13)</f>
-        <v>39.97888889</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G43" s="75"/>
       <c r="H43" s="75"/>
@@ -15727,13 +15623,13 @@
       <c r="D44" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="78">
+      <c r="E44" s="78" t="str">
         <f>AVERAGE(I14:I23)</f>
-        <v>-0.001328703704</v>
-      </c>
-      <c r="F44" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F44" s="6" t="str">
         <f>Intro!B6*(SUM(F14:F23))/SUMPRODUCT(E14:E23*D14:D23)</f>
-        <v>39.95</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
@@ -15760,7 +15656,7 @@
       </c>
       <c r="B47" s="79">
         <f>COUNTIF(D4:D8, TRUE())</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
@@ -15772,7 +15668,7 @@
       </c>
       <c r="B48" s="79">
         <f>COUNTIF(D9:D13, TRUE())</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
@@ -15783,7 +15679,7 @@
       </c>
       <c r="B49" s="79">
         <f>COUNTIF(D14:D18, TRUE())</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
@@ -15794,7 +15690,7 @@
       </c>
       <c r="B50" s="79">
         <f>COUNTIF(D19:D23, TRUE())</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
@@ -15805,7 +15701,7 @@
       </c>
       <c r="B51" s="79">
         <f>COUNTIF(D24:D27, TRUE())</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
@@ -15816,7 +15712,7 @@
       </c>
       <c r="B52" s="81">
         <f>COUNTIF(D28:D31, TRUE())</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>

</xml_diff>

<commit_message>
Add suggestions from VooDisss to spreadsheet
</commit_message>
<xml_diff>
--- a/Parametric Skew Calibration.xlsx
+++ b/Parametric Skew Calibration.xlsx
@@ -14,14 +14,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="XygZSYR9n+DChfGbaJpZdxSZagbycheTrwjnCVE666k="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="GCTscI0wMt40xwN+8/15XimzrYYm/EkNKdZTHev1Q64="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="104">
   <si>
     <t>Before you start, fill out the information below</t>
   </si>
@@ -218,7 +218,19 @@
     <t>Then type M500 in your console to save the settings</t>
   </si>
   <si>
+    <t xml:space="preserve">Please read the Klipper documentation to understand what you are doing! </t>
+  </si>
+  <si>
+    <t>Your skew correction gcode is:</t>
+  </si>
+  <si>
     <t>Skew compensation coming soon!</t>
+  </si>
+  <si>
+    <t>SKEW_PROFILE SAVE=my_skew_profile</t>
+  </si>
+  <si>
+    <t>To have Klipper calculate your skew, enter this into a console:</t>
   </si>
   <si>
     <t>In your printer.cfg, adjust</t>
@@ -276,6 +288,9 @@
   </si>
   <si>
     <t>Value</t>
+  </si>
+  <si>
+    <t>Accuracy</t>
   </si>
   <si>
     <t>sigma</t>
@@ -540,7 +555,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="84">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -578,13 +593,13 @@
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -596,24 +611,15 @@
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="1" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="1" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -718,20 +724,20 @@
     <xf borderId="9" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="0" fontId="6" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="6" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -763,10 +769,25 @@
     <xf borderId="6" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="1" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="167" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="167" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="8" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -5362,28 +5383,28 @@
         <f>IF(Helper!C7,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="24"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="20"/>
       <c r="G13" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="25"/>
-      <c r="B14" s="26" t="str">
+      <c r="A14" s="22"/>
+      <c r="B14" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C14" s="27" t="str">
+      <c r="C14" s="24" t="str">
         <f>IF(Helper!C8,(Intro!$B$4-4*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D14" s="28"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="31" t="str">
+      <c r="D14" s="25"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="28" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -5454,28 +5475,28 @@
         <f>IF(Helper!C12,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="24"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="20"/>
       <c r="G18" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="25"/>
-      <c r="B19" s="26" t="str">
+      <c r="A19" s="22"/>
+      <c r="B19" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C19" s="27" t="str">
+      <c r="C19" s="24" t="str">
         <f>IF(Helper!C13,(Intro!$B$4-4*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D19" s="32"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="31" t="str">
+      <c r="D19" s="29"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="28" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -5546,28 +5567,28 @@
         <f>IF(Helper!C17,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D23" s="22"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="24"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="20"/>
       <c r="G23" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="25"/>
-      <c r="B24" s="26" t="str">
+      <c r="A24" s="22"/>
+      <c r="B24" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C24" s="27" t="str">
+      <c r="C24" s="24" t="str">
         <f>IF(Helper!C18,(Intro!$B$4-4*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D24" s="28"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="31" t="str">
+      <c r="D24" s="25"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="28" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -5638,9 +5659,9 @@
         <f>IF(Helper!C22,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="24"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="20"/>
       <c r="G28" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5656,9 +5677,9 @@
         <f>IF(Helper!C23,(Intro!$B$4-4*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D29" s="22"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="24"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="20"/>
       <c r="G29" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5679,7 +5700,7 @@
       <c r="D30" s="12"/>
       <c r="E30" s="13"/>
       <c r="F30" s="14"/>
-      <c r="G30" s="33" t="str">
+      <c r="G30" s="30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -5712,9 +5733,9 @@
         <f>IF(Helper!C26, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>x</v>
       </c>
-      <c r="D32" s="22"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="24"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="20"/>
       <c r="G32" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5730,9 +5751,9 @@
         <f>IF(Helper!C27,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D33" s="22"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="24"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="20"/>
       <c r="G33" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5753,7 +5774,7 @@
       <c r="D34" s="12"/>
       <c r="E34" s="13"/>
       <c r="F34" s="14"/>
-      <c r="G34" s="33" t="str">
+      <c r="G34" s="30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -5771,7 +5792,7 @@
       <c r="D35" s="18"/>
       <c r="E35" s="19"/>
       <c r="F35" s="20"/>
-      <c r="G35" s="34" t="str">
+      <c r="G35" s="31" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -5786,28 +5807,28 @@
         <f>IF(Helper!C30, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>x</v>
       </c>
-      <c r="D36" s="22"/>
-      <c r="E36" s="23"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="34" t="str">
+      <c r="D36" s="18"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="31" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="25"/>
-      <c r="B37" s="26" t="str">
+      <c r="A37" s="22"/>
+      <c r="B37" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C37" s="27" t="str">
+      <c r="C37" s="24" t="str">
         <f>IF(Helper!C31,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D37" s="28"/>
-      <c r="E37" s="29"/>
-      <c r="F37" s="30"/>
-      <c r="G37" s="35" t="str">
+      <c r="D37" s="25"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="32" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -5815,11 +5836,11 @@
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="23"/>
-      <c r="F38" s="23"/>
-      <c r="G38" s="36"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="33"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="2"/>
@@ -5827,43 +5848,43 @@
       <c r="C39" s="2"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="37" t="s">
+      <c r="A40" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="B40" s="37"/>
-      <c r="C40" s="37"/>
-      <c r="D40" s="37"/>
-      <c r="E40" s="37"/>
-      <c r="F40" s="37"/>
-      <c r="G40" s="37"/>
-      <c r="H40" s="37"/>
-      <c r="I40" s="37"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="34"/>
+      <c r="D40" s="34"/>
+      <c r="E40" s="34"/>
+      <c r="F40" s="34"/>
+      <c r="G40" s="34"/>
+      <c r="H40" s="34"/>
+      <c r="I40" s="34"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="38" t="s">
+      <c r="A41" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="B41" s="38"/>
-      <c r="C41" s="38"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="38"/>
-      <c r="F41" s="38"/>
-      <c r="G41" s="38"/>
-      <c r="H41" s="38"/>
-      <c r="I41" s="38"/>
+      <c r="B41" s="35"/>
+      <c r="C41" s="35"/>
+      <c r="D41" s="35"/>
+      <c r="E41" s="35"/>
+      <c r="F41" s="35"/>
+      <c r="G41" s="35"/>
+      <c r="H41" s="35"/>
+      <c r="I41" s="35"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="39" t="s">
+      <c r="A42" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="B42" s="39"/>
-      <c r="C42" s="39"/>
-      <c r="D42" s="39"/>
-      <c r="E42" s="39"/>
-      <c r="F42" s="39"/>
-      <c r="G42" s="39"/>
-      <c r="H42" s="39"/>
-      <c r="I42" s="39"/>
+      <c r="B42" s="36"/>
+      <c r="C42" s="36"/>
+      <c r="D42" s="36"/>
+      <c r="E42" s="36"/>
+      <c r="F42" s="36"/>
+      <c r="G42" s="36"/>
+      <c r="H42" s="36"/>
+      <c r="I42" s="36"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="1" t="s">
@@ -5881,33 +5902,33 @@
       <c r="A45" s="1"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
-      <c r="W45" s="40"/>
-      <c r="X45" s="40"/>
+      <c r="W45" s="37"/>
+      <c r="X45" s="37"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
-      <c r="W46" s="40"/>
-      <c r="X46" s="40"/>
+      <c r="W46" s="37"/>
+      <c r="X46" s="37"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="1"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="L47" s="40"/>
-      <c r="O47" s="40"/>
-      <c r="P47" s="40"/>
-      <c r="W47" s="40"/>
-      <c r="X47" s="40"/>
+      <c r="L47" s="37"/>
+      <c r="O47" s="37"/>
+      <c r="P47" s="37"/>
+      <c r="W47" s="37"/>
+      <c r="X47" s="37"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="1"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
-      <c r="L48" s="40"/>
-      <c r="O48" s="40"/>
-      <c r="P48" s="40"/>
+      <c r="L48" s="37"/>
+      <c r="O48" s="37"/>
+      <c r="P48" s="37"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="1"/>
@@ -5918,30 +5939,30 @@
       <c r="A50" s="1"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
-      <c r="W50" s="23"/>
-      <c r="X50" s="23"/>
+      <c r="W50" s="19"/>
+      <c r="X50" s="19"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="1"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="L51" s="23"/>
-      <c r="O51" s="23"/>
-      <c r="P51" s="23"/>
-      <c r="S51" s="23"/>
-      <c r="T51" s="23"/>
-      <c r="W51" s="23"/>
-      <c r="X51" s="23"/>
+      <c r="L51" s="19"/>
+      <c r="O51" s="19"/>
+      <c r="P51" s="19"/>
+      <c r="S51" s="19"/>
+      <c r="T51" s="19"/>
+      <c r="W51" s="19"/>
+      <c r="X51" s="19"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="1"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="L52" s="23"/>
-      <c r="O52" s="23"/>
-      <c r="P52" s="23"/>
-      <c r="S52" s="23"/>
-      <c r="T52" s="23"/>
+      <c r="L52" s="19"/>
+      <c r="O52" s="19"/>
+      <c r="P52" s="19"/>
+      <c r="S52" s="19"/>
+      <c r="T52" s="19"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="2"/>
@@ -10914,7 +10935,7 @@
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="41"/>
+      <c r="E2" s="38"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="16"/>
@@ -10925,76 +10946,76 @@
       <c r="D3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="42" t="s">
+      <c r="G3" s="39" t="s">
         <v>45</v>
       </c>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
-      <c r="J3" s="43"/>
+      <c r="J3" s="40"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40" t="str">
+      <c r="B4" s="37"/>
+      <c r="C4" s="37" t="str">
         <f>Helper!E43</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D4" s="44">
+      <c r="D4" s="41">
         <f>SQRT(SUMSQ(Helper!K4:K13))</f>
         <v>0</v>
       </c>
-      <c r="E4" s="45" t="str">
+      <c r="E4" s="42" t="str">
         <f t="shared" ref="E4:E5" si="1">-C4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G4" s="46" t="s">
+      <c r="G4" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="37"/>
-      <c r="I4" s="37"/>
-      <c r="J4" s="47"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="44"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40" t="str">
+      <c r="B5" s="37"/>
+      <c r="C5" s="37" t="str">
         <f>Helper!E44</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D5" s="44">
+      <c r="D5" s="41">
         <f>SQRT(SUMSQ(Helper!K14:K23))</f>
         <v>0</v>
       </c>
-      <c r="E5" s="45" t="str">
+      <c r="E5" s="42" t="str">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="G5" s="48" t="s">
+      <c r="G5" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="38"/>
-      <c r="I5" s="38"/>
-      <c r="J5" s="49"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="46"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="23"/>
-      <c r="E6" s="41"/>
-      <c r="G6" s="50" t="s">
+      <c r="D6" s="19"/>
+      <c r="E6" s="38"/>
+      <c r="G6" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="52"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="49"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="16"/>
@@ -11002,58 +11023,58 @@
       <c r="C7" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="41" t="s">
+      <c r="E7" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="G7" s="50"/>
-      <c r="H7" s="51" t="s">
+      <c r="G7" s="47"/>
+      <c r="H7" s="48" t="s">
         <v>53</v>
       </c>
-      <c r="I7" s="51"/>
-      <c r="J7" s="53"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="50"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23" t="str">
+      <c r="B8" s="19"/>
+      <c r="C8" s="19" t="str">
         <f>Helper!B41</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D8" s="54" t="str">
+      <c r="D8" s="51" t="str">
         <f>Helper!B43</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E8" s="24"/>
-      <c r="G8" s="55" t="s">
+      <c r="E8" s="20"/>
+      <c r="G8" s="52" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="56"/>
-      <c r="I8" s="56"/>
-      <c r="J8" s="57"/>
+      <c r="H8" s="53"/>
+      <c r="I8" s="53"/>
+      <c r="J8" s="54"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="29"/>
-      <c r="C9" s="29" t="str">
+      <c r="B9" s="26"/>
+      <c r="C9" s="26" t="str">
         <f>C8-90</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D9" s="58" t="str">
+      <c r="D9" s="55" t="str">
         <f>Helper!B43</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E9" s="30" t="str">
+      <c r="E9" s="27" t="str">
         <f>-C9</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J9" s="23"/>
+      <c r="J9" s="19"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1"/>
@@ -11064,7 +11085,7 @@
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="59" t="s">
+      <c r="A12" s="12" t="s">
         <v>58</v>
       </c>
       <c r="B12" s="8"/>
@@ -11082,139 +11103,174 @@
       <c r="M12" s="9"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="60" t="s">
+      <c r="A13" s="56" t="s">
         <v>60</v>
       </c>
       <c r="E13" s="1"/>
-      <c r="F13" s="41"/>
+      <c r="F13" s="38"/>
       <c r="H13" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="M13" s="41"/>
+      <c r="M13" s="38"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="18" t="s">
         <v>62</v>
       </c>
       <c r="E14" s="1"/>
-      <c r="F14" s="41"/>
+      <c r="F14" s="38"/>
       <c r="H14" s="16"/>
       <c r="I14" s="1" t="str">
         <f>"M92 X"&amp;ROUND(Helper!F43,3)&amp;" Y"&amp;ROUND(Helper!F44,3)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="M14" s="41"/>
+      <c r="M14" s="38"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="22" t="str">
-        <f>"Length AC = "&amp;ROUND(Helper!B36,2)</f>
+      <c r="A15" s="18" t="str">
+        <f>"Length AC = "&amp;ROUND(Helper!B36,Helper!C36)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="E15" s="1"/>
-      <c r="F15" s="41"/>
+      <c r="F15" s="38"/>
       <c r="H15" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="M15" s="41"/>
+      <c r="M15" s="38"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="22" t="str">
-        <f>"Length BD = "&amp;ROUND(Helper!B37,2)</f>
+      <c r="A16" s="18" t="str">
+        <f>"Length BD = "&amp;ROUND(Helper!B37,Helper!C37)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F16" s="41"/>
+      <c r="F16" s="38"/>
       <c r="H16" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="M16" s="41"/>
+      <c r="M16" s="38"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="22" t="str">
-        <f>"Length AD = "&amp;ROUND(Helper!B38,2)</f>
+      <c r="A17" s="18" t="str">
+        <f>"Length AD = "&amp;ROUND(Helper!B38,Helper!C38)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F17" s="41"/>
+      <c r="F17" s="38"/>
       <c r="H17" s="16"/>
-      <c r="M17" s="41"/>
+      <c r="M17" s="38"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="18" t="str">
-        <f>"CALC_MEASURED_SKEW AC="&amp;ROUND(Helper!B36,2)&amp;" BD="&amp;ROUND(Helper!B37,2)&amp;" AD="&amp;ROUND(Helper!B38,2)</f>
+      <c r="A18" s="57"/>
+      <c r="F18" s="38"/>
+      <c r="H18" s="16"/>
+      <c r="M18" s="38"/>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="57" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" s="38"/>
+      <c r="H19" s="16"/>
+      <c r="M19" s="38"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="57" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="38"/>
+      <c r="H20" s="16"/>
+      <c r="M20" s="38"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="57" t="str">
+        <f>"SET_SKEW XY="&amp;ROUND(Helper!B36,Helper!C36)&amp;","&amp;ROUND(Helper!B37,Helper!C37)&amp;","&amp;ROUND(Helper!B38,Helper!C37)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F18" s="41"/>
-      <c r="H18" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="M18" s="41"/>
-    </row>
-    <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="F19" s="41"/>
-      <c r="H19" s="16"/>
-      <c r="M19" s="41"/>
-    </row>
-    <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="16" t="s">
+      <c r="F21" s="38"/>
+      <c r="H21" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="1" t="str">
+      <c r="M21" s="38"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="58" t="s">
+        <v>68</v>
+      </c>
+      <c r="F22" s="38"/>
+      <c r="H22" s="16"/>
+      <c r="M22" s="38"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="16"/>
+      <c r="F23" s="38"/>
+      <c r="H23" s="16"/>
+      <c r="M23" s="38"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="F24" s="38"/>
+      <c r="H24" s="16"/>
+      <c r="M24" s="38"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="16" t="str">
+        <f>"CALC_MEASURED_SKEW AC="&amp;ROUND(Helper!B36,Helper!C36)&amp;" BD="&amp;ROUND(Helper!B37,Helper!C37)&amp;" AD="&amp;ROUND(Helper!B38,Helper!C37)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F25" s="38"/>
+      <c r="H25" s="16"/>
+      <c r="M25" s="38"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="16"/>
+      <c r="F26" s="38"/>
+      <c r="H26" s="16"/>
+      <c r="M26" s="38"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F27" s="38"/>
+      <c r="H27" s="16"/>
+      <c r="M27" s="38"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" s="1" t="str">
         <f>ROUND(Helper!F43,3)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F20" s="41"/>
-      <c r="H20" s="16"/>
-      <c r="M20" s="41"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="B21" s="26" t="str">
+      <c r="C28" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F28" s="38"/>
+      <c r="H28" s="16"/>
+      <c r="M28" s="38"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" s="23" t="str">
         <f>ROUND(Helper!F44,3)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C21" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="61"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="26"/>
-      <c r="M21" s="61"/>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="2"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="2"/>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="2"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="2"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="2"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="2"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="2"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="2"/>
+      <c r="C29" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="59"/>
+      <c r="H29" s="22"/>
+      <c r="I29" s="23"/>
+      <c r="J29" s="23"/>
+      <c r="K29" s="23"/>
+      <c r="L29" s="23"/>
+      <c r="M29" s="59"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="2"/>
@@ -14128,6 +14184,30 @@
     </row>
     <row r="1000" ht="15.75" customHeight="1">
       <c r="A1000" s="2"/>
+    </row>
+    <row r="1001" ht="15.75" customHeight="1">
+      <c r="A1001" s="2"/>
+    </row>
+    <row r="1002" ht="15.75" customHeight="1">
+      <c r="A1002" s="2"/>
+    </row>
+    <row r="1003" ht="15.75" customHeight="1">
+      <c r="A1003" s="2"/>
+    </row>
+    <row r="1004" ht="15.75" customHeight="1">
+      <c r="A1004" s="2"/>
+    </row>
+    <row r="1005" ht="15.75" customHeight="1">
+      <c r="A1005" s="2"/>
+    </row>
+    <row r="1006" ht="15.75" customHeight="1">
+      <c r="A1006" s="2"/>
+    </row>
+    <row r="1007" ht="15.75" customHeight="1">
+      <c r="A1007" s="2"/>
+    </row>
+    <row r="1008" ht="15.75" customHeight="1">
+      <c r="A1008" s="2"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B4:E5">
@@ -14196,7 +14276,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B1" s="2"/>
       <c r="G1" s="2"/>
@@ -14209,34 +14289,34 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="B3" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E3" s="16" t="s">
         <v>25</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -14255,31 +14335,31 @@
         <f t="shared" ref="D4:D31" si="2">IFERROR(AND(NOT(F4=0),NOT(F4=""),C4),FALSE())</f>
         <v>0</v>
       </c>
-      <c r="E4" s="62">
+      <c r="E4" s="60">
         <f>IF(D4,'Post-print worksheet'!C10,0)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="63" t="str">
+      <c r="F4" s="13" t="str">
         <f>IF(C4, IFERROR(AVERAGE('Post-print worksheet'!D10:F10),""),"")</f>
         <v/>
       </c>
-      <c r="G4" s="63">
+      <c r="G4" s="13">
         <f>IF(C4, IFERROR(STDEV('Post-print worksheet'!D10:F10),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H4" s="63">
+      <c r="H4" s="13">
         <f>IF(C4, IFERROR(SQRT((Intro!$B$8/3)^2+G4^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I4" s="63" t="str">
+      <c r="I4" s="13" t="str">
         <f t="shared" ref="I4:I31" si="3">IF(D4, IFERROR((F4-E4)/E4,0),"")</f>
         <v/>
       </c>
-      <c r="J4" s="63" t="str">
+      <c r="J4" s="13" t="str">
         <f t="shared" ref="J4:J22" si="4">IF(D4, 1/(($B$47+$B$48)*E4),"")</f>
         <v/>
       </c>
-      <c r="K4" s="63" t="str">
+      <c r="K4" s="13" t="str">
         <f t="shared" ref="K4:K23" si="5">IF(D4,J4*H4,"")</f>
         <v/>
       </c>
@@ -14298,31 +14378,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E5" s="64">
+      <c r="E5" s="61">
         <f>IF(D5,'Post-print worksheet'!C11,0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="23" t="str">
+      <c r="F5" s="19" t="str">
         <f>IF(C5, IFERROR(AVERAGE('Post-print worksheet'!D11:F11),""),"")</f>
         <v/>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="19">
         <f>IF(C5, IFERROR(STDEV('Post-print worksheet'!D11:F11),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H5" s="23">
+      <c r="H5" s="19">
         <f>IF(C5, IFERROR(SQRT((Intro!$B$8/3)^2+G5^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I5" s="23" t="str">
+      <c r="I5" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J5" s="23" t="str">
+      <c r="J5" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K5" s="23" t="str">
+      <c r="K5" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14341,31 +14421,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E6" s="64">
+      <c r="E6" s="61">
         <f>IF(D6,'Post-print worksheet'!C12,0)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="23" t="str">
+      <c r="F6" s="19" t="str">
         <f>IF(C6, IFERROR(AVERAGE('Post-print worksheet'!D12:F12),""),"")</f>
         <v/>
       </c>
-      <c r="G6" s="23">
+      <c r="G6" s="19">
         <f>IF(C6, IFERROR(STDEV('Post-print worksheet'!D12:F12),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H6" s="23">
+      <c r="H6" s="19">
         <f>IF(C6, IFERROR(SQRT((Intro!$B$8/3)^2+G6^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I6" s="23" t="str">
+      <c r="I6" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J6" s="23" t="str">
+      <c r="J6" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K6" s="23" t="str">
+      <c r="K6" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14384,74 +14464,74 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E7" s="64">
+      <c r="E7" s="61">
         <f>IF(D7,'Post-print worksheet'!C13,0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="23" t="str">
+      <c r="F7" s="19" t="str">
         <f>IF(C7, IFERROR(AVERAGE('Post-print worksheet'!D13:F13),""),"")</f>
         <v/>
       </c>
-      <c r="G7" s="23" t="str">
+      <c r="G7" s="19" t="str">
         <f>IF(C7, IFERROR(STDEV('Post-print worksheet'!D13:F13),0),"")</f>
         <v/>
       </c>
-      <c r="H7" s="23" t="str">
+      <c r="H7" s="19" t="str">
         <f>IF(C7, IFERROR(SQRT((Intro!$B$8/3)^2+G7^2),0),"")</f>
         <v/>
       </c>
-      <c r="I7" s="23" t="str">
+      <c r="I7" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J7" s="23" t="str">
+      <c r="J7" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K7" s="23" t="str">
+      <c r="K7" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="26"/>
-      <c r="B8" s="26" t="str">
+      <c r="A8" s="23"/>
+      <c r="B8" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C8" s="26" t="b">
+      <c r="C8" s="23" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D8" s="26" t="b">
+      <c r="D8" s="23" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E8" s="65">
+      <c r="E8" s="62">
         <f>IF(D8,'Post-print worksheet'!C14,0)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="29" t="str">
+      <c r="F8" s="26" t="str">
         <f>IF(C8, IFERROR(AVERAGE('Post-print worksheet'!D14:F14),""),"")</f>
         <v/>
       </c>
-      <c r="G8" s="29" t="str">
+      <c r="G8" s="26" t="str">
         <f>IF(C8, IFERROR(STDEV('Post-print worksheet'!D14:F14),0),"")</f>
         <v/>
       </c>
-      <c r="H8" s="29" t="str">
+      <c r="H8" s="26" t="str">
         <f>IF(C8, IFERROR(SQRT((Intro!$B$8/3)^2+G8^2),0),"")</f>
         <v/>
       </c>
-      <c r="I8" s="29" t="str">
+      <c r="I8" s="26" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J8" s="29" t="str">
+      <c r="J8" s="26" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K8" s="29" t="str">
+      <c r="K8" s="26" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14472,31 +14552,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E9" s="64">
+      <c r="E9" s="61">
         <f>IF(D9,'Post-print worksheet'!C15,0)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="23" t="str">
+      <c r="F9" s="19" t="str">
         <f>IF(C9, IFERROR(AVERAGE('Post-print worksheet'!D15:F15),""),"")</f>
         <v/>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="19">
         <f>IF(C9, IFERROR(STDEV('Post-print worksheet'!D15:F15),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="19">
         <f>IF(C9, IFERROR(SQRT((Intro!$B$8/3)^2+G9^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I9" s="23" t="str">
+      <c r="I9" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J9" s="23" t="str">
+      <c r="J9" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K9" s="23" t="str">
+      <c r="K9" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14515,31 +14595,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E10" s="64">
+      <c r="E10" s="61">
         <f>IF(D10,'Post-print worksheet'!C16,0)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="23" t="str">
+      <c r="F10" s="19" t="str">
         <f>IF(C10, IFERROR(AVERAGE('Post-print worksheet'!D16:F16),""),"")</f>
         <v/>
       </c>
-      <c r="G10" s="23">
+      <c r="G10" s="19">
         <f>IF(C10, IFERROR(STDEV('Post-print worksheet'!D16:F16),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H10" s="23">
+      <c r="H10" s="19">
         <f>IF(C10, IFERROR(SQRT((Intro!$B$8/3)^2+G10^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I10" s="23" t="str">
+      <c r="I10" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J10" s="23" t="str">
+      <c r="J10" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K10" s="23" t="str">
+      <c r="K10" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14558,31 +14638,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E11" s="64">
+      <c r="E11" s="61">
         <f>IF(D11,'Post-print worksheet'!C17,0)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="23" t="str">
+      <c r="F11" s="19" t="str">
         <f>IF(C11, IFERROR(AVERAGE('Post-print worksheet'!D17:F17),""),"")</f>
         <v/>
       </c>
-      <c r="G11" s="23">
+      <c r="G11" s="19">
         <f>IF(C11, IFERROR(STDEV('Post-print worksheet'!D17:F17),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="19">
         <f>IF(C11, IFERROR(SQRT((Intro!$B$8/3)^2+G11^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I11" s="23" t="str">
+      <c r="I11" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J11" s="23" t="str">
+      <c r="J11" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K11" s="23" t="str">
+      <c r="K11" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14601,74 +14681,74 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E12" s="64">
+      <c r="E12" s="61">
         <f>IF(D12,'Post-print worksheet'!C18,0)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="23" t="str">
+      <c r="F12" s="19" t="str">
         <f>IF(C12, IFERROR(AVERAGE('Post-print worksheet'!D18:F18),""),"")</f>
         <v/>
       </c>
-      <c r="G12" s="23" t="str">
+      <c r="G12" s="19" t="str">
         <f>IF(C12, IFERROR(STDEV('Post-print worksheet'!D18:F18),0),"")</f>
         <v/>
       </c>
-      <c r="H12" s="23" t="str">
+      <c r="H12" s="19" t="str">
         <f>IF(C12, IFERROR(SQRT((Intro!$B$8/3)^2+G12^2),0),"")</f>
         <v/>
       </c>
-      <c r="I12" s="23" t="str">
+      <c r="I12" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J12" s="23" t="str">
+      <c r="J12" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K12" s="23" t="str">
+      <c r="K12" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="26"/>
-      <c r="B13" s="26" t="str">
+      <c r="A13" s="23"/>
+      <c r="B13" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C13" s="26" t="b">
+      <c r="C13" s="23" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D13" s="26" t="b">
+      <c r="D13" s="23" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E13" s="65">
+      <c r="E13" s="62">
         <f>IF(D13,'Post-print worksheet'!C19,0)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="29" t="str">
+      <c r="F13" s="26" t="str">
         <f>IF(C13, IFERROR(AVERAGE('Post-print worksheet'!D19:F19),""),"")</f>
         <v/>
       </c>
-      <c r="G13" s="29" t="str">
+      <c r="G13" s="26" t="str">
         <f>IF(C13, IFERROR(STDEV('Post-print worksheet'!D19:F19),0),"")</f>
         <v/>
       </c>
-      <c r="H13" s="29" t="str">
+      <c r="H13" s="26" t="str">
         <f>IF(C13, IFERROR(SQRT((Intro!$B$8/3)^2+G13^2),0),"")</f>
         <v/>
       </c>
-      <c r="I13" s="29" t="str">
+      <c r="I13" s="26" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J13" s="29" t="str">
+      <c r="J13" s="26" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K13" s="29" t="str">
+      <c r="K13" s="26" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14689,31 +14769,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E14" s="64">
+      <c r="E14" s="61">
         <f>IF(D14,'Post-print worksheet'!C20,0)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="23" t="str">
+      <c r="F14" s="19" t="str">
         <f>IF(C14, IFERROR(AVERAGE('Post-print worksheet'!D20:F20),""),"")</f>
         <v/>
       </c>
-      <c r="G14" s="23">
+      <c r="G14" s="19">
         <f>IF(C14, IFERROR(STDEV('Post-print worksheet'!D20:F20),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H14" s="23">
+      <c r="H14" s="19">
         <f>IF(C14, IFERROR(SQRT((Intro!$B$8/3)^2+G14^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I14" s="23" t="str">
+      <c r="I14" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J14" s="23" t="str">
+      <c r="J14" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K14" s="23" t="str">
+      <c r="K14" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14732,31 +14812,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E15" s="64">
+      <c r="E15" s="61">
         <f>IF(D15,'Post-print worksheet'!C21,0)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="23" t="str">
+      <c r="F15" s="19" t="str">
         <f>IF(C15, IFERROR(AVERAGE('Post-print worksheet'!D21:F21),""),"")</f>
         <v/>
       </c>
-      <c r="G15" s="23">
+      <c r="G15" s="19">
         <f>IF(C15, IFERROR(STDEV('Post-print worksheet'!D21:F21),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H15" s="23">
+      <c r="H15" s="19">
         <f>IF(C15, IFERROR(SQRT((Intro!$B$8/3)^2+G15^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I15" s="23" t="str">
+      <c r="I15" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J15" s="23" t="str">
+      <c r="J15" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K15" s="23" t="str">
+      <c r="K15" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14775,31 +14855,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E16" s="64">
+      <c r="E16" s="61">
         <f>IF(D16,'Post-print worksheet'!C22,0)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="23" t="str">
+      <c r="F16" s="19" t="str">
         <f>IF(C16, IFERROR(AVERAGE('Post-print worksheet'!D22:F22),""),"")</f>
         <v/>
       </c>
-      <c r="G16" s="23">
+      <c r="G16" s="19">
         <f>IF(C16, IFERROR(STDEV('Post-print worksheet'!D22:F22),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H16" s="23">
+      <c r="H16" s="19">
         <f>IF(C16, IFERROR(SQRT((Intro!$B$8/3)^2+G16^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I16" s="23" t="str">
+      <c r="I16" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J16" s="23" t="str">
+      <c r="J16" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K16" s="23" t="str">
+      <c r="K16" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14818,74 +14898,74 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E17" s="64">
+      <c r="E17" s="61">
         <f>IF(D17,'Post-print worksheet'!C23,0)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="23" t="str">
+      <c r="F17" s="19" t="str">
         <f>IF(C17, IFERROR(AVERAGE('Post-print worksheet'!D23:F23),""),"")</f>
         <v/>
       </c>
-      <c r="G17" s="23" t="str">
+      <c r="G17" s="19" t="str">
         <f>IF(C17, IFERROR(STDEV('Post-print worksheet'!D23:F23),0),"")</f>
         <v/>
       </c>
-      <c r="H17" s="23" t="str">
+      <c r="H17" s="19" t="str">
         <f>IF(C17, IFERROR(SQRT((Intro!$B$8/3)^2+G17^2),0),"")</f>
         <v/>
       </c>
-      <c r="I17" s="23" t="str">
+      <c r="I17" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J17" s="23" t="str">
+      <c r="J17" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K17" s="23" t="str">
+      <c r="K17" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="26"/>
-      <c r="B18" s="26" t="str">
+      <c r="A18" s="23"/>
+      <c r="B18" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C18" s="26" t="b">
+      <c r="C18" s="23" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D18" s="26" t="b">
+      <c r="D18" s="23" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E18" s="65">
+      <c r="E18" s="62">
         <f>IF(D18,'Post-print worksheet'!C24,0)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="29" t="str">
+      <c r="F18" s="26" t="str">
         <f>IF(C18, IFERROR(AVERAGE('Post-print worksheet'!D24:F24),""),"")</f>
         <v/>
       </c>
-      <c r="G18" s="29" t="str">
+      <c r="G18" s="26" t="str">
         <f>IF(C18, IFERROR(STDEV('Post-print worksheet'!D24:F24),0),"")</f>
         <v/>
       </c>
-      <c r="H18" s="29" t="str">
+      <c r="H18" s="26" t="str">
         <f>IF(C18, IFERROR(SQRT((Intro!$B$8/3)^2+G18^2),0),"")</f>
         <v/>
       </c>
-      <c r="I18" s="29" t="str">
+      <c r="I18" s="26" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J18" s="29" t="str">
+      <c r="J18" s="26" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K18" s="29" t="str">
+      <c r="K18" s="26" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14906,31 +14986,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E19" s="64">
+      <c r="E19" s="61">
         <f>IF(D19,'Post-print worksheet'!C25,0)</f>
         <v>0</v>
       </c>
-      <c r="F19" s="23" t="str">
+      <c r="F19" s="19" t="str">
         <f>IF(C19, IFERROR(AVERAGE('Post-print worksheet'!D25:F25),""),"")</f>
         <v/>
       </c>
-      <c r="G19" s="23">
+      <c r="G19" s="19">
         <f>IF(C19, IFERROR(STDEV('Post-print worksheet'!D25:F25),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H19" s="23">
+      <c r="H19" s="19">
         <f>IF(C19, IFERROR(SQRT((Intro!$B$8/3)^2+G19^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I19" s="23" t="str">
+      <c r="I19" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J19" s="23" t="str">
+      <c r="J19" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K19" s="23" t="str">
+      <c r="K19" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14949,31 +15029,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E20" s="64">
+      <c r="E20" s="61">
         <f>IF(D20,'Post-print worksheet'!C26,0)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="23" t="str">
+      <c r="F20" s="19" t="str">
         <f>IF(C20, IFERROR(AVERAGE('Post-print worksheet'!D26:F26),""),"")</f>
         <v/>
       </c>
-      <c r="G20" s="23">
+      <c r="G20" s="19">
         <f>IF(C20, IFERROR(STDEV('Post-print worksheet'!D26:F26),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H20" s="23">
+      <c r="H20" s="19">
         <f>IF(C20, IFERROR(SQRT((Intro!$B$8/3)^2+G20^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I20" s="23" t="str">
+      <c r="I20" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J20" s="23" t="str">
+      <c r="J20" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K20" s="23" t="str">
+      <c r="K20" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14992,31 +15072,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E21" s="64">
+      <c r="E21" s="61">
         <f>IF(D21,'Post-print worksheet'!C27,0)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="23" t="str">
+      <c r="F21" s="19" t="str">
         <f>IF(C21, IFERROR(AVERAGE('Post-print worksheet'!D27:F27),""),"")</f>
         <v/>
       </c>
-      <c r="G21" s="23">
+      <c r="G21" s="19">
         <f>IF(C21, IFERROR(STDEV('Post-print worksheet'!D27:F27),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H21" s="23">
+      <c r="H21" s="19">
         <f>IF(C21, IFERROR(SQRT((Intro!$B$8/3)^2+G21^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I21" s="23" t="str">
+      <c r="I21" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J21" s="23" t="str">
+      <c r="J21" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K21" s="23" t="str">
+      <c r="K21" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -15035,81 +15115,81 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E22" s="64">
+      <c r="E22" s="61">
         <f>IF(D22,'Post-print worksheet'!C28,0)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="23" t="str">
+      <c r="F22" s="19" t="str">
         <f>IF(C22, IFERROR(AVERAGE('Post-print worksheet'!D28:F28),""),"")</f>
         <v/>
       </c>
-      <c r="G22" s="23" t="str">
+      <c r="G22" s="19" t="str">
         <f>IF(C22, IFERROR(STDEV('Post-print worksheet'!D28:F28),0),"")</f>
         <v/>
       </c>
-      <c r="H22" s="23" t="str">
+      <c r="H22" s="19" t="str">
         <f>IF(C22, IFERROR(SQRT((Intro!$B$8/3)^2+G22^2),0),"")</f>
         <v/>
       </c>
-      <c r="I22" s="23" t="str">
+      <c r="I22" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J22" s="23" t="str">
+      <c r="J22" s="19" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K22" s="23" t="str">
+      <c r="K22" s="19" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="26"/>
-      <c r="B23" s="26" t="str">
+      <c r="A23" s="23"/>
+      <c r="B23" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C23" s="26" t="b">
+      <c r="C23" s="23" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D23" s="26" t="b">
+      <c r="D23" s="23" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E23" s="65">
+      <c r="E23" s="62">
         <f>IF(D23,'Post-print worksheet'!C29,0)</f>
         <v>0</v>
       </c>
-      <c r="F23" s="29" t="str">
+      <c r="F23" s="26" t="str">
         <f>IF(C23, IFERROR(AVERAGE('Post-print worksheet'!D29:F29),""),"")</f>
         <v/>
       </c>
-      <c r="G23" s="29" t="str">
+      <c r="G23" s="26" t="str">
         <f>IF(C23, IFERROR(STDEV('Post-print worksheet'!D29:F29),0),"")</f>
         <v/>
       </c>
-      <c r="H23" s="29" t="str">
+      <c r="H23" s="26" t="str">
         <f>IF(C23, IFERROR(SQRT((Intro!$B$8/3)^2+G23^2),0),"")</f>
         <v/>
       </c>
-      <c r="I23" s="29" t="str">
+      <c r="I23" s="26" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J23" s="29" t="str">
+      <c r="J23" s="26" t="str">
         <f>IF(C23, 1/(2*Intro!B$3*E23),"")</f>
         <v/>
       </c>
-      <c r="K23" s="29" t="str">
+      <c r="K23" s="26" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B24" s="1">
         <f>IF(2 &lt;= Intro!B$3, 1, "")</f>
@@ -15123,28 +15203,28 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E24" s="64">
+      <c r="E24" s="61">
         <f>IF(D24,'Post-print worksheet'!C30,0)</f>
         <v>0</v>
       </c>
-      <c r="F24" s="23" t="str">
+      <c r="F24" s="19" t="str">
         <f>IF(C24, IFERROR(AVERAGE('Post-print worksheet'!D30:F30),""),"")</f>
         <v/>
       </c>
-      <c r="G24" s="23">
+      <c r="G24" s="19">
         <f>IF(C24, IFERROR(STDEV('Post-print worksheet'!D30:F30),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H24" s="23">
+      <c r="H24" s="19">
         <f>IF(C24, IFERROR(SQRT((Intro!$B$8/3)^2+G24^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I24" s="23" t="str">
+      <c r="I24" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J24" s="66"/>
-      <c r="K24" s="66"/>
+      <c r="J24" s="63"/>
+      <c r="K24" s="63"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1"/>
@@ -15160,28 +15240,28 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E25" s="64">
+      <c r="E25" s="61">
         <f>IF(D25,'Post-print worksheet'!C31,0)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="23" t="str">
+      <c r="F25" s="19" t="str">
         <f>IF(C25, IFERROR(AVERAGE('Post-print worksheet'!D31:F31),""),"")</f>
         <v/>
       </c>
-      <c r="G25" s="23">
+      <c r="G25" s="19">
         <f>IF(C25, IFERROR(STDEV('Post-print worksheet'!D31:F31),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H25" s="23">
+      <c r="H25" s="19">
         <f>IF(C25, IFERROR(SQRT((Intro!$B$8/3)^2+G25^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I25" s="23" t="str">
+      <c r="I25" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J25" s="66"/>
-      <c r="K25" s="66"/>
+      <c r="J25" s="63"/>
+      <c r="K25" s="63"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1"/>
@@ -15197,69 +15277,69 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E26" s="64">
+      <c r="E26" s="61">
         <f>IF(D26,'Post-print worksheet'!C32,0)</f>
         <v>0</v>
       </c>
-      <c r="F26" s="23" t="str">
+      <c r="F26" s="19" t="str">
         <f>IF(C26, IFERROR(AVERAGE('Post-print worksheet'!D32:F32),""),"")</f>
         <v/>
       </c>
-      <c r="G26" s="23" t="str">
+      <c r="G26" s="19" t="str">
         <f>IF(C26, IFERROR(STDEV('Post-print worksheet'!D32:F32),0),"")</f>
         <v/>
       </c>
-      <c r="H26" s="23" t="str">
+      <c r="H26" s="19" t="str">
         <f>IF(C26, IFERROR(SQRT((Intro!$B$8/3)^2+G26^2),0),"")</f>
         <v/>
       </c>
-      <c r="I26" s="23" t="str">
+      <c r="I26" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J26" s="66"/>
-      <c r="K26" s="66"/>
+      <c r="J26" s="63"/>
+      <c r="K26" s="63"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="26"/>
-      <c r="B27" s="26" t="str">
+      <c r="A27" s="23"/>
+      <c r="B27" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C27" s="26" t="b">
+      <c r="C27" s="23" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D27" s="26" t="b">
+      <c r="D27" s="23" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E27" s="65">
+      <c r="E27" s="62">
         <f>IF(D27,'Post-print worksheet'!C33,0)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="29" t="str">
+      <c r="F27" s="26" t="str">
         <f>IF(C27, IFERROR(AVERAGE('Post-print worksheet'!D33:F33),""),"")</f>
         <v/>
       </c>
-      <c r="G27" s="29" t="str">
+      <c r="G27" s="26" t="str">
         <f>IF(C27, IFERROR(STDEV('Post-print worksheet'!D33:F33),0),"")</f>
         <v/>
       </c>
-      <c r="H27" s="29" t="str">
+      <c r="H27" s="26" t="str">
         <f>IF(C27, IFERROR(SQRT((Intro!$B$8/3)^2+G27^2),0),"")</f>
         <v/>
       </c>
-      <c r="I27" s="29" t="str">
+      <c r="I27" s="26" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J27" s="67"/>
-      <c r="K27" s="67"/>
+      <c r="J27" s="64"/>
+      <c r="K27" s="64"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B28" s="1">
         <f>IF(2 &lt;= Intro!B$3, 1, "")</f>
@@ -15273,28 +15353,28 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E28" s="64">
+      <c r="E28" s="61">
         <f>IF(D28,'Post-print worksheet'!C34,0)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="23" t="str">
+      <c r="F28" s="19" t="str">
         <f>IF(C28, IFERROR(AVERAGE('Post-print worksheet'!D34:F34),""),"")</f>
         <v/>
       </c>
-      <c r="G28" s="23">
+      <c r="G28" s="19">
         <f>IF(C28, IFERROR(STDEV('Post-print worksheet'!D34:F34),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H28" s="23">
+      <c r="H28" s="19">
         <f>IF(C28, IFERROR(SQRT((Intro!$B$8/3)^2+G28^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I28" s="23" t="str">
+      <c r="I28" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J28" s="66"/>
-      <c r="K28" s="66"/>
+      <c r="J28" s="63"/>
+      <c r="K28" s="63"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="B29" s="1">
@@ -15309,28 +15389,28 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E29" s="64">
+      <c r="E29" s="61">
         <f>IF(D29,'Post-print worksheet'!C35,0)</f>
         <v>0</v>
       </c>
-      <c r="F29" s="23" t="str">
+      <c r="F29" s="19" t="str">
         <f>IF(C29, IFERROR(AVERAGE('Post-print worksheet'!D35:F35),""),"")</f>
         <v/>
       </c>
-      <c r="G29" s="23">
+      <c r="G29" s="19">
         <f>IF(C29, IFERROR(STDEV('Post-print worksheet'!D35:F35),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H29" s="23">
+      <c r="H29" s="19">
         <f>IF(C29, IFERROR(SQRT((Intro!$B$8/3)^2+G29^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I29" s="23" t="str">
+      <c r="I29" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J29" s="66"/>
-      <c r="K29" s="66"/>
+      <c r="J29" s="63"/>
+      <c r="K29" s="63"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="B30" s="1" t="str">
@@ -15345,65 +15425,65 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E30" s="64">
+      <c r="E30" s="61">
         <f>IF(D30,'Post-print worksheet'!C36,0)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="23" t="str">
+      <c r="F30" s="19" t="str">
         <f>IF(C30, IFERROR(AVERAGE('Post-print worksheet'!D36:F36),""),"")</f>
         <v/>
       </c>
-      <c r="G30" s="23" t="str">
+      <c r="G30" s="19" t="str">
         <f>IF(C30, IFERROR(STDEV('Post-print worksheet'!D36:F36),0),"")</f>
         <v/>
       </c>
-      <c r="H30" s="23" t="str">
+      <c r="H30" s="19" t="str">
         <f>IF(C30, IFERROR(SQRT((Intro!$B$8/3)^2+G30^2),0),"")</f>
         <v/>
       </c>
-      <c r="I30" s="23" t="str">
+      <c r="I30" s="19" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J30" s="66"/>
-      <c r="K30" s="66"/>
+      <c r="J30" s="63"/>
+      <c r="K30" s="63"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="26"/>
-      <c r="B31" s="26" t="str">
+      <c r="A31" s="23"/>
+      <c r="B31" s="23" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C31" s="26" t="b">
+      <c r="C31" s="23" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D31" s="26" t="b">
+      <c r="D31" s="23" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E31" s="65">
+      <c r="E31" s="62">
         <f>IF(D31,'Post-print worksheet'!C37,0)</f>
         <v>0</v>
       </c>
-      <c r="F31" s="29" t="str">
+      <c r="F31" s="26" t="str">
         <f>IF(C31, IFERROR(AVERAGE('Post-print worksheet'!D37:F37),""),"")</f>
         <v/>
       </c>
-      <c r="G31" s="29" t="str">
+      <c r="G31" s="26" t="str">
         <f>IF(C31, IFERROR(STDEV('Post-print worksheet'!D37:F37),0),"")</f>
         <v/>
       </c>
-      <c r="H31" s="29" t="str">
+      <c r="H31" s="26" t="str">
         <f>IF(C31, IFERROR(SQRT((Intro!$B$8/3)^2+G31^2),0),"")</f>
         <v/>
       </c>
-      <c r="I31" s="29" t="str">
+      <c r="I31" s="26" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J31" s="67"/>
-      <c r="K31" s="67"/>
+      <c r="J31" s="64"/>
+      <c r="K31" s="64"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="B32" s="2"/>
@@ -15416,105 +15496,116 @@
       <c r="H33" s="2"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="68"/>
+      <c r="A34" s="65"/>
       <c r="B34" s="9" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C34" s="1"/>
-      <c r="D34" s="69" t="s">
-        <v>83</v>
-      </c>
-      <c r="E34" s="70"/>
-      <c r="F34" s="71"/>
+      <c r="D34" s="66" t="s">
+        <v>87</v>
+      </c>
+      <c r="E34" s="67"/>
+      <c r="F34" s="68"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="72"/>
-      <c r="B35" s="41" t="s">
-        <v>84</v>
-      </c>
-      <c r="C35" s="1"/>
+      <c r="A35" s="69"/>
+      <c r="B35" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="D35" s="16" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F35" s="41" t="s">
-        <v>79</v>
+        <v>91</v>
+      </c>
+      <c r="F35" s="38" t="s">
+        <v>83</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="B36" s="73" t="str">
+        <v>92</v>
+      </c>
+      <c r="B36" s="70" t="str">
         <f>SUM(F24:F27)/SUMPRODUCT(D24:D27*E24:E27)*Intro!$B$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C36" s="74"/>
-      <c r="D36" s="22" t="str">
+      <c r="C36" s="71" t="str">
+        <f t="shared" ref="C36:C38" si="6">CEILING(-LOG10(D36),1)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D36" s="72" t="str">
         <f>SQRT(SUMSQ(H24:H27))/SUMPRODUCT(D24:D27*E24:E27)*Intro!$B$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E36" s="23" t="str">
+      <c r="E36" s="51" t="str">
         <f>-B36/(2*B38*B39*SIN(B41*PI()/180))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F36" s="24" t="str">
-        <f t="shared" ref="F36:F39" si="6">D36*E36</f>
+      <c r="F36" s="73" t="str">
+        <f t="shared" ref="F36:F39" si="7">D36*E36</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
-      <c r="J36" s="75"/>
+      <c r="J36" s="74"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="B37" s="73" t="str">
+        <v>93</v>
+      </c>
+      <c r="B37" s="70" t="str">
         <f>SUM(F28:F31)/SUMPRODUCT(D28:D31*E28:E31)*Intro!$B$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C37" s="74"/>
-      <c r="D37" s="22" t="str">
+      <c r="C37" s="71" t="str">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D37" s="72" t="str">
         <f>SQRT(SUMSQ(H28:H31))/SUMPRODUCT(D28:D31*E28:E31)*Intro!$B$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E37" s="23" t="str">
+      <c r="E37" s="51" t="str">
         <f>B37/(2*B38*B39*SIN(B41*PI()/180))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F37" s="24" t="str">
+      <c r="F37" s="73" t="str">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B38" s="70" t="str">
+        <f>SQRT(2)*Intro!B4/2*SUM(F4:F8)/(SUMPRODUCT(D4:D8*E4:E8))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C38" s="71" t="str">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="B38" s="73" t="str">
-        <f>SQRT(2)*Intro!B4/2*SUM(F4:F8)/(SUMPRODUCT(D4:D8*E4:E8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C38" s="74"/>
-      <c r="D38" s="22" t="str">
+      <c r="D38" s="72" t="str">
         <f>SQRT(2)*Intro!B4/2*SQRT(SUMSQ(H4:H8))/(SUMPRODUCT(D4:D8*E4:E8))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E38" s="23" t="str">
+      <c r="E38" s="51" t="str">
         <f>(B36^2-B37^2)/(4*B38^2*B39*SIN(B41*PI()/180))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F38" s="24" t="str">
-        <f t="shared" si="6"/>
+      <c r="F38" s="73" t="str">
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="G38" s="2"/>
@@ -15522,23 +15613,23 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="B39" s="73" t="str">
+        <v>95</v>
+      </c>
+      <c r="B39" s="70" t="str">
         <f>SQRT(2)*Intro!B4/2*SUM(F14:F18)/(SUMPRODUCT(D14:D18*E14:E18))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C39" s="74"/>
-      <c r="D39" s="28" t="str">
+      <c r="C39" s="75"/>
+      <c r="D39" s="76" t="str">
         <f>SQRT(2)*Intro!B4/2*SQRT(SUMSQ(H14:H18))/(SUMPRODUCT(D14:D18*E14:E18))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E39" s="29" t="str">
+      <c r="E39" s="55" t="str">
         <f>(B36^2-B37^2)/(4*B38*B39^2*SIN(B41*PI()/180))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F39" s="30" t="str">
-        <f t="shared" si="6"/>
+      <c r="F39" s="77" t="str">
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="G39" s="2"/>
@@ -15546,68 +15637,68 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="B40" s="76" t="str">
+        <v>96</v>
+      </c>
+      <c r="B40" s="78" t="str">
         <f>(B36^2-B37^2)/(4*B38*B39)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C40" s="75"/>
-      <c r="D40" s="75"/>
-      <c r="E40" s="75"/>
-      <c r="F40" s="75"/>
-      <c r="G40" s="75"/>
-      <c r="H40" s="75"/>
+      <c r="C40" s="74"/>
+      <c r="D40" s="74"/>
+      <c r="E40" s="74"/>
+      <c r="F40" s="74"/>
+      <c r="G40" s="74"/>
+      <c r="H40" s="74"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="B41" s="76" t="str">
+        <v>97</v>
+      </c>
+      <c r="B41" s="78" t="str">
         <f>ACOS(B40)*180/PI()</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C41" s="75"/>
-      <c r="D41" s="75"/>
-      <c r="E41" s="75"/>
-      <c r="F41" s="75"/>
-      <c r="G41" s="75"/>
-      <c r="H41" s="75"/>
+      <c r="C41" s="74"/>
+      <c r="D41" s="74"/>
+      <c r="E41" s="74"/>
+      <c r="F41" s="74"/>
+      <c r="G41" s="74"/>
+      <c r="H41" s="74"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="B42" s="76" t="str">
+        <v>98</v>
+      </c>
+      <c r="B42" s="78" t="str">
         <f>B41-90</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C42" s="75"/>
-      <c r="D42" s="75" t="s">
-        <v>94</v>
-      </c>
-      <c r="E42" s="75" t="s">
-        <v>95</v>
-      </c>
-      <c r="F42" s="75" t="s">
-        <v>96</v>
-      </c>
-      <c r="G42" s="75"/>
-      <c r="H42" s="75"/>
+      <c r="C42" s="74"/>
+      <c r="D42" s="74" t="s">
+        <v>99</v>
+      </c>
+      <c r="E42" s="74" t="s">
+        <v>100</v>
+      </c>
+      <c r="F42" s="74" t="s">
+        <v>101</v>
+      </c>
+      <c r="G42" s="74"/>
+      <c r="H42" s="74"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="B43" s="77" t="str">
+      <c r="A43" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="B43" s="79" t="str">
         <f>SQRT(SUMSQ(F36:F39))*180/PI()</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C43" s="75"/>
-      <c r="D43" s="75" t="s">
+      <c r="C43" s="74"/>
+      <c r="D43" s="74" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="23" t="str">
+      <c r="E43" s="19" t="str">
         <f>AVERAGE(I4:I13)</f>
         <v>#DIV/0!</v>
       </c>
@@ -15615,15 +15706,15 @@
         <f>Intro!B6*(SUM(F4:F13))/SUMPRODUCT(E4:E13*D4:D13)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G43" s="75"/>
-      <c r="H43" s="75"/>
+      <c r="G43" s="74"/>
+      <c r="H43" s="74"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="B44" s="2"/>
       <c r="D44" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="78" t="str">
+      <c r="E44" s="80" t="str">
         <f>AVERAGE(I14:I23)</f>
         <v>#DIV/0!</v>
       </c>
@@ -15641,20 +15732,20 @@
       <c r="L45" s="1"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="68" t="s">
-        <v>98</v>
-      </c>
-      <c r="B46" s="71"/>
+      <c r="A46" s="65" t="s">
+        <v>103</v>
+      </c>
+      <c r="B46" s="68"/>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="72" t="s">
+      <c r="A47" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="B47" s="79">
+      <c r="B47" s="81">
         <f>COUNTIF(D4:D8, TRUE())</f>
         <v>0</v>
       </c>
@@ -15663,10 +15754,10 @@
       <c r="K47" s="1"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="72" t="s">
+      <c r="A48" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="B48" s="79">
+      <c r="B48" s="81">
         <f>COUNTIF(D9:D13, TRUE())</f>
         <v>0</v>
       </c>
@@ -15674,10 +15765,10 @@
       <c r="H48" s="2"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="72" t="s">
+      <c r="A49" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="B49" s="79">
+      <c r="B49" s="81">
         <f>COUNTIF(D14:D18, TRUE())</f>
         <v>0</v>
       </c>
@@ -15685,10 +15776,10 @@
       <c r="H49" s="2"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="72" t="s">
+      <c r="A50" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="B50" s="79">
+      <c r="B50" s="81">
         <f>COUNTIF(D19:D23, TRUE())</f>
         <v>0</v>
       </c>
@@ -15696,10 +15787,10 @@
       <c r="H50" s="2"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="72" t="s">
-        <v>80</v>
-      </c>
-      <c r="B51" s="79">
+      <c r="A51" s="69" t="s">
+        <v>84</v>
+      </c>
+      <c r="B51" s="81">
         <f>COUNTIF(D24:D27, TRUE())</f>
         <v>0</v>
       </c>
@@ -15707,10 +15798,10 @@
       <c r="H51" s="2"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="80" t="s">
-        <v>81</v>
-      </c>
-      <c r="B52" s="81">
+      <c r="A52" s="82" t="s">
+        <v>85</v>
+      </c>
+      <c r="B52" s="83">
         <f>COUNTIF(D28:D31, TRUE())</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Spreadsheet updates and caveats.
1. Add CoreXY option (averages x/y-step adjustments)
2. Warning about iterative skew correction
</commit_message>
<xml_diff>
--- a/Parametric Skew Calibration.xlsx
+++ b/Parametric Skew Calibration.xlsx
@@ -9,19 +9,19 @@
     <sheet state="visible" name="Helper" sheetId="4" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Post-print worksheet'!$C$9:$C$37</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Post-print worksheet'!$C$13:$C$41</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="GCTscI0wMt40xwN+8/15XimzrYYm/EkNKdZTHev1Q64="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="Nh9WLC80wVRXmab31sSloM0dJwwUTSlQnXbIMEFdsek="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="115">
   <si>
     <t>Before you start, fill out the information below</t>
   </si>
@@ -38,13 +38,16 @@
     <t>Did you do any additional scaling before printing the model? (Not recommended). If not, keep this as a 1</t>
   </si>
   <si>
-    <t>X E-steps</t>
+    <t>X steps/mm</t>
   </si>
   <si>
-    <t>Your printer's current E-steps (M503), or rotation_distance in Klipper printer.cfg</t>
+    <t>Your printer's current X-steps (M503), or rotation_distance in Klipper printer.cfg</t>
   </si>
   <si>
-    <t>Y E-steps</t>
+    <t>Y steps/mm</t>
+  </si>
+  <si>
+    <t>Your printer's current Y-steps (M503), or rotation_distance in Klipper printer.cfg</t>
   </si>
   <si>
     <t>Caliper error (mm)</t>
@@ -57,6 +60,21 @@
   </si>
   <si>
     <t>Whether or not you want to use the measurements in the estimate of error, or just the caliper error you inputted above. You'll probably get smaller error estimates here, but they will likely be smaller than they actually are</t>
+  </si>
+  <si>
+    <t>Is your printer coreXY?</t>
+  </si>
+  <si>
+    <t>Set TRUE for coreXY, otherwise set to FALSE</t>
+  </si>
+  <si>
+    <t>Tips for best results:</t>
+  </si>
+  <si>
+    <t>1. Allow the print to cool completely before measuring</t>
+  </si>
+  <si>
+    <t>2. Remove the print from the bed</t>
   </si>
   <si>
     <t>Measure in this order:</t>
@@ -141,6 +159,18 @@
   </si>
   <si>
     <t>For best results, make sure for every outer measurement you have a corresponding inner measurement.</t>
+  </si>
+  <si>
+    <t>Read me first!</t>
+  </si>
+  <si>
+    <t>Skew cannot be iteratively tuned. Therefore, if you have already attempted to correct your skew, you should remove the correction before trying again</t>
+  </si>
+  <si>
+    <t>If you're using a CoreXY printer, ensure you have "CoreXY" set to TRUE on the Intro sheet</t>
+  </si>
+  <si>
+    <t>Ensure your current x- and y-steps are up to date on the Intro sheet</t>
   </si>
   <si>
     <t>Results</t>
@@ -326,7 +356,10 @@
     <t>Percentage</t>
   </si>
   <si>
-    <t>New E-step</t>
+    <t>Cartesian steps</t>
+  </si>
+  <si>
+    <t>CoreXY steps</t>
   </si>
   <si>
     <t>skew standard deviation</t>
@@ -339,13 +372,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.000000000000"/>
     <numFmt numFmtId="165" formatCode="#,##0.00000%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.0000000"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="0.0000000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -363,6 +397,17 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="17.0"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -370,12 +415,13 @@
     </font>
     <font>
       <sz val="11.0"/>
-      <color rgb="FF000000"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
+      <b/>
+      <sz val="13.0"/>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -555,7 +601,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="93">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -568,13 +614,19 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -593,13 +645,13 @@
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -643,6 +695,15 @@
     <xf borderId="11" fillId="0" fontId="1" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="8" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -664,11 +725,14 @@
     <xf borderId="12" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="12" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="12" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -712,7 +776,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="15" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="15" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="16" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -724,7 +788,7 @@
     <xf borderId="9" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="6" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="0" fontId="8" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -732,6 +796,12 @@
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="167" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="1" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -754,7 +824,7 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -778,7 +848,7 @@
     <xf borderId="6" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="167" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="168" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -790,13 +860,16 @@
     <xf borderId="10" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="1" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="6" fillId="0" fontId="1" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="1" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="168" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="1" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -891,14 +964,14 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6753225" cy="6553200"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1174,53 +1247,60 @@
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="1">
         <v>40.0</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="1">
         <v>40.0</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>6</v>
+      <c r="C7" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" s="3">
         <v>0.01</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" s="1" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="2"/>
-      <c r="C10" s="2"/>
+      <c r="A10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="2"/>
@@ -5204,8 +5284,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>12</v>
+      <c r="A1" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5214,49 +5294,39 @@
       <c r="G1" s="1"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="A2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="A3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="2"/>
-      <c r="B4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="2"/>
-      <c r="B5" s="1" t="s">
+      <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -5274,22 +5344,23 @@
       <c r="G6" s="1"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2"/>
+      <c r="B7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="2"/>
+      <c r="C7" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="5" t="s">
+      <c r="A8" s="2"/>
+      <c r="B8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="C8" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E8" s="1"/>
@@ -5297,692 +5368,719 @@
       <c r="G8" s="1"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8" t="s">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="2"/>
+      <c r="B10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="C10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="B11" s="6"/>
+      <c r="C11" s="2"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="D12" s="8" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="7" t="s">
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="9"/>
+      <c r="B13" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="8">
+      <c r="C13" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="10">
         <f>IF(1 &lt;= Intro!B$3, 1, "")</f>
         <v>1</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C14" s="13">
         <f>IF(Helper!C4,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="15" t="str">
-        <f t="shared" ref="G10:G37" si="1">IF(OR(B10="",ISBLANK(D10)), "", AVERAGE(D10:F10))</f>
+      <c r="D14" s="14"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="17" t="str">
+        <f t="shared" ref="G14:G41" si="1">IF(OR(B14="",ISBLANK(D14)), "", AVERAGE(D14:F14))</f>
         <v/>
       </c>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="16"/>
-      <c r="B11" s="1">
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="18"/>
+      <c r="B15" s="1">
         <f>IF(2 &lt;= Intro!B$3, 2, "")</f>
         <v>2</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C15" s="19">
         <f>IF(Helper!C5,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D11" s="18"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="21" t="str">
+      <c r="D15" s="20"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="16"/>
-      <c r="B12" s="1">
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="18"/>
+      <c r="B16" s="1">
         <f>IF(3 &lt;= Intro!B$3, 3, "")</f>
         <v>3</v>
       </c>
-      <c r="C12" s="17">
+      <c r="C16" s="19">
         <f>IF(Helper!C6, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D12" s="18"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="21" t="str">
+      <c r="D16" s="20"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="16"/>
-      <c r="B13" s="1" t="str">
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="18"/>
+      <c r="B17" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C13" s="17" t="str">
+      <c r="C17" s="19" t="str">
         <f>IF(Helper!C7,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D13" s="18"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="21" t="str">
+      <c r="D17" s="20"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="22"/>
-      <c r="B14" s="23" t="str">
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="24"/>
+      <c r="B18" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C14" s="24" t="str">
+      <c r="C18" s="26" t="str">
         <f>IF(Helper!C8,(Intro!$B$4-4*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="28" t="str">
+      <c r="D18" s="27"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="8">
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="10">
         <f>IF(1 &lt;= Intro!B$3, 1, "")</f>
         <v>1</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C19" s="13">
         <f>IF(Helper!C9,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="15" t="str">
+      <c r="D19" s="31"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="16"/>
-      <c r="B16" s="1">
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="18"/>
+      <c r="B20" s="1">
         <f>IF(2 &lt;= Intro!B$3, 2, "")</f>
         <v>2</v>
       </c>
-      <c r="C16" s="17">
+      <c r="C20" s="19">
         <f>IF(Helper!C10,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D16" s="18"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="21" t="str">
+      <c r="D20" s="20"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="16"/>
-      <c r="B17" s="1">
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="18"/>
+      <c r="B21" s="1">
         <f>IF(3 &lt;= Intro!B$3, 3, "")</f>
         <v>3</v>
       </c>
-      <c r="C17" s="17">
+      <c r="C21" s="19">
         <f>IF(Helper!C11, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D17" s="18"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="21" t="str">
+      <c r="D21" s="20"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="16"/>
-      <c r="B18" s="1" t="str">
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="18"/>
+      <c r="B22" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C18" s="17" t="str">
+      <c r="C22" s="19" t="str">
         <f>IF(Helper!C12,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D18" s="18"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="21" t="str">
+      <c r="D22" s="20"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="22"/>
-      <c r="B19" s="23" t="str">
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="24"/>
+      <c r="B23" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C19" s="24" t="str">
+      <c r="C23" s="26" t="str">
         <f>IF(Helper!C13,(Intro!$B$4-4*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D19" s="29"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="28" t="str">
+      <c r="D23" s="34"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="8">
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="10">
         <f>IF(1 &lt;= Intro!B$3, 1, "")</f>
         <v>1</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C24" s="13">
         <f>IF(Helper!C14,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D20" s="12"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="15" t="str">
+      <c r="D24" s="31"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="16"/>
-      <c r="B21" s="1">
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="18"/>
+      <c r="B25" s="1">
         <f>IF(2 &lt;= Intro!B$3, 2, "")</f>
         <v>2</v>
       </c>
-      <c r="C21" s="17">
+      <c r="C25" s="19">
         <f>IF(Helper!C15,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D21" s="18"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="21" t="str">
+      <c r="D25" s="20"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="16"/>
-      <c r="B22" s="1">
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="18"/>
+      <c r="B26" s="1">
         <f>IF(3 &lt;= Intro!B$3, 3, "")</f>
         <v>3</v>
       </c>
-      <c r="C22" s="17">
+      <c r="C26" s="19">
         <f>IF(Helper!C16, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D22" s="18"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="21" t="str">
+      <c r="D26" s="20"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="16"/>
-      <c r="B23" s="1" t="str">
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="18"/>
+      <c r="B27" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C23" s="17" t="str">
+      <c r="C27" s="19" t="str">
         <f>IF(Helper!C17,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D23" s="18"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="21" t="str">
+      <c r="D27" s="20"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="22"/>
-      <c r="B24" s="23" t="str">
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="24"/>
+      <c r="B28" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C24" s="24" t="str">
+      <c r="C28" s="26" t="str">
         <f>IF(Helper!C18,(Intro!$B$4-4*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D24" s="25"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="28" t="str">
+      <c r="D28" s="27"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" s="8">
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="10">
         <f>IF(1 &lt;= Intro!B$3, 1, "")</f>
         <v>1</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C29" s="13">
         <f>IF(Helper!C19,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D25" s="12"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="15" t="str">
+      <c r="D29" s="31"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="16"/>
-      <c r="B26" s="1">
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="18"/>
+      <c r="B30" s="1">
         <f>IF(2 &lt;= Intro!B$3, 2, "")</f>
         <v>2</v>
       </c>
-      <c r="C26" s="17">
+      <c r="C30" s="19">
         <f>IF(Helper!C20,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D26" s="18"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="21" t="str">
+      <c r="D30" s="20"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="16"/>
-      <c r="B27" s="1">
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="18"/>
+      <c r="B31" s="1">
         <f>IF(3 &lt;= Intro!B$3, 3, "")</f>
         <v>3</v>
       </c>
-      <c r="C27" s="17">
+      <c r="C31" s="19">
         <f>IF(Helper!C21, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>40</v>
       </c>
-      <c r="D27" s="18"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="21" t="str">
+      <c r="D31" s="20"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="16"/>
-      <c r="B28" s="1" t="str">
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="18"/>
+      <c r="B32" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C28" s="17" t="str">
+      <c r="C32" s="19" t="str">
         <f>IF(Helper!C22,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D28" s="18"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="21" t="str">
+      <c r="D32" s="20"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="16"/>
-      <c r="B29" s="1" t="str">
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="18"/>
+      <c r="B33" s="1" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C29" s="17" t="str">
+      <c r="C33" s="19" t="str">
         <f>IF(Helper!C23,(Intro!$B$4-4*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D29" s="18"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="21" t="str">
+      <c r="D33" s="20"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30" s="8">
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B34" s="10">
         <f>IF(2 &lt;= Intro!B$3, 1, "")</f>
         <v>1</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C34" s="13">
         <f>IF(Helper!C24,Intro!B$4*Intro!$B$5,"x")</f>
         <v>120</v>
       </c>
-      <c r="D30" s="12"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="30" t="str">
+      <c r="D34" s="31"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="33"/>
+      <c r="G34" s="35" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="16"/>
-      <c r="B31" s="1">
-        <f>IF(3 &lt;= Intro!B$3, 2, "")</f>
-        <v>2</v>
-      </c>
-      <c r="C31" s="17">
-        <f>IF(Helper!C25,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
-        <v>80</v>
-      </c>
-      <c r="D31" s="18"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="21" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="16"/>
-      <c r="B32" s="1" t="str">
-        <f>IF(4 &lt;= Intro!B$3, 3, "")</f>
-        <v/>
-      </c>
-      <c r="C32" s="17" t="str">
-        <f>IF(Helper!C26, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
-        <v>x</v>
-      </c>
-      <c r="D32" s="18"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="21" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="16"/>
-      <c r="B33" s="1" t="str">
-        <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
-        <v/>
-      </c>
-      <c r="C33" s="17" t="str">
-        <f>IF(Helper!C27,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
-        <v>x</v>
-      </c>
-      <c r="D33" s="18"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="21" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" s="8">
-        <f>IF(2 &lt;= Intro!B$3, 1, "")</f>
-        <v>1</v>
-      </c>
-      <c r="C34" s="11">
-        <f>IF(Helper!C28,Intro!B$4*Intro!$B$5,"x")</f>
-        <v>120</v>
-      </c>
-      <c r="D34" s="12"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="30" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="16"/>
+      <c r="A35" s="18"/>
       <c r="B35" s="1">
         <f>IF(3 &lt;= Intro!B$3, 2, "")</f>
         <v>2</v>
       </c>
-      <c r="C35" s="17">
-        <f>IF(Helper!C29,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
+      <c r="C35" s="19">
+        <f>IF(Helper!C25,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>80</v>
       </c>
-      <c r="D35" s="18"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="31" t="str">
+      <c r="D35" s="20"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="16"/>
+      <c r="A36" s="18"/>
       <c r="B36" s="1" t="str">
         <f>IF(4 &lt;= Intro!B$3, 3, "")</f>
         <v/>
       </c>
-      <c r="C36" s="17" t="str">
+      <c r="C36" s="19" t="str">
+        <f>IF(Helper!C26, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
+        <v>x</v>
+      </c>
+      <c r="D36" s="20"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="18"/>
+      <c r="B37" s="1" t="str">
+        <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
+        <v/>
+      </c>
+      <c r="C37" s="19" t="str">
+        <f>IF(Helper!C27,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
+        <v>x</v>
+      </c>
+      <c r="D37" s="20"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="10">
+        <f>IF(2 &lt;= Intro!B$3, 1, "")</f>
+        <v>1</v>
+      </c>
+      <c r="C38" s="13">
+        <f>IF(Helper!C28,Intro!B$4*Intro!$B$5,"x")</f>
+        <v>120</v>
+      </c>
+      <c r="D38" s="31"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="33"/>
+      <c r="G38" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="18"/>
+      <c r="B39" s="1">
+        <f>IF(3 &lt;= Intro!B$3, 2, "")</f>
+        <v>2</v>
+      </c>
+      <c r="C39" s="19">
+        <f>IF(Helper!C29,(Intro!$B$4-Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
+        <v>80</v>
+      </c>
+      <c r="D39" s="20"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="36" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="18"/>
+      <c r="B40" s="1" t="str">
+        <f>IF(4 &lt;= Intro!B$3, 3, "")</f>
+        <v/>
+      </c>
+      <c r="C40" s="19" t="str">
         <f>IF(Helper!C30, (Intro!$B$4-Intro!$B$4/Intro!$B$3*2)*Intro!$B$5, "x")</f>
         <v>x</v>
       </c>
-      <c r="D36" s="18"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="31" t="str">
+      <c r="D40" s="20"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="36" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="22"/>
-      <c r="B37" s="23" t="str">
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="24"/>
+      <c r="B41" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C37" s="24" t="str">
+      <c r="C41" s="26" t="str">
         <f>IF(Helper!C31,(Intro!$B$4-3*Intro!$B$4/Intro!$B$3)*Intro!$B$5,"x")</f>
         <v>x</v>
       </c>
-      <c r="D37" s="25"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="32" t="str">
+      <c r="D41" s="27"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="37" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="1"/>
-      <c r="B38" s="1"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="33"/>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-    </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
-      <c r="E40" s="34"/>
-      <c r="F40" s="34"/>
-      <c r="G40" s="34"/>
-      <c r="H40" s="34"/>
-      <c r="I40" s="34"/>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="B41" s="35"/>
-      <c r="C41" s="35"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="35"/>
-      <c r="F41" s="35"/>
-      <c r="G41" s="35"/>
-      <c r="H41" s="35"/>
-      <c r="I41" s="35"/>
-    </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="36" t="s">
-        <v>38</v>
-      </c>
-      <c r="B42" s="36"/>
-      <c r="C42" s="36"/>
-      <c r="D42" s="36"/>
-      <c r="E42" s="36"/>
-      <c r="F42" s="36"/>
-      <c r="G42" s="36"/>
-      <c r="H42" s="36"/>
-      <c r="I42" s="36"/>
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="21"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="21"/>
+      <c r="G42" s="38"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B43" s="1"/>
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
       <c r="C43" s="2"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="1"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
+      <c r="A44" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" s="39"/>
+      <c r="C44" s="39"/>
+      <c r="D44" s="39"/>
+      <c r="E44" s="39"/>
+      <c r="F44" s="39"/>
+      <c r="G44" s="39"/>
+      <c r="H44" s="39"/>
+      <c r="I44" s="39"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="1"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="W45" s="37"/>
-      <c r="X45" s="37"/>
+      <c r="A45" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" s="40"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="40"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="40"/>
+      <c r="I45" s="40"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="W46" s="37"/>
-      <c r="X46" s="37"/>
+      <c r="A46" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" s="41"/>
+      <c r="C46" s="41"/>
+      <c r="D46" s="41"/>
+      <c r="E46" s="41"/>
+      <c r="F46" s="41"/>
+      <c r="G46" s="41"/>
+      <c r="H46" s="41"/>
+      <c r="I46" s="41"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="1"/>
-      <c r="B47" s="2"/>
+      <c r="A47" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B47" s="1"/>
       <c r="C47" s="2"/>
-      <c r="L47" s="37"/>
-      <c r="O47" s="37"/>
-      <c r="P47" s="37"/>
-      <c r="W47" s="37"/>
-      <c r="X47" s="37"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="1"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
-      <c r="L48" s="37"/>
-      <c r="O48" s="37"/>
-      <c r="P48" s="37"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="1"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
+      <c r="W49" s="42"/>
+      <c r="X49" s="42"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="1"/>
+      <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
-      <c r="W50" s="19"/>
-      <c r="X50" s="19"/>
+      <c r="W50" s="42"/>
+      <c r="X50" s="42"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="1"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="L51" s="19"/>
-      <c r="O51" s="19"/>
-      <c r="P51" s="19"/>
-      <c r="S51" s="19"/>
-      <c r="T51" s="19"/>
-      <c r="W51" s="19"/>
-      <c r="X51" s="19"/>
+      <c r="L51" s="42"/>
+      <c r="O51" s="42"/>
+      <c r="P51" s="42"/>
+      <c r="W51" s="42"/>
+      <c r="X51" s="42"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="1"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="L52" s="19"/>
-      <c r="O52" s="19"/>
-      <c r="P52" s="19"/>
-      <c r="S52" s="19"/>
-      <c r="T52" s="19"/>
+      <c r="L52" s="42"/>
+      <c r="O52" s="42"/>
+      <c r="P52" s="42"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="2"/>
+      <c r="A53" s="1"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="2"/>
+      <c r="A54" s="1"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
+      <c r="W54" s="21"/>
+      <c r="X54" s="21"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="1"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
+      <c r="L55" s="21"/>
+      <c r="O55" s="21"/>
+      <c r="P55" s="21"/>
+      <c r="S55" s="21"/>
+      <c r="T55" s="21"/>
+      <c r="W55" s="21"/>
+      <c r="X55" s="21"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="2"/>
+      <c r="A56" s="1"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
+      <c r="L56" s="21"/>
+      <c r="O56" s="21"/>
+      <c r="P56" s="21"/>
+      <c r="S56" s="21"/>
+      <c r="T56" s="21"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="2"/>
@@ -5995,7 +6093,7 @@
       <c r="C58" s="2"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="2"/>
+      <c r="A59" s="1"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
     </row>
@@ -10879,26 +10977,46 @@
       <c r="B1035" s="2"/>
       <c r="C1035" s="2"/>
     </row>
+    <row r="1036" ht="15.75" customHeight="1">
+      <c r="A1036" s="2"/>
+      <c r="B1036" s="2"/>
+      <c r="C1036" s="2"/>
+    </row>
+    <row r="1037" ht="15.75" customHeight="1">
+      <c r="A1037" s="2"/>
+      <c r="B1037" s="2"/>
+      <c r="C1037" s="2"/>
+    </row>
+    <row r="1038" ht="15.75" customHeight="1">
+      <c r="A1038" s="2"/>
+      <c r="B1038" s="2"/>
+      <c r="C1038" s="2"/>
+    </row>
+    <row r="1039" ht="15.75" customHeight="1">
+      <c r="A1039" s="2"/>
+      <c r="B1039" s="2"/>
+      <c r="C1039" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$C$9:$C$37"/>
-  <conditionalFormatting sqref="D10:F38">
+  <autoFilter ref="$C$13:$C$41"/>
+  <conditionalFormatting sqref="D14:F42">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>LEN(TRIM(D10))=0</formula>
+      <formula>LEN(TRIM(D14))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D10:F38">
+  <conditionalFormatting sqref="D14:F42">
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>ABS(D10-$C10)&lt;=0.5</formula>
+      <formula>ABS(D14-$C14)&lt;=0.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D10:F38">
+  <conditionalFormatting sqref="D14:F42">
     <cfRule type="expression" dxfId="2" priority="3">
-      <formula>ABS(D10-$C10)&lt;=1</formula>
+      <formula>ABS(D14-$C14)&lt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D10:F38">
+  <conditionalFormatting sqref="D14:F42">
     <cfRule type="expression" dxfId="3" priority="4">
-      <formula>ABS(D10-$C10)&gt;1</formula>
+      <formula>ABS(D14-$C14)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions/>
@@ -10920,375 +11038,407 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="9"/>
+      <c r="A1" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="16" t="s">
-        <v>41</v>
+      <c r="A2" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="38"/>
+      <c r="E2" s="1"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="16"/>
+      <c r="A3" s="3" t="s">
+        <v>48</v>
+      </c>
       <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="40"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37" t="str">
+      <c r="A4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="11"/>
+    </row>
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="44"/>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="18"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" s="45" t="s">
+        <v>55</v>
+      </c>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="46"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="42"/>
+      <c r="C10" s="42" t="str">
         <f>Helper!E43</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D4" s="41">
+      <c r="D10" s="47">
         <f>SQRT(SUMSQ(Helper!K4:K13))</f>
         <v>0</v>
       </c>
-      <c r="E4" s="42" t="str">
-        <f t="shared" ref="E4:E5" si="1">-C4</f>
+      <c r="E10" s="48" t="str">
+        <f t="shared" ref="E10:E11" si="1">-C10</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G4" s="43" t="s">
-        <v>47</v>
-      </c>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="44"/>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37" t="str">
+      <c r="G10" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="H10" s="39"/>
+      <c r="I10" s="39"/>
+      <c r="J10" s="50"/>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42" t="str">
         <f>Helper!E44</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D5" s="41">
+      <c r="D11" s="47">
         <f>SQRT(SUMSQ(Helper!K14:K23))</f>
         <v>0</v>
       </c>
-      <c r="E5" s="42" t="str">
+      <c r="E11" s="48" t="str">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="G5" s="45" t="s">
-        <v>49</v>
-      </c>
-      <c r="H5" s="35"/>
-      <c r="I5" s="35"/>
-      <c r="J5" s="46"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="38"/>
-      <c r="G6" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="49"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="16"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48" t="s">
+      <c r="G11" s="51" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="52"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="21"/>
+      <c r="E12" s="44"/>
+      <c r="G12" s="53" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" s="54"/>
+      <c r="I12" s="54"/>
+      <c r="J12" s="55"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="18"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="50"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="16" t="s">
+      <c r="E13" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19" t="str">
+      <c r="G13" s="53"/>
+      <c r="H13" s="54" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" s="54"/>
+      <c r="J13" s="56"/>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21" t="str">
         <f>Helper!B41</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D8" s="51" t="str">
+      <c r="D14" s="57" t="str">
         <f>Helper!B43</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E8" s="20"/>
-      <c r="G8" s="52" t="s">
-        <v>55</v>
-      </c>
-      <c r="H8" s="53"/>
-      <c r="I8" s="53"/>
-      <c r="J8" s="54"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26" t="str">
-        <f>C8-90</f>
+      <c r="E14" s="22"/>
+      <c r="G14" s="58" t="s">
+        <v>65</v>
+      </c>
+      <c r="H14" s="59"/>
+      <c r="I14" s="59"/>
+      <c r="J14" s="60"/>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28" t="str">
+        <f>C14-90</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D9" s="55" t="str">
+      <c r="D15" s="61" t="str">
         <f>Helper!B43</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E9" s="27" t="str">
-        <f>-C9</f>
+      <c r="E15" s="29" t="str">
+        <f>-C15</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J9" s="19"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="1"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="9"/>
-      <c r="H12" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="9"/>
-    </row>
-    <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="56" t="s">
-        <v>60</v>
-      </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="38"/>
-      <c r="H13" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="M13" s="38"/>
-    </row>
-    <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="38"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="1" t="str">
+      <c r="J15" s="21"/>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="1"/>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="11"/>
+      <c r="H18" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="11"/>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="62" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" s="1"/>
+      <c r="F19" s="44"/>
+      <c r="H19" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="M19" s="44"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="44"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="1" t="str">
         <f>"M92 X"&amp;ROUND(Helper!F43,3)&amp;" Y"&amp;ROUND(Helper!F44,3)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="M14" s="38"/>
-    </row>
-    <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="18" t="str">
+      <c r="M20" s="44"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="20" t="str">
         <f>"Length AC = "&amp;ROUND(Helper!B36,Helper!C36)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E15" s="1"/>
-      <c r="F15" s="38"/>
-      <c r="H15" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="M15" s="38"/>
-    </row>
-    <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="18" t="str">
+      <c r="E21" s="1"/>
+      <c r="F21" s="44"/>
+      <c r="H21" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="M21" s="44"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="20" t="str">
         <f>"Length BD = "&amp;ROUND(Helper!B37,Helper!C37)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F16" s="38"/>
-      <c r="H16" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="M16" s="38"/>
-    </row>
-    <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="18" t="str">
+      <c r="F22" s="44"/>
+      <c r="H22" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="M22" s="44"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="20" t="str">
         <f>"Length AD = "&amp;ROUND(Helper!B38,Helper!C38)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F17" s="38"/>
-      <c r="H17" s="16"/>
-      <c r="M17" s="38"/>
-    </row>
-    <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="57"/>
-      <c r="F18" s="38"/>
-      <c r="H18" s="16"/>
-      <c r="M18" s="38"/>
-    </row>
-    <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="57" t="s">
-        <v>65</v>
-      </c>
-      <c r="F19" s="38"/>
-      <c r="H19" s="16"/>
-      <c r="M19" s="38"/>
-    </row>
-    <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="57" t="s">
-        <v>66</v>
-      </c>
-      <c r="F20" s="38"/>
-      <c r="H20" s="16"/>
-      <c r="M20" s="38"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="57" t="str">
+      <c r="F23" s="44"/>
+      <c r="H23" s="18"/>
+      <c r="M23" s="44"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="63"/>
+      <c r="F24" s="44"/>
+      <c r="H24" s="18"/>
+      <c r="M24" s="44"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="63" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" s="44"/>
+      <c r="H25" s="18"/>
+      <c r="M25" s="44"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" s="44"/>
+      <c r="H26" s="18"/>
+      <c r="M26" s="44"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="63" t="str">
         <f>"SET_SKEW XY="&amp;ROUND(Helper!B36,Helper!C36)&amp;","&amp;ROUND(Helper!B37,Helper!C37)&amp;","&amp;ROUND(Helper!B38,Helper!C37)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F21" s="38"/>
-      <c r="H21" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="M21" s="38"/>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="58" t="s">
-        <v>68</v>
-      </c>
-      <c r="F22" s="38"/>
-      <c r="H22" s="16"/>
-      <c r="M22" s="38"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="16"/>
-      <c r="F23" s="38"/>
-      <c r="H23" s="16"/>
-      <c r="M23" s="38"/>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="F24" s="38"/>
-      <c r="H24" s="16"/>
-      <c r="M24" s="38"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="16" t="str">
+      <c r="F27" s="44"/>
+      <c r="H27" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="M27" s="44"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="64" t="s">
+        <v>78</v>
+      </c>
+      <c r="F28" s="44"/>
+      <c r="H28" s="18"/>
+      <c r="M28" s="44"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="18"/>
+      <c r="F29" s="44"/>
+      <c r="H29" s="18"/>
+      <c r="M29" s="44"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" s="44"/>
+      <c r="H30" s="18"/>
+      <c r="M30" s="44"/>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="18" t="str">
         <f>"CALC_MEASURED_SKEW AC="&amp;ROUND(Helper!B36,Helper!C36)&amp;" BD="&amp;ROUND(Helper!B37,Helper!C37)&amp;" AD="&amp;ROUND(Helper!B38,Helper!C37)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F25" s="38"/>
-      <c r="H25" s="16"/>
-      <c r="M25" s="38"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="16"/>
-      <c r="F26" s="38"/>
-      <c r="H26" s="16"/>
-      <c r="M26" s="38"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="F27" s="38"/>
-      <c r="H27" s="16"/>
-      <c r="M27" s="38"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="B28" s="1" t="str">
-        <f>ROUND(Helper!F43,3)</f>
+      <c r="F31" s="44"/>
+      <c r="H31" s="18"/>
+      <c r="M31" s="44"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="18"/>
+      <c r="F32" s="44"/>
+      <c r="H32" s="18"/>
+      <c r="M32" s="44"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="F33" s="44"/>
+      <c r="H33" s="18"/>
+      <c r="M33" s="44"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B34" s="65" t="str">
+        <f>IF(Intro!B10, ROUND(Helper!G43,3),ROUND(Helper!F43,3))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F28" s="38"/>
-      <c r="H28" s="16"/>
-      <c r="M28" s="38"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="B29" s="23" t="str">
-        <f>ROUND(Helper!F44,3)</f>
+      <c r="C34" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F34" s="44"/>
+      <c r="H34" s="18"/>
+      <c r="M34" s="44"/>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" s="66" t="str">
+        <f>IF(Intro!B10, ROUND(Helper!G44,3),ROUND(Helper!F44,3))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C29" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="59"/>
-      <c r="H29" s="22"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="23"/>
-      <c r="K29" s="23"/>
-      <c r="L29" s="23"/>
-      <c r="M29" s="59"/>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="2"/>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="2"/>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="2"/>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="2"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="2"/>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="2"/>
+      <c r="C35" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="D35" s="25"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="67"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="25"/>
+      <c r="K35" s="25"/>
+      <c r="L35" s="25"/>
+      <c r="M35" s="67"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="2"/>
@@ -14209,49 +14359,67 @@
     <row r="1008" ht="15.75" customHeight="1">
       <c r="A1008" s="2"/>
     </row>
+    <row r="1009" ht="15.75" customHeight="1">
+      <c r="A1009" s="2"/>
+    </row>
+    <row r="1010" ht="15.75" customHeight="1">
+      <c r="A1010" s="2"/>
+    </row>
+    <row r="1011" ht="15.75" customHeight="1">
+      <c r="A1011" s="2"/>
+    </row>
+    <row r="1012" ht="15.75" customHeight="1">
+      <c r="A1012" s="2"/>
+    </row>
+    <row r="1013" ht="15.75" customHeight="1">
+      <c r="A1013" s="2"/>
+    </row>
+    <row r="1014" ht="15.75" customHeight="1">
+      <c r="A1014" s="2"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B4:E5">
+  <conditionalFormatting sqref="B10:E11">
     <cfRule type="expression" dxfId="1" priority="1">
-      <formula>ABS($C4)/$D4&lt;=1</formula>
+      <formula>ABS($C10)/$D10&lt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:E5">
+  <conditionalFormatting sqref="B10:E11">
     <cfRule type="expression" dxfId="2" priority="2">
-      <formula>ABS($C4)/$D4&lt;=2</formula>
+      <formula>ABS($C10)/$D10&lt;=2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:E5">
+  <conditionalFormatting sqref="B10:E11">
     <cfRule type="expression" dxfId="4" priority="3">
-      <formula>ABS($C4)/$D4&lt;=3</formula>
+      <formula>ABS($C10)/$D10&lt;=3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:E5">
+  <conditionalFormatting sqref="B10:E11">
     <cfRule type="expression" dxfId="3" priority="4">
-      <formula>ABS($C4)/$D4&gt;3</formula>
+      <formula>ABS($C10)/$D10&gt;3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E9">
+  <conditionalFormatting sqref="B14:E15">
     <cfRule type="expression" dxfId="1" priority="5">
-      <formula>ABS($C$8-90)/$D$8&lt;=1</formula>
+      <formula>ABS($C$14-90)/$D$14&lt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E9">
+  <conditionalFormatting sqref="B14:E15">
     <cfRule type="expression" dxfId="2" priority="6">
-      <formula>ABS($C$8-90)/$D$8&lt;=2</formula>
+      <formula>ABS($C$14-90)/$D$14&lt;=2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E9">
+  <conditionalFormatting sqref="B14:E15">
     <cfRule type="expression" dxfId="4" priority="7">
-      <formula>ABS($C$8-90)/$D$8&lt;=3</formula>
+      <formula>ABS($C$14-90)/$D$14&lt;=3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:E9">
+  <conditionalFormatting sqref="B14:E15">
     <cfRule type="expression" dxfId="3" priority="8">
-      <formula>ABS($C$8-90)/$D$8&gt;3</formula>
+      <formula>ABS($C$14-90)/$D$14&gt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A13"/>
+    <hyperlink r:id="rId1" ref="A19"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.984027777777778" footer="0.0" header="0.0" left="0.747916666666667" right="0.747916666666667" top="0.984027777777778"/>
@@ -14276,7 +14444,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B1" s="2"/>
       <c r="G1" s="2"/>
@@ -14289,77 +14457,77 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="B3" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>25</v>
+        <v>87</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>31</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="8">
+      <c r="A4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="10">
         <f>IF(1 &lt;= Intro!B$3, 1, "")</f>
         <v>1</v>
       </c>
-      <c r="C4" s="8" t="b">
+      <c r="C4" s="10" t="b">
         <f t="shared" ref="C4:C31" si="1">NOT(B4="")</f>
         <v>1</v>
       </c>
-      <c r="D4" s="8" t="b">
+      <c r="D4" s="10" t="b">
         <f t="shared" ref="D4:D31" si="2">IFERROR(AND(NOT(F4=0),NOT(F4=""),C4),FALSE())</f>
         <v>0</v>
       </c>
-      <c r="E4" s="60">
-        <f>IF(D4,'Post-print worksheet'!C10,0)</f>
+      <c r="E4" s="68">
+        <f>IF(D4,'Post-print worksheet'!C14,0)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="13" t="str">
-        <f>IF(C4, IFERROR(AVERAGE('Post-print worksheet'!D10:F10),""),"")</f>
+      <c r="F4" s="32" t="str">
+        <f>IF(C4, IFERROR(AVERAGE('Post-print worksheet'!D14:F14),""),"")</f>
         <v/>
       </c>
-      <c r="G4" s="13">
-        <f>IF(C4, IFERROR(STDEV('Post-print worksheet'!D10:F10),0),"")</f>
+      <c r="G4" s="32">
+        <f>IF(C4, IFERROR(STDEV('Post-print worksheet'!D14:F14),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H4" s="13">
+      <c r="H4" s="32">
         <f>IF(C4, IFERROR(SQRT((Intro!$B$8/3)^2+G4^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I4" s="13" t="str">
+      <c r="I4" s="32" t="str">
         <f t="shared" ref="I4:I31" si="3">IF(D4, IFERROR((F4-E4)/E4,0),"")</f>
         <v/>
       </c>
-      <c r="J4" s="13" t="str">
+      <c r="J4" s="32" t="str">
         <f t="shared" ref="J4:J22" si="4">IF(D4, 1/(($B$47+$B$48)*E4),"")</f>
         <v/>
       </c>
-      <c r="K4" s="13" t="str">
+      <c r="K4" s="32" t="str">
         <f t="shared" ref="K4:K23" si="5">IF(D4,J4*H4,"")</f>
         <v/>
       </c>
@@ -14378,31 +14546,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E5" s="61">
-        <f>IF(D5,'Post-print worksheet'!C11,0)</f>
+      <c r="E5" s="69">
+        <f>IF(D5,'Post-print worksheet'!C15,0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="19" t="str">
-        <f>IF(C5, IFERROR(AVERAGE('Post-print worksheet'!D11:F11),""),"")</f>
+      <c r="F5" s="21" t="str">
+        <f>IF(C5, IFERROR(AVERAGE('Post-print worksheet'!D15:F15),""),"")</f>
         <v/>
       </c>
-      <c r="G5" s="19">
-        <f>IF(C5, IFERROR(STDEV('Post-print worksheet'!D11:F11),0),"")</f>
+      <c r="G5" s="21">
+        <f>IF(C5, IFERROR(STDEV('Post-print worksheet'!D15:F15),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="21">
         <f>IF(C5, IFERROR(SQRT((Intro!$B$8/3)^2+G5^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I5" s="19" t="str">
+      <c r="I5" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J5" s="19" t="str">
+      <c r="J5" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K5" s="19" t="str">
+      <c r="K5" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14421,31 +14589,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E6" s="61">
-        <f>IF(D6,'Post-print worksheet'!C12,0)</f>
+      <c r="E6" s="69">
+        <f>IF(D6,'Post-print worksheet'!C16,0)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="19" t="str">
-        <f>IF(C6, IFERROR(AVERAGE('Post-print worksheet'!D12:F12),""),"")</f>
+      <c r="F6" s="21" t="str">
+        <f>IF(C6, IFERROR(AVERAGE('Post-print worksheet'!D16:F16),""),"")</f>
         <v/>
       </c>
-      <c r="G6" s="19">
-        <f>IF(C6, IFERROR(STDEV('Post-print worksheet'!D12:F12),0),"")</f>
+      <c r="G6" s="21">
+        <f>IF(C6, IFERROR(STDEV('Post-print worksheet'!D16:F16),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="21">
         <f>IF(C6, IFERROR(SQRT((Intro!$B$8/3)^2+G6^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I6" s="19" t="str">
+      <c r="I6" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J6" s="19" t="str">
+      <c r="J6" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K6" s="19" t="str">
+      <c r="K6" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14464,81 +14632,81 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E7" s="61">
-        <f>IF(D7,'Post-print worksheet'!C13,0)</f>
+      <c r="E7" s="69">
+        <f>IF(D7,'Post-print worksheet'!C17,0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="19" t="str">
-        <f>IF(C7, IFERROR(AVERAGE('Post-print worksheet'!D13:F13),""),"")</f>
+      <c r="F7" s="21" t="str">
+        <f>IF(C7, IFERROR(AVERAGE('Post-print worksheet'!D17:F17),""),"")</f>
         <v/>
       </c>
-      <c r="G7" s="19" t="str">
-        <f>IF(C7, IFERROR(STDEV('Post-print worksheet'!D13:F13),0),"")</f>
+      <c r="G7" s="21" t="str">
+        <f>IF(C7, IFERROR(STDEV('Post-print worksheet'!D17:F17),0),"")</f>
         <v/>
       </c>
-      <c r="H7" s="19" t="str">
+      <c r="H7" s="21" t="str">
         <f>IF(C7, IFERROR(SQRT((Intro!$B$8/3)^2+G7^2),0),"")</f>
         <v/>
       </c>
-      <c r="I7" s="19" t="str">
+      <c r="I7" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J7" s="19" t="str">
+      <c r="J7" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K7" s="19" t="str">
+      <c r="K7" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="23"/>
-      <c r="B8" s="23" t="str">
+      <c r="A8" s="25"/>
+      <c r="B8" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C8" s="23" t="b">
+      <c r="C8" s="25" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D8" s="23" t="b">
+      <c r="D8" s="25" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E8" s="62">
-        <f>IF(D8,'Post-print worksheet'!C14,0)</f>
+      <c r="E8" s="70">
+        <f>IF(D8,'Post-print worksheet'!C18,0)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="26" t="str">
-        <f>IF(C8, IFERROR(AVERAGE('Post-print worksheet'!D14:F14),""),"")</f>
+      <c r="F8" s="28" t="str">
+        <f>IF(C8, IFERROR(AVERAGE('Post-print worksheet'!D18:F18),""),"")</f>
         <v/>
       </c>
-      <c r="G8" s="26" t="str">
-        <f>IF(C8, IFERROR(STDEV('Post-print worksheet'!D14:F14),0),"")</f>
+      <c r="G8" s="28" t="str">
+        <f>IF(C8, IFERROR(STDEV('Post-print worksheet'!D18:F18),0),"")</f>
         <v/>
       </c>
-      <c r="H8" s="26" t="str">
+      <c r="H8" s="28" t="str">
         <f>IF(C8, IFERROR(SQRT((Intro!$B$8/3)^2+G8^2),0),"")</f>
         <v/>
       </c>
-      <c r="I8" s="26" t="str">
+      <c r="I8" s="28" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J8" s="26" t="str">
+      <c r="J8" s="28" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K8" s="26" t="str">
+      <c r="K8" s="28" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B9" s="1">
         <f>IF(1 &lt;= Intro!B$3, 1, "")</f>
@@ -14552,31 +14720,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E9" s="61">
-        <f>IF(D9,'Post-print worksheet'!C15,0)</f>
+      <c r="E9" s="69">
+        <f>IF(D9,'Post-print worksheet'!C19,0)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="19" t="str">
-        <f>IF(C9, IFERROR(AVERAGE('Post-print worksheet'!D15:F15),""),"")</f>
+      <c r="F9" s="21" t="str">
+        <f>IF(C9, IFERROR(AVERAGE('Post-print worksheet'!D19:F19),""),"")</f>
         <v/>
       </c>
-      <c r="G9" s="19">
-        <f>IF(C9, IFERROR(STDEV('Post-print worksheet'!D15:F15),0),"")</f>
+      <c r="G9" s="21">
+        <f>IF(C9, IFERROR(STDEV('Post-print worksheet'!D19:F19),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="21">
         <f>IF(C9, IFERROR(SQRT((Intro!$B$8/3)^2+G9^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I9" s="19" t="str">
+      <c r="I9" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J9" s="19" t="str">
+      <c r="J9" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K9" s="19" t="str">
+      <c r="K9" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14595,31 +14763,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E10" s="61">
-        <f>IF(D10,'Post-print worksheet'!C16,0)</f>
+      <c r="E10" s="69">
+        <f>IF(D10,'Post-print worksheet'!C20,0)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="19" t="str">
-        <f>IF(C10, IFERROR(AVERAGE('Post-print worksheet'!D16:F16),""),"")</f>
+      <c r="F10" s="21" t="str">
+        <f>IF(C10, IFERROR(AVERAGE('Post-print worksheet'!D20:F20),""),"")</f>
         <v/>
       </c>
-      <c r="G10" s="19">
-        <f>IF(C10, IFERROR(STDEV('Post-print worksheet'!D16:F16),0),"")</f>
+      <c r="G10" s="21">
+        <f>IF(C10, IFERROR(STDEV('Post-print worksheet'!D20:F20),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="21">
         <f>IF(C10, IFERROR(SQRT((Intro!$B$8/3)^2+G10^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I10" s="19" t="str">
+      <c r="I10" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J10" s="19" t="str">
+      <c r="J10" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K10" s="19" t="str">
+      <c r="K10" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14638,31 +14806,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E11" s="61">
-        <f>IF(D11,'Post-print worksheet'!C17,0)</f>
+      <c r="E11" s="69">
+        <f>IF(D11,'Post-print worksheet'!C21,0)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="19" t="str">
-        <f>IF(C11, IFERROR(AVERAGE('Post-print worksheet'!D17:F17),""),"")</f>
+      <c r="F11" s="21" t="str">
+        <f>IF(C11, IFERROR(AVERAGE('Post-print worksheet'!D21:F21),""),"")</f>
         <v/>
       </c>
-      <c r="G11" s="19">
-        <f>IF(C11, IFERROR(STDEV('Post-print worksheet'!D17:F17),0),"")</f>
+      <c r="G11" s="21">
+        <f>IF(C11, IFERROR(STDEV('Post-print worksheet'!D21:F21),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="21">
         <f>IF(C11, IFERROR(SQRT((Intro!$B$8/3)^2+G11^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I11" s="19" t="str">
+      <c r="I11" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J11" s="19" t="str">
+      <c r="J11" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K11" s="19" t="str">
+      <c r="K11" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14681,81 +14849,81 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E12" s="61">
-        <f>IF(D12,'Post-print worksheet'!C18,0)</f>
+      <c r="E12" s="69">
+        <f>IF(D12,'Post-print worksheet'!C22,0)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="19" t="str">
-        <f>IF(C12, IFERROR(AVERAGE('Post-print worksheet'!D18:F18),""),"")</f>
+      <c r="F12" s="21" t="str">
+        <f>IF(C12, IFERROR(AVERAGE('Post-print worksheet'!D22:F22),""),"")</f>
         <v/>
       </c>
-      <c r="G12" s="19" t="str">
-        <f>IF(C12, IFERROR(STDEV('Post-print worksheet'!D18:F18),0),"")</f>
+      <c r="G12" s="21" t="str">
+        <f>IF(C12, IFERROR(STDEV('Post-print worksheet'!D22:F22),0),"")</f>
         <v/>
       </c>
-      <c r="H12" s="19" t="str">
+      <c r="H12" s="21" t="str">
         <f>IF(C12, IFERROR(SQRT((Intro!$B$8/3)^2+G12^2),0),"")</f>
         <v/>
       </c>
-      <c r="I12" s="19" t="str">
+      <c r="I12" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J12" s="19" t="str">
+      <c r="J12" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K12" s="19" t="str">
+      <c r="K12" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="23"/>
-      <c r="B13" s="23" t="str">
+      <c r="A13" s="25"/>
+      <c r="B13" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C13" s="23" t="b">
+      <c r="C13" s="25" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D13" s="23" t="b">
+      <c r="D13" s="25" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E13" s="62">
-        <f>IF(D13,'Post-print worksheet'!C19,0)</f>
+      <c r="E13" s="70">
+        <f>IF(D13,'Post-print worksheet'!C23,0)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="26" t="str">
-        <f>IF(C13, IFERROR(AVERAGE('Post-print worksheet'!D19:F19),""),"")</f>
+      <c r="F13" s="28" t="str">
+        <f>IF(C13, IFERROR(AVERAGE('Post-print worksheet'!D23:F23),""),"")</f>
         <v/>
       </c>
-      <c r="G13" s="26" t="str">
-        <f>IF(C13, IFERROR(STDEV('Post-print worksheet'!D19:F19),0),"")</f>
+      <c r="G13" s="28" t="str">
+        <f>IF(C13, IFERROR(STDEV('Post-print worksheet'!D23:F23),0),"")</f>
         <v/>
       </c>
-      <c r="H13" s="26" t="str">
+      <c r="H13" s="28" t="str">
         <f>IF(C13, IFERROR(SQRT((Intro!$B$8/3)^2+G13^2),0),"")</f>
         <v/>
       </c>
-      <c r="I13" s="26" t="str">
+      <c r="I13" s="28" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J13" s="26" t="str">
+      <c r="J13" s="28" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K13" s="26" t="str">
+      <c r="K13" s="28" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B14" s="1">
         <f>IF(1 &lt;= Intro!B$3, 1, "")</f>
@@ -14769,31 +14937,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E14" s="61">
-        <f>IF(D14,'Post-print worksheet'!C20,0)</f>
+      <c r="E14" s="69">
+        <f>IF(D14,'Post-print worksheet'!C24,0)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="19" t="str">
-        <f>IF(C14, IFERROR(AVERAGE('Post-print worksheet'!D20:F20),""),"")</f>
+      <c r="F14" s="21" t="str">
+        <f>IF(C14, IFERROR(AVERAGE('Post-print worksheet'!D24:F24),""),"")</f>
         <v/>
       </c>
-      <c r="G14" s="19">
-        <f>IF(C14, IFERROR(STDEV('Post-print worksheet'!D20:F20),0),"")</f>
+      <c r="G14" s="21">
+        <f>IF(C14, IFERROR(STDEV('Post-print worksheet'!D24:F24),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="21">
         <f>IF(C14, IFERROR(SQRT((Intro!$B$8/3)^2+G14^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I14" s="19" t="str">
+      <c r="I14" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J14" s="19" t="str">
+      <c r="J14" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K14" s="19" t="str">
+      <c r="K14" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14812,31 +14980,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E15" s="61">
-        <f>IF(D15,'Post-print worksheet'!C21,0)</f>
+      <c r="E15" s="69">
+        <f>IF(D15,'Post-print worksheet'!C25,0)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="19" t="str">
-        <f>IF(C15, IFERROR(AVERAGE('Post-print worksheet'!D21:F21),""),"")</f>
+      <c r="F15" s="21" t="str">
+        <f>IF(C15, IFERROR(AVERAGE('Post-print worksheet'!D25:F25),""),"")</f>
         <v/>
       </c>
-      <c r="G15" s="19">
-        <f>IF(C15, IFERROR(STDEV('Post-print worksheet'!D21:F21),0),"")</f>
+      <c r="G15" s="21">
+        <f>IF(C15, IFERROR(STDEV('Post-print worksheet'!D25:F25),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H15" s="19">
+      <c r="H15" s="21">
         <f>IF(C15, IFERROR(SQRT((Intro!$B$8/3)^2+G15^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I15" s="19" t="str">
+      <c r="I15" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J15" s="19" t="str">
+      <c r="J15" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K15" s="19" t="str">
+      <c r="K15" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14855,31 +15023,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E16" s="61">
-        <f>IF(D16,'Post-print worksheet'!C22,0)</f>
+      <c r="E16" s="69">
+        <f>IF(D16,'Post-print worksheet'!C26,0)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="19" t="str">
-        <f>IF(C16, IFERROR(AVERAGE('Post-print worksheet'!D22:F22),""),"")</f>
+      <c r="F16" s="21" t="str">
+        <f>IF(C16, IFERROR(AVERAGE('Post-print worksheet'!D26:F26),""),"")</f>
         <v/>
       </c>
-      <c r="G16" s="19">
-        <f>IF(C16, IFERROR(STDEV('Post-print worksheet'!D22:F22),0),"")</f>
+      <c r="G16" s="21">
+        <f>IF(C16, IFERROR(STDEV('Post-print worksheet'!D26:F26),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="21">
         <f>IF(C16, IFERROR(SQRT((Intro!$B$8/3)^2+G16^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I16" s="19" t="str">
+      <c r="I16" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J16" s="19" t="str">
+      <c r="J16" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K16" s="19" t="str">
+      <c r="K16" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -14898,81 +15066,81 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E17" s="61">
-        <f>IF(D17,'Post-print worksheet'!C23,0)</f>
+      <c r="E17" s="69">
+        <f>IF(D17,'Post-print worksheet'!C27,0)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="19" t="str">
-        <f>IF(C17, IFERROR(AVERAGE('Post-print worksheet'!D23:F23),""),"")</f>
+      <c r="F17" s="21" t="str">
+        <f>IF(C17, IFERROR(AVERAGE('Post-print worksheet'!D27:F27),""),"")</f>
         <v/>
       </c>
-      <c r="G17" s="19" t="str">
-        <f>IF(C17, IFERROR(STDEV('Post-print worksheet'!D23:F23),0),"")</f>
+      <c r="G17" s="21" t="str">
+        <f>IF(C17, IFERROR(STDEV('Post-print worksheet'!D27:F27),0),"")</f>
         <v/>
       </c>
-      <c r="H17" s="19" t="str">
+      <c r="H17" s="21" t="str">
         <f>IF(C17, IFERROR(SQRT((Intro!$B$8/3)^2+G17^2),0),"")</f>
         <v/>
       </c>
-      <c r="I17" s="19" t="str">
+      <c r="I17" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J17" s="19" t="str">
+      <c r="J17" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K17" s="19" t="str">
+      <c r="K17" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23" t="str">
+      <c r="A18" s="25"/>
+      <c r="B18" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C18" s="23" t="b">
+      <c r="C18" s="25" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D18" s="23" t="b">
+      <c r="D18" s="25" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E18" s="62">
-        <f>IF(D18,'Post-print worksheet'!C24,0)</f>
+      <c r="E18" s="70">
+        <f>IF(D18,'Post-print worksheet'!C28,0)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="26" t="str">
-        <f>IF(C18, IFERROR(AVERAGE('Post-print worksheet'!D24:F24),""),"")</f>
+      <c r="F18" s="28" t="str">
+        <f>IF(C18, IFERROR(AVERAGE('Post-print worksheet'!D28:F28),""),"")</f>
         <v/>
       </c>
-      <c r="G18" s="26" t="str">
-        <f>IF(C18, IFERROR(STDEV('Post-print worksheet'!D24:F24),0),"")</f>
+      <c r="G18" s="28" t="str">
+        <f>IF(C18, IFERROR(STDEV('Post-print worksheet'!D28:F28),0),"")</f>
         <v/>
       </c>
-      <c r="H18" s="26" t="str">
+      <c r="H18" s="28" t="str">
         <f>IF(C18, IFERROR(SQRT((Intro!$B$8/3)^2+G18^2),0),"")</f>
         <v/>
       </c>
-      <c r="I18" s="26" t="str">
+      <c r="I18" s="28" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J18" s="26" t="str">
+      <c r="J18" s="28" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K18" s="26" t="str">
+      <c r="K18" s="28" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B19" s="1">
         <f>IF(1 &lt;= Intro!B$3, 1, "")</f>
@@ -14986,31 +15154,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E19" s="61">
-        <f>IF(D19,'Post-print worksheet'!C25,0)</f>
+      <c r="E19" s="69">
+        <f>IF(D19,'Post-print worksheet'!C29,0)</f>
         <v>0</v>
       </c>
-      <c r="F19" s="19" t="str">
-        <f>IF(C19, IFERROR(AVERAGE('Post-print worksheet'!D25:F25),""),"")</f>
+      <c r="F19" s="21" t="str">
+        <f>IF(C19, IFERROR(AVERAGE('Post-print worksheet'!D29:F29),""),"")</f>
         <v/>
       </c>
-      <c r="G19" s="19">
-        <f>IF(C19, IFERROR(STDEV('Post-print worksheet'!D25:F25),0),"")</f>
+      <c r="G19" s="21">
+        <f>IF(C19, IFERROR(STDEV('Post-print worksheet'!D29:F29),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H19" s="19">
+      <c r="H19" s="21">
         <f>IF(C19, IFERROR(SQRT((Intro!$B$8/3)^2+G19^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I19" s="19" t="str">
+      <c r="I19" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J19" s="19" t="str">
+      <c r="J19" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K19" s="19" t="str">
+      <c r="K19" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -15029,31 +15197,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E20" s="61">
-        <f>IF(D20,'Post-print worksheet'!C26,0)</f>
+      <c r="E20" s="69">
+        <f>IF(D20,'Post-print worksheet'!C30,0)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="19" t="str">
-        <f>IF(C20, IFERROR(AVERAGE('Post-print worksheet'!D26:F26),""),"")</f>
+      <c r="F20" s="21" t="str">
+        <f>IF(C20, IFERROR(AVERAGE('Post-print worksheet'!D30:F30),""),"")</f>
         <v/>
       </c>
-      <c r="G20" s="19">
-        <f>IF(C20, IFERROR(STDEV('Post-print worksheet'!D26:F26),0),"")</f>
+      <c r="G20" s="21">
+        <f>IF(C20, IFERROR(STDEV('Post-print worksheet'!D30:F30),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="21">
         <f>IF(C20, IFERROR(SQRT((Intro!$B$8/3)^2+G20^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I20" s="19" t="str">
+      <c r="I20" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J20" s="19" t="str">
+      <c r="J20" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K20" s="19" t="str">
+      <c r="K20" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -15072,31 +15240,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E21" s="61">
-        <f>IF(D21,'Post-print worksheet'!C27,0)</f>
+      <c r="E21" s="69">
+        <f>IF(D21,'Post-print worksheet'!C31,0)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="19" t="str">
-        <f>IF(C21, IFERROR(AVERAGE('Post-print worksheet'!D27:F27),""),"")</f>
+      <c r="F21" s="21" t="str">
+        <f>IF(C21, IFERROR(AVERAGE('Post-print worksheet'!D31:F31),""),"")</f>
         <v/>
       </c>
-      <c r="G21" s="19">
-        <f>IF(C21, IFERROR(STDEV('Post-print worksheet'!D27:F27),0),"")</f>
+      <c r="G21" s="21">
+        <f>IF(C21, IFERROR(STDEV('Post-print worksheet'!D31:F31),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="21">
         <f>IF(C21, IFERROR(SQRT((Intro!$B$8/3)^2+G21^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I21" s="19" t="str">
+      <c r="I21" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J21" s="19" t="str">
+      <c r="J21" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K21" s="19" t="str">
+      <c r="K21" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -15115,81 +15283,81 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E22" s="61">
-        <f>IF(D22,'Post-print worksheet'!C28,0)</f>
+      <c r="E22" s="69">
+        <f>IF(D22,'Post-print worksheet'!C32,0)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="19" t="str">
-        <f>IF(C22, IFERROR(AVERAGE('Post-print worksheet'!D28:F28),""),"")</f>
+      <c r="F22" s="21" t="str">
+        <f>IF(C22, IFERROR(AVERAGE('Post-print worksheet'!D32:F32),""),"")</f>
         <v/>
       </c>
-      <c r="G22" s="19" t="str">
-        <f>IF(C22, IFERROR(STDEV('Post-print worksheet'!D28:F28),0),"")</f>
+      <c r="G22" s="21" t="str">
+        <f>IF(C22, IFERROR(STDEV('Post-print worksheet'!D32:F32),0),"")</f>
         <v/>
       </c>
-      <c r="H22" s="19" t="str">
+      <c r="H22" s="21" t="str">
         <f>IF(C22, IFERROR(SQRT((Intro!$B$8/3)^2+G22^2),0),"")</f>
         <v/>
       </c>
-      <c r="I22" s="19" t="str">
+      <c r="I22" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J22" s="19" t="str">
+      <c r="J22" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="K22" s="19" t="str">
+      <c r="K22" s="21" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23" t="str">
+      <c r="A23" s="25"/>
+      <c r="B23" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 5, "")</f>
         <v/>
       </c>
-      <c r="C23" s="23" t="b">
+      <c r="C23" s="25" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D23" s="23" t="b">
+      <c r="D23" s="25" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E23" s="62">
-        <f>IF(D23,'Post-print worksheet'!C29,0)</f>
+      <c r="E23" s="70">
+        <f>IF(D23,'Post-print worksheet'!C33,0)</f>
         <v>0</v>
       </c>
-      <c r="F23" s="26" t="str">
-        <f>IF(C23, IFERROR(AVERAGE('Post-print worksheet'!D29:F29),""),"")</f>
+      <c r="F23" s="28" t="str">
+        <f>IF(C23, IFERROR(AVERAGE('Post-print worksheet'!D33:F33),""),"")</f>
         <v/>
       </c>
-      <c r="G23" s="26" t="str">
-        <f>IF(C23, IFERROR(STDEV('Post-print worksheet'!D29:F29),0),"")</f>
+      <c r="G23" s="28" t="str">
+        <f>IF(C23, IFERROR(STDEV('Post-print worksheet'!D33:F33),0),"")</f>
         <v/>
       </c>
-      <c r="H23" s="26" t="str">
+      <c r="H23" s="28" t="str">
         <f>IF(C23, IFERROR(SQRT((Intro!$B$8/3)^2+G23^2),0),"")</f>
         <v/>
       </c>
-      <c r="I23" s="26" t="str">
+      <c r="I23" s="28" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J23" s="26" t="str">
+      <c r="J23" s="28" t="str">
         <f>IF(C23, 1/(2*Intro!B$3*E23),"")</f>
         <v/>
       </c>
-      <c r="K23" s="26" t="str">
+      <c r="K23" s="28" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="B24" s="1">
         <f>IF(2 &lt;= Intro!B$3, 1, "")</f>
@@ -15203,28 +15371,28 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E24" s="61">
-        <f>IF(D24,'Post-print worksheet'!C30,0)</f>
+      <c r="E24" s="69">
+        <f>IF(D24,'Post-print worksheet'!C34,0)</f>
         <v>0</v>
       </c>
-      <c r="F24" s="19" t="str">
-        <f>IF(C24, IFERROR(AVERAGE('Post-print worksheet'!D30:F30),""),"")</f>
+      <c r="F24" s="21" t="str">
+        <f>IF(C24, IFERROR(AVERAGE('Post-print worksheet'!D34:F34),""),"")</f>
         <v/>
       </c>
-      <c r="G24" s="19">
-        <f>IF(C24, IFERROR(STDEV('Post-print worksheet'!D30:F30),0),"")</f>
+      <c r="G24" s="21">
+        <f>IF(C24, IFERROR(STDEV('Post-print worksheet'!D34:F34),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="21">
         <f>IF(C24, IFERROR(SQRT((Intro!$B$8/3)^2+G24^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I24" s="19" t="str">
+      <c r="I24" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J24" s="63"/>
-      <c r="K24" s="63"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="71"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1"/>
@@ -15240,28 +15408,28 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E25" s="61">
-        <f>IF(D25,'Post-print worksheet'!C31,0)</f>
+      <c r="E25" s="69">
+        <f>IF(D25,'Post-print worksheet'!C35,0)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="19" t="str">
-        <f>IF(C25, IFERROR(AVERAGE('Post-print worksheet'!D31:F31),""),"")</f>
+      <c r="F25" s="21" t="str">
+        <f>IF(C25, IFERROR(AVERAGE('Post-print worksheet'!D35:F35),""),"")</f>
         <v/>
       </c>
-      <c r="G25" s="19">
-        <f>IF(C25, IFERROR(STDEV('Post-print worksheet'!D31:F31),0),"")</f>
+      <c r="G25" s="21">
+        <f>IF(C25, IFERROR(STDEV('Post-print worksheet'!D35:F35),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H25" s="19">
+      <c r="H25" s="21">
         <f>IF(C25, IFERROR(SQRT((Intro!$B$8/3)^2+G25^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I25" s="19" t="str">
+      <c r="I25" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J25" s="63"/>
-      <c r="K25" s="63"/>
+      <c r="J25" s="71"/>
+      <c r="K25" s="71"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1"/>
@@ -15277,69 +15445,69 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E26" s="61">
-        <f>IF(D26,'Post-print worksheet'!C32,0)</f>
+      <c r="E26" s="69">
+        <f>IF(D26,'Post-print worksheet'!C36,0)</f>
         <v>0</v>
       </c>
-      <c r="F26" s="19" t="str">
-        <f>IF(C26, IFERROR(AVERAGE('Post-print worksheet'!D32:F32),""),"")</f>
+      <c r="F26" s="21" t="str">
+        <f>IF(C26, IFERROR(AVERAGE('Post-print worksheet'!D36:F36),""),"")</f>
         <v/>
       </c>
-      <c r="G26" s="19" t="str">
-        <f>IF(C26, IFERROR(STDEV('Post-print worksheet'!D32:F32),0),"")</f>
+      <c r="G26" s="21" t="str">
+        <f>IF(C26, IFERROR(STDEV('Post-print worksheet'!D36:F36),0),"")</f>
         <v/>
       </c>
-      <c r="H26" s="19" t="str">
+      <c r="H26" s="21" t="str">
         <f>IF(C26, IFERROR(SQRT((Intro!$B$8/3)^2+G26^2),0),"")</f>
         <v/>
       </c>
-      <c r="I26" s="19" t="str">
+      <c r="I26" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J26" s="63"/>
-      <c r="K26" s="63"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="71"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23" t="str">
+      <c r="A27" s="25"/>
+      <c r="B27" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C27" s="23" t="b">
+      <c r="C27" s="25" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D27" s="23" t="b">
+      <c r="D27" s="25" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E27" s="62">
-        <f>IF(D27,'Post-print worksheet'!C33,0)</f>
+      <c r="E27" s="70">
+        <f>IF(D27,'Post-print worksheet'!C37,0)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="26" t="str">
-        <f>IF(C27, IFERROR(AVERAGE('Post-print worksheet'!D33:F33),""),"")</f>
+      <c r="F27" s="28" t="str">
+        <f>IF(C27, IFERROR(AVERAGE('Post-print worksheet'!D37:F37),""),"")</f>
         <v/>
       </c>
-      <c r="G27" s="26" t="str">
-        <f>IF(C27, IFERROR(STDEV('Post-print worksheet'!D33:F33),0),"")</f>
+      <c r="G27" s="28" t="str">
+        <f>IF(C27, IFERROR(STDEV('Post-print worksheet'!D37:F37),0),"")</f>
         <v/>
       </c>
-      <c r="H27" s="26" t="str">
+      <c r="H27" s="28" t="str">
         <f>IF(C27, IFERROR(SQRT((Intro!$B$8/3)^2+G27^2),0),"")</f>
         <v/>
       </c>
-      <c r="I27" s="26" t="str">
+      <c r="I27" s="28" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J27" s="64"/>
-      <c r="K27" s="64"/>
+      <c r="J27" s="72"/>
+      <c r="K27" s="72"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="B28" s="1">
         <f>IF(2 &lt;= Intro!B$3, 1, "")</f>
@@ -15353,28 +15521,28 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E28" s="61">
-        <f>IF(D28,'Post-print worksheet'!C34,0)</f>
+      <c r="E28" s="69">
+        <f>IF(D28,'Post-print worksheet'!C38,0)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="19" t="str">
-        <f>IF(C28, IFERROR(AVERAGE('Post-print worksheet'!D34:F34),""),"")</f>
+      <c r="F28" s="21" t="str">
+        <f>IF(C28, IFERROR(AVERAGE('Post-print worksheet'!D38:F38),""),"")</f>
         <v/>
       </c>
-      <c r="G28" s="19">
-        <f>IF(C28, IFERROR(STDEV('Post-print worksheet'!D34:F34),0),"")</f>
+      <c r="G28" s="21">
+        <f>IF(C28, IFERROR(STDEV('Post-print worksheet'!D38:F38),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H28" s="19">
+      <c r="H28" s="21">
         <f>IF(C28, IFERROR(SQRT((Intro!$B$8/3)^2+G28^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I28" s="19" t="str">
+      <c r="I28" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J28" s="63"/>
-      <c r="K28" s="63"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="71"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="B29" s="1">
@@ -15389,28 +15557,28 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E29" s="61">
-        <f>IF(D29,'Post-print worksheet'!C35,0)</f>
+      <c r="E29" s="69">
+        <f>IF(D29,'Post-print worksheet'!C39,0)</f>
         <v>0</v>
       </c>
-      <c r="F29" s="19" t="str">
-        <f>IF(C29, IFERROR(AVERAGE('Post-print worksheet'!D35:F35),""),"")</f>
+      <c r="F29" s="21" t="str">
+        <f>IF(C29, IFERROR(AVERAGE('Post-print worksheet'!D39:F39),""),"")</f>
         <v/>
       </c>
-      <c r="G29" s="19">
-        <f>IF(C29, IFERROR(STDEV('Post-print worksheet'!D35:F35),0),"")</f>
+      <c r="G29" s="21">
+        <f>IF(C29, IFERROR(STDEV('Post-print worksheet'!D39:F39),0),"")</f>
         <v>0</v>
       </c>
-      <c r="H29" s="19">
+      <c r="H29" s="21">
         <f>IF(C29, IFERROR(SQRT((Intro!$B$8/3)^2+G29^2),0),"")</f>
         <v>0.003333333333</v>
       </c>
-      <c r="I29" s="19" t="str">
+      <c r="I29" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J29" s="63"/>
-      <c r="K29" s="63"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="71"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="B30" s="1" t="str">
@@ -15425,65 +15593,65 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E30" s="61">
-        <f>IF(D30,'Post-print worksheet'!C36,0)</f>
+      <c r="E30" s="69">
+        <f>IF(D30,'Post-print worksheet'!C40,0)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="19" t="str">
-        <f>IF(C30, IFERROR(AVERAGE('Post-print worksheet'!D36:F36),""),"")</f>
+      <c r="F30" s="21" t="str">
+        <f>IF(C30, IFERROR(AVERAGE('Post-print worksheet'!D40:F40),""),"")</f>
         <v/>
       </c>
-      <c r="G30" s="19" t="str">
-        <f>IF(C30, IFERROR(STDEV('Post-print worksheet'!D36:F36),0),"")</f>
+      <c r="G30" s="21" t="str">
+        <f>IF(C30, IFERROR(STDEV('Post-print worksheet'!D40:F40),0),"")</f>
         <v/>
       </c>
-      <c r="H30" s="19" t="str">
+      <c r="H30" s="21" t="str">
         <f>IF(C30, IFERROR(SQRT((Intro!$B$8/3)^2+G30^2),0),"")</f>
         <v/>
       </c>
-      <c r="I30" s="19" t="str">
+      <c r="I30" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J30" s="63"/>
-      <c r="K30" s="63"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="71"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="23"/>
-      <c r="B31" s="23" t="str">
+      <c r="A31" s="25"/>
+      <c r="B31" s="25" t="str">
         <f>IF(5 &lt;= Intro!B$3, 4, "")</f>
         <v/>
       </c>
-      <c r="C31" s="23" t="b">
+      <c r="C31" s="25" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D31" s="23" t="b">
+      <c r="D31" s="25" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E31" s="62">
-        <f>IF(D31,'Post-print worksheet'!C37,0)</f>
+      <c r="E31" s="70">
+        <f>IF(D31,'Post-print worksheet'!C41,0)</f>
         <v>0</v>
       </c>
-      <c r="F31" s="26" t="str">
-        <f>IF(C31, IFERROR(AVERAGE('Post-print worksheet'!D37:F37),""),"")</f>
+      <c r="F31" s="28" t="str">
+        <f>IF(C31, IFERROR(AVERAGE('Post-print worksheet'!D41:F41),""),"")</f>
         <v/>
       </c>
-      <c r="G31" s="26" t="str">
-        <f>IF(C31, IFERROR(STDEV('Post-print worksheet'!D37:F37),0),"")</f>
+      <c r="G31" s="28" t="str">
+        <f>IF(C31, IFERROR(STDEV('Post-print worksheet'!D41:F41),0),"")</f>
         <v/>
       </c>
-      <c r="H31" s="26" t="str">
+      <c r="H31" s="28" t="str">
         <f>IF(C31, IFERROR(SQRT((Intro!$B$8/3)^2+G31^2),0),"")</f>
         <v/>
       </c>
-      <c r="I31" s="26" t="str">
+      <c r="I31" s="28" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="J31" s="64"/>
-      <c r="K31" s="64"/>
+      <c r="J31" s="72"/>
+      <c r="K31" s="72"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="B32" s="2"/>
@@ -15496,88 +15664,88 @@
       <c r="H33" s="2"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="65"/>
-      <c r="B34" s="9" t="s">
-        <v>86</v>
+      <c r="A34" s="73"/>
+      <c r="B34" s="11" t="s">
+        <v>96</v>
       </c>
       <c r="C34" s="1"/>
-      <c r="D34" s="66" t="s">
-        <v>87</v>
-      </c>
-      <c r="E34" s="67"/>
-      <c r="F34" s="68"/>
+      <c r="D34" s="74" t="s">
+        <v>97</v>
+      </c>
+      <c r="E34" s="75"/>
+      <c r="F34" s="76"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="69"/>
-      <c r="B35" s="38" t="s">
-        <v>88</v>
+      <c r="A35" s="77"/>
+      <c r="B35" s="44" t="s">
+        <v>98</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="D35" s="16" t="s">
-        <v>90</v>
+        <v>99</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>100</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="F35" s="38" t="s">
-        <v>83</v>
+        <v>101</v>
+      </c>
+      <c r="F35" s="44" t="s">
+        <v>93</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="B36" s="70" t="str">
+      <c r="A36" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B36" s="78" t="str">
         <f>SUM(F24:F27)/SUMPRODUCT(D24:D27*E24:E27)*Intro!$B$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C36" s="71" t="str">
+      <c r="C36" s="79" t="str">
         <f t="shared" ref="C36:C38" si="6">CEILING(-LOG10(D36),1)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D36" s="72" t="str">
+      <c r="D36" s="80" t="str">
         <f>SQRT(SUMSQ(H24:H27))/SUMPRODUCT(D24:D27*E24:E27)*Intro!$B$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E36" s="51" t="str">
+      <c r="E36" s="57" t="str">
         <f>-B36/(2*B38*B39*SIN(B41*PI()/180))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F36" s="73" t="str">
+      <c r="F36" s="81" t="str">
         <f t="shared" ref="F36:F39" si="7">D36*E36</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
-      <c r="J36" s="74"/>
+      <c r="J36" s="82"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="B37" s="70" t="str">
+      <c r="A37" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" s="78" t="str">
         <f>SUM(F28:F31)/SUMPRODUCT(D28:D31*E28:E31)*Intro!$B$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C37" s="71" t="str">
+      <c r="C37" s="79" t="str">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D37" s="72" t="str">
+      <c r="D37" s="80" t="str">
         <f>SQRT(SUMSQ(H28:H31))/SUMPRODUCT(D28:D31*E28:E31)*Intro!$B$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E37" s="51" t="str">
+      <c r="E37" s="57" t="str">
         <f>B37/(2*B38*B39*SIN(B41*PI()/180))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F37" s="73" t="str">
+      <c r="F37" s="81" t="str">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
@@ -15585,26 +15753,26 @@
       <c r="H37" s="2"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="B38" s="70" t="str">
+      <c r="A38" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38" s="78" t="str">
         <f>SQRT(2)*Intro!B4/2*SUM(F4:F8)/(SUMPRODUCT(D4:D8*E4:E8))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C38" s="71" t="str">
+      <c r="C38" s="79" t="str">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="D38" s="72" t="str">
+      <c r="D38" s="80" t="str">
         <f>SQRT(2)*Intro!B4/2*SQRT(SUMSQ(H4:H8))/(SUMPRODUCT(D4:D8*E4:E8))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E38" s="51" t="str">
+      <c r="E38" s="57" t="str">
         <f>(B36^2-B37^2)/(4*B38^2*B39*SIN(B41*PI()/180))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F38" s="73" t="str">
+      <c r="F38" s="81" t="str">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
@@ -15612,23 +15780,23 @@
       <c r="H38" s="2"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="B39" s="70" t="str">
+      <c r="A39" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="B39" s="78" t="str">
         <f>SQRT(2)*Intro!B4/2*SUM(F14:F18)/(SUMPRODUCT(D14:D18*E14:E18))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C39" s="75"/>
-      <c r="D39" s="76" t="str">
+      <c r="C39" s="83"/>
+      <c r="D39" s="84" t="str">
         <f>SQRT(2)*Intro!B4/2*SQRT(SUMSQ(H14:H18))/(SUMPRODUCT(D14:D18*E14:E18))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E39" s="55" t="str">
+      <c r="E39" s="61" t="str">
         <f>(B36^2-B37^2)/(4*B38*B39^2*SIN(B41*PI()/180))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F39" s="77" t="str">
+      <c r="F39" s="85" t="str">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
@@ -15636,69 +15804,71 @@
       <c r="H39" s="2"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="B40" s="78" t="str">
+      <c r="A40" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="B40" s="86" t="str">
         <f>(B36^2-B37^2)/(4*B38*B39)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C40" s="74"/>
-      <c r="D40" s="74"/>
-      <c r="E40" s="74"/>
-      <c r="F40" s="74"/>
-      <c r="G40" s="74"/>
-      <c r="H40" s="74"/>
+      <c r="C40" s="82"/>
+      <c r="D40" s="82"/>
+      <c r="E40" s="82"/>
+      <c r="F40" s="82"/>
+      <c r="G40" s="82"/>
+      <c r="H40" s="82"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="B41" s="78" t="str">
+      <c r="A41" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41" s="86" t="str">
         <f>ACOS(B40)*180/PI()</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C41" s="74"/>
-      <c r="D41" s="74"/>
-      <c r="E41" s="74"/>
-      <c r="F41" s="74"/>
-      <c r="G41" s="74"/>
-      <c r="H41" s="74"/>
+      <c r="C41" s="82"/>
+      <c r="D41" s="82"/>
+      <c r="E41" s="82"/>
+      <c r="F41" s="82"/>
+      <c r="G41" s="82"/>
+      <c r="H41" s="82"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="B42" s="78" t="str">
+      <c r="A42" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B42" s="86" t="str">
         <f>B41-90</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C42" s="74"/>
-      <c r="D42" s="74" t="s">
-        <v>99</v>
-      </c>
-      <c r="E42" s="74" t="s">
-        <v>100</v>
-      </c>
-      <c r="F42" s="74" t="s">
-        <v>101</v>
-      </c>
-      <c r="G42" s="74"/>
-      <c r="H42" s="74"/>
+      <c r="C42" s="82"/>
+      <c r="D42" s="82" t="s">
+        <v>109</v>
+      </c>
+      <c r="E42" s="82" t="s">
+        <v>110</v>
+      </c>
+      <c r="F42" s="87" t="s">
+        <v>111</v>
+      </c>
+      <c r="G42" s="87" t="s">
+        <v>112</v>
+      </c>
+      <c r="H42" s="82"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="B43" s="79" t="str">
+      <c r="A43" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="B43" s="88" t="str">
         <f>SQRT(SUMSQ(F36:F39))*180/PI()</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C43" s="74"/>
-      <c r="D43" s="74" t="s">
-        <v>46</v>
-      </c>
-      <c r="E43" s="19" t="str">
+      <c r="C43" s="82"/>
+      <c r="D43" s="82" t="s">
+        <v>56</v>
+      </c>
+      <c r="E43" s="21" t="str">
         <f>AVERAGE(I4:I13)</f>
         <v>#DIV/0!</v>
       </c>
@@ -15706,23 +15876,29 @@
         <f>Intro!B6*(SUM(F4:F13))/SUMPRODUCT(E4:E13*D4:D13)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G43" s="74"/>
-      <c r="H43" s="74"/>
+      <c r="G43" s="82" t="str">
+        <f>Intro!B6*(SUM(F4:F23))/SUMPRODUCT(E4:E23*D4:D23)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H43" s="82"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="B44" s="2"/>
-      <c r="D44" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E44" s="80" t="str">
+      <c r="D44" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E44" s="89" t="str">
         <f>AVERAGE(I14:I23)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F44" s="6" t="str">
+      <c r="F44" s="8" t="str">
         <f>Intro!B6*(SUM(F14:F23))/SUMPRODUCT(E14:E23*D14:D23)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G44" s="2"/>
+      <c r="G44" s="8" t="str">
+        <f>Intro!B6*(SUM(F4:F23))/SUMPRODUCT(E4:E23*D4:D23)</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="H44" s="2"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
@@ -15732,20 +15908,20 @@
       <c r="L45" s="1"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="B46" s="68"/>
+      <c r="A46" s="73" t="s">
+        <v>114</v>
+      </c>
+      <c r="B46" s="76"/>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="69" t="s">
-        <v>30</v>
-      </c>
-      <c r="B47" s="81">
+      <c r="A47" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="B47" s="90">
         <f>COUNTIF(D4:D8, TRUE())</f>
         <v>0</v>
       </c>
@@ -15754,10 +15930,10 @@
       <c r="K47" s="1"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="69" t="s">
-        <v>31</v>
-      </c>
-      <c r="B48" s="81">
+      <c r="A48" s="77" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48" s="90">
         <f>COUNTIF(D9:D13, TRUE())</f>
         <v>0</v>
       </c>
@@ -15765,10 +15941,10 @@
       <c r="H48" s="2"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="69" t="s">
-        <v>32</v>
-      </c>
-      <c r="B49" s="81">
+      <c r="A49" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="B49" s="90">
         <f>COUNTIF(D14:D18, TRUE())</f>
         <v>0</v>
       </c>
@@ -15776,10 +15952,10 @@
       <c r="H49" s="2"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="69" t="s">
-        <v>33</v>
-      </c>
-      <c r="B50" s="81">
+      <c r="A50" s="77" t="s">
+        <v>39</v>
+      </c>
+      <c r="B50" s="90">
         <f>COUNTIF(D19:D23, TRUE())</f>
         <v>0</v>
       </c>
@@ -15787,10 +15963,10 @@
       <c r="H50" s="2"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="69" t="s">
-        <v>84</v>
-      </c>
-      <c r="B51" s="81">
+      <c r="A51" s="77" t="s">
+        <v>94</v>
+      </c>
+      <c r="B51" s="90">
         <f>COUNTIF(D24:D27, TRUE())</f>
         <v>0</v>
       </c>
@@ -15798,10 +15974,10 @@
       <c r="H51" s="2"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="82" t="s">
-        <v>85</v>
-      </c>
-      <c r="B52" s="83">
+      <c r="A52" s="91" t="s">
+        <v>95</v>
+      </c>
+      <c r="B52" s="92">
         <f>COUNTIF(D28:D31, TRUE())</f>
         <v>0</v>
       </c>

</xml_diff>